<commit_message>
update_open_items.py: add How to Test column (14th)
Auto-rebuild Excel script now mirrors the registry schema. Previous
version stopped at 13 columns (commit / date_fixed); didn't pick up
the how_to_test field added 2026-05-10.

Changes:
  - headers list: append "How to Test"
  - row build: append it.get("how_to_test") to each row
  - width: 60 (wide column for command snippets)
  - alignment: left + wrap (long prose); Menlo 9pt (commands)
  - row height calc: includes how_to_test in max_len

Auto-rebuild hook (.git/hooks/pre-commit) calls this script when
data/open_items.json changes — so future Excel regenerations include
the new column automatically.

Output verified: cache/open_items_2026-05-10.xlsx now has 14 columns,
header[14] = "How to Test", populated with concrete test instructions
for 33 of 57 items (placeholders for the rest).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-10.xlsx
+++ b/cache/open_items_2026-05-10.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -43,6 +43,10 @@
     <font>
       <name val="Menlo"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Menlo"/>
+      <sz val="9"/>
     </font>
     <font>
       <b val="1"/>
@@ -175,7 +179,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -192,11 +196,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
@@ -204,37 +211,37 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="16" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -608,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M58"/>
+  <dimension ref="A1:N58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -624,6 +631,7 @@
     <col width="13" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
     <col width="13" customWidth="1" min="13" max="13"/>
+    <col width="60" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -692,6 +700,11 @@
           <t>Commit</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>How to Test</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="60" customHeight="1">
       <c r="A2" s="2" t="n">
@@ -749,6 +762,11 @@
       </c>
       <c r="L2" s="2" t="inlineStr"/>
       <c r="M2" s="3" t="inlineStr"/>
+      <c r="N2" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="2" t="n">
@@ -806,6 +824,11 @@
       </c>
       <c r="L3" s="2" t="inlineStr"/>
       <c r="M3" s="3" t="inlineStr"/>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="45" customHeight="1">
       <c r="A4" s="2" t="n">
@@ -863,6 +886,11 @@
       </c>
       <c r="L4" s="2" t="inlineStr"/>
       <c r="M4" s="3" t="inlineStr"/>
+      <c r="N4" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="45" customHeight="1">
       <c r="A5" s="2" t="n">
@@ -873,7 +901,7 @@
           <t>CLEAN-1</t>
         </is>
       </c>
-      <c r="C5" s="8" t="inlineStr">
+      <c r="C5" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -920,6 +948,11 @@
       </c>
       <c r="L5" s="2" t="inlineStr"/>
       <c r="M5" s="3" t="inlineStr"/>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="60" customHeight="1">
       <c r="A6" s="2" t="n">
@@ -930,7 +963,7 @@
           <t>CLEAN-3</t>
         </is>
       </c>
-      <c r="C6" s="8" t="inlineStr">
+      <c r="C6" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -977,6 +1010,11 @@
       </c>
       <c r="L6" s="2" t="inlineStr"/>
       <c r="M6" s="3" t="inlineStr"/>
+      <c r="N6" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="45" customHeight="1">
       <c r="A7" s="2" t="n">
@@ -987,7 +1025,7 @@
           <t>OPS-1</t>
         </is>
       </c>
-      <c r="C7" s="8" t="inlineStr">
+      <c r="C7" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1034,6 +1072,11 @@
       </c>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="45" customHeight="1">
       <c r="A8" s="2" t="n">
@@ -1044,7 +1087,7 @@
           <t>PERF-6</t>
         </is>
       </c>
-      <c r="C8" s="8" t="inlineStr">
+      <c r="C8" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1087,6 +1130,11 @@
       </c>
       <c r="L8" s="2" t="inlineStr"/>
       <c r="M8" s="3" t="inlineStr"/>
+      <c r="N8" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="75" customHeight="1">
       <c r="A9" s="2" t="n">
@@ -1097,7 +1145,7 @@
           <t>PERF-7</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C9" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1144,6 +1192,11 @@
       </c>
       <c r="L9" s="2" t="inlineStr"/>
       <c r="M9" s="3" t="inlineStr"/>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="45" customHeight="1">
       <c r="A10" s="2" t="n">
@@ -1154,7 +1207,7 @@
           <t>QUANT-3</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C10" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1197,6 +1250,11 @@
       </c>
       <c r="L10" s="2" t="inlineStr"/>
       <c r="M10" s="3" t="inlineStr"/>
+      <c r="N10" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="n">
@@ -1207,7 +1265,7 @@
           <t>QUANT-4</t>
         </is>
       </c>
-      <c r="C11" s="8" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1254,6 +1312,11 @@
       </c>
       <c r="L11" s="2" t="inlineStr"/>
       <c r="M11" s="3" t="inlineStr"/>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="n">
@@ -1264,7 +1327,7 @@
           <t>QUANT-5</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C12" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1311,6 +1374,11 @@
       </c>
       <c r="L12" s="2" t="inlineStr"/>
       <c r="M12" s="3" t="inlineStr"/>
+      <c r="N12" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="60" customHeight="1">
       <c r="A13" s="2" t="n">
@@ -1321,7 +1389,7 @@
           <t>QUANT-6</t>
         </is>
       </c>
-      <c r="C13" s="8" t="inlineStr">
+      <c r="C13" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1364,6 +1432,11 @@
       </c>
       <c r="L13" s="2" t="inlineStr"/>
       <c r="M13" s="3" t="inlineStr"/>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="n">
@@ -1374,7 +1447,7 @@
           <t>MOD-2</t>
         </is>
       </c>
-      <c r="C14" s="8" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1417,6 +1490,11 @@
       </c>
       <c r="L14" s="2" t="inlineStr"/>
       <c r="M14" s="3" t="inlineStr"/>
+      <c r="N14" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="45" customHeight="1">
       <c r="A15" s="2" t="n">
@@ -1427,7 +1505,7 @@
           <t>CLEAN-4</t>
         </is>
       </c>
-      <c r="C15" s="9" t="inlineStr">
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1474,6 +1552,11 @@
       </c>
       <c r="L15" s="2" t="inlineStr"/>
       <c r="M15" s="3" t="inlineStr"/>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="60" customHeight="1">
       <c r="A16" s="2" t="n">
@@ -1484,7 +1567,7 @@
           <t>OPS-2</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1527,6 +1610,11 @@
       </c>
       <c r="L16" s="2" t="inlineStr"/>
       <c r="M16" s="3" t="inlineStr"/>
+      <c r="N16" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="n">
@@ -1537,7 +1625,7 @@
           <t>OPS-3</t>
         </is>
       </c>
-      <c r="C17" s="9" t="inlineStr">
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1580,6 +1668,11 @@
       </c>
       <c r="L17" s="2" t="inlineStr"/>
       <c r="M17" s="3" t="inlineStr"/>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45" customHeight="1">
       <c r="A18" s="2" t="n">
@@ -1590,7 +1683,7 @@
           <t>OPS-4</t>
         </is>
       </c>
-      <c r="C18" s="9" t="inlineStr">
+      <c r="C18" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1633,6 +1726,11 @@
       </c>
       <c r="L18" s="2" t="inlineStr"/>
       <c r="M18" s="3" t="inlineStr"/>
+      <c r="N18" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="60" customHeight="1">
       <c r="A19" s="2" t="n">
@@ -1643,7 +1741,7 @@
           <t>MOD-1</t>
         </is>
       </c>
-      <c r="C19" s="9" t="inlineStr">
+      <c r="C19" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -1690,6 +1788,11 @@
       </c>
       <c r="L19" s="2" t="inlineStr"/>
       <c r="M19" s="3" t="inlineStr"/>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="n">
@@ -1740,13 +1843,18 @@
           <t>Concerning: 30+ min into backtest, still 0 BUYs across 5 months simulated. Likely needs per-band kill (TC at score 60-79 only) instead of full kill.</t>
         </is>
       </c>
-      <c r="K20" s="10" t="inlineStr">
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="L20" s="2" t="inlineStr"/>
       <c r="M20" s="3" t="inlineStr"/>
+      <c r="N20" s="8" t="inlineStr">
+        <is>
+          <t>ps -p 29239 → if alive backtest still running. When done: ls cache/portfolio_backtest_750d_*.json | head -1 → check PF, total_return_pct.</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="60" customHeight="1">
       <c r="A21" s="2" t="n">
@@ -1757,7 +1865,7 @@
           <t>A5-followup</t>
         </is>
       </c>
-      <c r="C21" s="8" t="inlineStr">
+      <c r="C21" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -1797,7 +1905,7 @@
           <t>Wilson LB clears 40% threshold. Don't enable until subtype investigation done.</t>
         </is>
       </c>
-      <c r="K21" s="10" t="inlineStr">
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>IN_PROGRESS</t>
         </is>
@@ -1806,6 +1914,11 @@
       <c r="M21" s="3" t="inlineStr">
         <is>
           <t>1e40d30fc</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>grep -A20 'pullback_bull_701' config/config.json → _validations entry present with n=134 wr_lb=0.446. _enabled stays false.</t>
         </is>
       </c>
     </row>
@@ -1858,7 +1971,7 @@
           <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
         </is>
       </c>
-      <c r="K22" s="11" t="inlineStr">
+      <c r="K22" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -1871,6 +1984,11 @@
       <c r="M22" s="3" t="inlineStr">
         <is>
           <t>2c9b9f339</t>
+        </is>
+      </c>
+      <c r="N22" s="8" t="inlineStr">
+        <is>
+          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
         </is>
       </c>
     </row>
@@ -1923,7 +2041,7 @@
           <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
         </is>
       </c>
-      <c r="K23" s="11" t="inlineStr">
+      <c r="K23" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -1936,6 +2054,11 @@
       <c r="M23" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
         </is>
       </c>
     </row>
@@ -1988,7 +2111,7 @@
           <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
         </is>
       </c>
-      <c r="K24" s="11" t="inlineStr">
+      <c r="K24" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2001,6 +2124,11 @@
       <c r="M24" s="3" t="inlineStr">
         <is>
           <t>0574c60d4</t>
+        </is>
+      </c>
+      <c r="N24" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2181,7 @@
           <t>Gate for everything below — do not proceed if numbers diverge. · verified inline against cache/portfolio_backtest_750d_20260509_100501.json: TC@score&gt;=80 PF 0.54, VCP@score&gt;=80 n=1, Near-VCP@score&gt;=80 PF 1.05, 90-100 band PF 0.55</t>
         </is>
       </c>
-      <c r="K25" s="11" t="inlineStr">
+      <c r="K25" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2066,6 +2194,11 @@
       <c r="M25" s="3" t="inlineStr">
         <is>
           <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>python3 -c 'import json; d=json.load(open("cache/portfolio_backtest_750d_20260509_100501.json")); print(d["profit_factor"])' → 0.70 confirmed.</t>
         </is>
       </c>
     </row>
@@ -2118,7 +2251,7 @@
           <t>Lesson: filter to 'what new config would have allowed' before extrapolating.</t>
         </is>
       </c>
-      <c r="K26" s="11" t="inlineStr">
+      <c r="K26" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2131,6 +2264,11 @@
       <c r="M26" s="3" t="inlineStr">
         <is>
           <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N26" s="8" t="inlineStr">
+        <is>
+          <t>grep -A5 '"VCP Breakout"' config/config.json → setup_score_multiplier shows 0.0 (was 1.2). git diff confirms revert.</t>
         </is>
       </c>
     </row>
@@ -2183,7 +2321,7 @@
           <t>PF 1.07 has wide CI 0.85-1.30 OOS. Verify with Q1-step4 250d backtest.</t>
         </is>
       </c>
-      <c r="K27" s="11" t="inlineStr">
+      <c r="K27" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2196,6 +2334,11 @@
       <c r="M27" s="3" t="inlineStr">
         <is>
           <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>grep -A5 '"Near-VCP Breakout"' config/config.json → setup_score_multiplier shows 1.0 (was 0.7).</t>
         </is>
       </c>
     </row>
@@ -2248,7 +2391,7 @@
           <t>Pure additive. Does not affect existing analysis.</t>
         </is>
       </c>
-      <c r="K28" s="11" t="inlineStr">
+      <c r="K28" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2261,6 +2404,11 @@
       <c r="M28" s="3" t="inlineStr">
         <is>
           <t>f35f0c124</t>
+        </is>
+      </c>
+      <c r="N28" s="8" t="inlineStr">
+        <is>
+          <t>Run a fresh backtest (after current finishes). Open cache/portfolio_backtest_*.json → trade records contain regime, entry_quality, sector, mae_pct, mfe_pct fields.</t>
         </is>
       </c>
     </row>
@@ -2313,7 +2461,7 @@
           <t>Bug fix in 6ceca2d18: bare-string kill_list entries silently rejected — required dict format.</t>
         </is>
       </c>
-      <c r="K29" s="11" t="inlineStr">
+      <c r="K29" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2326,6 +2474,11 @@
       <c r="M29" s="3" t="inlineStr">
         <is>
           <t>fc76c9ec8 + 6ceca2d18</t>
+        </is>
+      </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>grep -A5 'static_setup_kill_list' config/config.json → 'Trend Continuation' present in dict format with n=264 wr_lb=0.195.</t>
         </is>
       </c>
     </row>
@@ -2378,7 +2531,7 @@
           <t>REVERT CANDIDATE. Sunday plan step 2: revert to 0.0.</t>
         </is>
       </c>
-      <c r="K30" s="11" t="inlineStr">
+      <c r="K30" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2391,6 +2544,11 @@
       <c r="M30" s="3" t="inlineStr">
         <is>
           <t>fc76c9ec8</t>
+        </is>
+      </c>
+      <c r="N30" s="8" t="inlineStr">
+        <is>
+          <t>Same as Q1-step2 verification — VCP Breakout multiplier should NOW be 0.0 (reverted from Saturday's 1.2).</t>
         </is>
       </c>
     </row>
@@ -2443,7 +2601,7 @@
           <t>Longs only. Sanity-bounded to prevent bad fractal detection from blowing out stops.</t>
         </is>
       </c>
-      <c r="K31" s="11" t="inlineStr">
+      <c r="K31" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2456,6 +2614,11 @@
       <c r="M31" s="3" t="inlineStr">
         <is>
           <t>3d4eb71d7</t>
+        </is>
+      </c>
+      <c r="N31" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py deep AAPL → check that stop value ≤ indicators.fractal_low (or within 0.10×ATR buffer below it). NEVER above fractal_low.</t>
         </is>
       </c>
     </row>
@@ -2508,7 +2671,7 @@
           <t>Flip config['signal_filter']['_enabled']=true after per-subtype A5 attribution review.</t>
         </is>
       </c>
-      <c r="K32" s="11" t="inlineStr">
+      <c r="K32" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2521,6 +2684,11 @@
       <c r="M32" s="3" t="inlineStr">
         <is>
           <t>4129e5565</t>
+        </is>
+      </c>
+      <c r="N32" s="8" t="inlineStr">
+        <is>
+          <t>1) cat config/config.json | grep -A3 signal_filter → confirm _enabled=false. 2) Toggle to true via --config-override → run scan → BUY count drops. Toggle off → restored.</t>
         </is>
       </c>
     </row>
@@ -2573,7 +2741,7 @@
           <t>Existing positions unaffected (exits run via separate paths).</t>
         </is>
       </c>
-      <c r="K33" s="11" t="inlineStr">
+      <c r="K33" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2586,6 +2754,11 @@
       <c r="M33" s="3" t="inlineStr">
         <is>
           <t>1e40d30fc</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
+          <t>Run scan during simulated risk_off regime (set regime via --config-override) → confirm zero BUY verdicts emitted. Audit gate 'regime_gate' marked failed.</t>
         </is>
       </c>
     </row>
@@ -2598,7 +2771,7 @@
           <t>B1</t>
         </is>
       </c>
-      <c r="C34" s="8" t="inlineStr">
+      <c r="C34" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2638,7 +2811,7 @@
           <t>Fix deferred until standalone 750d backtest finishes.</t>
         </is>
       </c>
-      <c r="K34" s="11" t="inlineStr">
+      <c r="K34" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2651,6 +2824,11 @@
       <c r="M34" s="3" t="inlineStr">
         <is>
           <t>9bc015562</t>
+        </is>
+      </c>
+      <c r="N34" s="8" t="inlineStr">
+        <is>
+          <t>cat diagnose_as_of_membership.py output OR re-run: python3 diagnose_as_of_membership.py → '88.3% OHLCV coverage' confirmed; bug elsewhere in pipeline.</t>
         </is>
       </c>
     </row>
@@ -2663,7 +2841,7 @@
           <t>G3</t>
         </is>
       </c>
-      <c r="C35" s="8" t="inlineStr">
+      <c r="C35" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2703,7 +2881,7 @@
           <t>A7 dashboard tile not yet built — registry has the data when needed.</t>
         </is>
       </c>
-      <c r="K35" s="11" t="inlineStr">
+      <c r="K35" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2716,6 +2894,11 @@
       <c r="M35" s="3" t="inlineStr">
         <is>
           <t>4129e5565</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>psql or Supabase Studio → confirm signal_filter_decisions table exists + signal_filter_drift_30d view returns query plan.</t>
         </is>
       </c>
     </row>
@@ -2728,7 +2911,7 @@
           <t>F11</t>
         </is>
       </c>
-      <c r="C36" s="8" t="inlineStr">
+      <c r="C36" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2768,7 +2951,7 @@
           <t>8 pre-existing JSON-only fields documented as tech debt.</t>
         </is>
       </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="K36" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2781,6 +2964,11 @@
       <c r="M36" s="3" t="inlineStr">
         <is>
           <t>1e40d30fc</t>
+        </is>
+      </c>
+      <c r="N36" s="8" t="inlineStr">
+        <is>
+          <t>Stage a JSON change with NEW key. git commit → hook fires drift check on NEW key only (not full repo). Pre-existing drift not blocking.</t>
         </is>
       </c>
     </row>
@@ -2793,7 +2981,7 @@
           <t>PERF-4</t>
         </is>
       </c>
-      <c r="C37" s="8" t="inlineStr">
+      <c r="C37" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2833,7 +3021,7 @@
           <t>Verify Cloudflare tunnel doesn't strip br encoding.</t>
         </is>
       </c>
-      <c r="K37" s="11" t="inlineStr">
+      <c r="K37" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2846,6 +3034,11 @@
       <c r="M37" s="3" t="inlineStr">
         <is>
           <t>2eb4e3b3d</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>Browser DevTools → Network tab → reload dashboard → Content-Encoding header on data.json reads 'br' (Brotli) when supported, else 'gzip'.</t>
         </is>
       </c>
     </row>
@@ -2858,7 +3051,7 @@
           <t>PERF-5</t>
         </is>
       </c>
-      <c r="C38" s="8" t="inlineStr">
+      <c r="C38" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2898,7 +3091,7 @@
           <t>Trivial fix; verify no race with first user interaction.</t>
         </is>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="K38" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2911,6 +3104,11 @@
       <c r="M38" s="3" t="inlineStr">
         <is>
           <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N38" s="8" t="inlineStr">
+        <is>
+          <t>Browser DevTools → Performance → reload dashboard → _capScanAndDisableButtons fires AFTER init-end (in idle callback), not during sync init.</t>
         </is>
       </c>
     </row>
@@ -2923,7 +3121,7 @@
           <t>A5</t>
         </is>
       </c>
-      <c r="C39" s="8" t="inlineStr">
+      <c r="C39" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2963,7 +3161,7 @@
           <t>A5-followup wired the meta-family Wilson rule into signal_filter (status DRAFT until subtype attribution).</t>
         </is>
       </c>
-      <c r="K39" s="11" t="inlineStr">
+      <c r="K39" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -2976,6 +3174,11 @@
       <c r="M39" s="3" t="inlineStr">
         <is>
           <t>1e40d30fc</t>
+        </is>
+      </c>
+      <c r="N39" s="8" t="inlineStr">
+        <is>
+          <t>Open cache/catalyst_decomposition_2026-05-09.html → see ranked sub-strategies. Top survivor: 'pullback excl. Breakout/TC' n=134 WR 53% PF 1.83.</t>
         </is>
       </c>
     </row>
@@ -2988,7 +3191,7 @@
           <t>K1</t>
         </is>
       </c>
-      <c r="C40" s="8" t="inlineStr">
+      <c r="C40" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3028,7 +3231,7 @@
           <t>Longs only. Try/except wrapped — never fails trade_plan.</t>
         </is>
       </c>
-      <c r="K40" s="11" t="inlineStr">
+      <c r="K40" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3041,6 +3244,11 @@
       <c r="M40" s="3" t="inlineStr">
         <is>
           <t>3d4eb71d7</t>
+        </is>
+      </c>
+      <c r="N40" s="8" t="inlineStr">
+        <is>
+          <t>Run: python3 swing_trade.py deep HPE → Plan tab → confirm stop is near a Fib retracement OR EMA50 (within 1%). Should NOT be a flat 1.25×ATR distance.</t>
         </is>
       </c>
     </row>
@@ -3053,7 +3261,7 @@
           <t>K2</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C41" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3093,7 +3301,7 @@
           <t>Vinod said 'hard check' but blocking would over-fire — flag is right level.</t>
         </is>
       </c>
-      <c r="K41" s="11" t="inlineStr">
+      <c r="K41" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3106,6 +3314,11 @@
       <c r="M41" s="3" t="inlineStr">
         <is>
           <t>3d4eb71d7</t>
+        </is>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>Find a ticker where VWAP &lt; stop. Run: python3 swing_trade.py deep &lt;TICKER&gt; → Plan tab → confirm risk_flags includes 'vwap_below_stop' with severity=high.</t>
         </is>
       </c>
     </row>
@@ -3118,7 +3331,7 @@
           <t>K5</t>
         </is>
       </c>
-      <c r="C42" s="8" t="inlineStr">
+      <c r="C42" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3158,7 +3371,7 @@
           <t>Wave 2 corrective + low-confidence Wave 3 informational only — don't override default targets.</t>
         </is>
       </c>
-      <c r="K42" s="11" t="inlineStr">
+      <c r="K42" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3171,6 +3384,11 @@
       <c r="M42" s="3" t="inlineStr">
         <is>
           <t>302e9ea00</t>
+        </is>
+      </c>
+      <c r="N42" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py deep HPE → Models tab → Elliott section shows wave=3, type=impulse, T1/T2 as Fib extensions (1.272×, 1.618× of swing).</t>
         </is>
       </c>
     </row>
@@ -3183,7 +3401,7 @@
           <t>K4</t>
         </is>
       </c>
-      <c r="C43" s="8" t="inlineStr">
+      <c r="C43" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3223,7 +3441,7 @@
           <t>Score weight pending 30-day signal corpus + backtest validation.</t>
         </is>
       </c>
-      <c r="K43" s="11" t="inlineStr">
+      <c r="K43" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3236,6 +3454,11 @@
       <c r="M43" s="3" t="inlineStr">
         <is>
           <t>PENDING</t>
+        </is>
+      </c>
+      <c r="N43" s="8" t="inlineStr">
+        <is>
+          <t>python3 swing_trade.py deep AAPL → Technicals tab → confirm EMA 5 and EMA 13 both display with current values. ema5_above_13 boolean visible.</t>
         </is>
       </c>
     </row>
@@ -3248,7 +3471,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C44" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3288,7 +3511,7 @@
           <t>Additive — only renders if #driftBody container exists in DOM.</t>
         </is>
       </c>
-      <c r="K44" s="11" t="inlineStr">
+      <c r="K44" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3301,6 +3524,11 @@
       <c r="M44" s="3" t="inlineStr">
         <is>
           <t>16a26b201</t>
+        </is>
+      </c>
+      <c r="N44" s="8" t="inlineStr">
+        <is>
+          <t>Open https://localhost:7432/dashboard → Status tab → drift tile renders. If no drift_alerts.jsonl yet, shows 'No drift alerts yet'. Else shows per-setup Δ pp.</t>
         </is>
       </c>
     </row>
@@ -3313,7 +3541,7 @@
           <t>MOD-3</t>
         </is>
       </c>
-      <c r="C45" s="8" t="inlineStr">
+      <c r="C45" s="9" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3353,7 +3581,7 @@
           <t>Trivial.</t>
         </is>
       </c>
-      <c r="K45" s="11" t="inlineStr">
+      <c r="K45" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3366,6 +3594,11 @@
       <c r="M45" s="3" t="inlineStr">
         <is>
           <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N45" s="8" t="inlineStr">
+        <is>
+          <t>open tests/README.md → SWING_USER + SWING_PASS env var docs. SWING_USER=foo SWING_PASS=bar npx playwright test runs auth suite.</t>
         </is>
       </c>
     </row>
@@ -3378,7 +3611,7 @@
           <t>J1</t>
         </is>
       </c>
-      <c r="C46" s="9" t="inlineStr">
+      <c r="C46" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3414,7 +3647,7 @@
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr"/>
-      <c r="K46" s="11" t="inlineStr">
+      <c r="K46" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3427,6 +3660,11 @@
       <c r="M46" s="3" t="inlineStr">
         <is>
           <t>1e40d30fc</t>
+        </is>
+      </c>
+      <c r="N46" s="8" t="inlineStr">
+        <is>
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3677,7 @@
           <t>J2</t>
         </is>
       </c>
-      <c r="C47" s="9" t="inlineStr">
+      <c r="C47" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3479,7 +3717,7 @@
           <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
         </is>
       </c>
-      <c r="K47" s="11" t="inlineStr">
+      <c r="K47" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3492,6 +3730,11 @@
       <c r="M47" s="3" t="inlineStr">
         <is>
           <t>d8c08399b</t>
+        </is>
+      </c>
+      <c r="N47" s="8" t="inlineStr">
+        <is>
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
         </is>
       </c>
     </row>
@@ -3504,7 +3747,7 @@
           <t>J3</t>
         </is>
       </c>
-      <c r="C48" s="9" t="inlineStr">
+      <c r="C48" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3540,7 +3783,7 @@
         </is>
       </c>
       <c r="J48" s="5" t="inlineStr"/>
-      <c r="K48" s="11" t="inlineStr">
+      <c r="K48" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3553,6 +3796,11 @@
       <c r="M48" s="3" t="inlineStr">
         <is>
           <t>4129e5565</t>
+        </is>
+      </c>
+      <c r="N48" s="8" t="inlineStr">
+        <is>
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
         </is>
       </c>
     </row>
@@ -3565,7 +3813,7 @@
           <t>F11-followup</t>
         </is>
       </c>
-      <c r="C49" s="9" t="inlineStr">
+      <c r="C49" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3605,7 +3853,7 @@
           <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
-      <c r="K49" s="11" t="inlineStr">
+      <c r="K49" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3620,8 +3868,13 @@
           <t>1e40d30fc</t>
         </is>
       </c>
-    </row>
-    <row r="50" ht="45" customHeight="1">
+      <c r="N49" s="8" t="inlineStr">
+        <is>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
@@ -3630,7 +3883,7 @@
           <t>OPS-5</t>
         </is>
       </c>
-      <c r="C50" s="9" t="inlineStr">
+      <c r="C50" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3670,7 +3923,7 @@
           <t>Trivial CLI wrapper.</t>
         </is>
       </c>
-      <c r="K50" s="11" t="inlineStr">
+      <c r="K50" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3683,6 +3936,11 @@
       <c r="M50" s="3" t="inlineStr">
         <is>
           <t>2b7d2f40f</t>
+        </is>
+      </c>
+      <c r="N50" s="8" t="inlineStr">
+        <is>
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3953,7 @@
           <t>B4</t>
         </is>
       </c>
-      <c r="C51" s="12" t="inlineStr">
+      <c r="C51" s="13" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -3735,7 +3993,7 @@
           <t>3 snapshot files present. Validates cb1f5a010.</t>
         </is>
       </c>
-      <c r="K51" s="11" t="inlineStr">
+      <c r="K51" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3746,6 +4004,11 @@
         </is>
       </c>
       <c r="M51" s="3" t="inlineStr"/>
+      <c r="N51" s="8" t="inlineStr">
+        <is>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="45" customHeight="1">
       <c r="A52" s="2" t="n">
@@ -3756,7 +4019,7 @@
           <t>I4</t>
         </is>
       </c>
-      <c r="C52" s="12" t="inlineStr">
+      <c r="C52" s="13" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -3796,7 +4059,7 @@
           <t>7 backup dirs present, latest 2026-05-08.</t>
         </is>
       </c>
-      <c r="K52" s="11" t="inlineStr">
+      <c r="K52" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
@@ -3807,6 +4070,11 @@
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr"/>
+      <c r="N52" s="8" t="inlineStr">
+        <is>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="45" customHeight="1">
       <c r="A53" s="2" t="n">
@@ -3817,7 +4085,7 @@
           <t>CLEAN-2</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
+      <c r="C53" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3857,13 +4125,18 @@
           <t>Standard data-migration retention practice.</t>
         </is>
       </c>
-      <c r="K53" s="13" t="inlineStr">
+      <c r="K53" s="14" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
       </c>
       <c r="L53" s="2" t="inlineStr"/>
       <c r="M53" s="3" t="inlineStr"/>
+      <c r="N53" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="45" customHeight="1">
       <c r="A54" s="2" t="n">
@@ -3874,7 +4147,7 @@
           <t>MOB-1</t>
         </is>
       </c>
-      <c r="C54" s="9" t="inlineStr">
+      <c r="C54" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3910,13 +4183,18 @@
           <t>Deferred — desktop is primary use case.</t>
         </is>
       </c>
-      <c r="K54" s="13" t="inlineStr">
+      <c r="K54" s="14" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
       </c>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="3" t="inlineStr"/>
+      <c r="N54" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="45" customHeight="1">
       <c r="A55" s="2" t="n">
@@ -3927,7 +4205,7 @@
           <t>MOB-2</t>
         </is>
       </c>
-      <c r="C55" s="9" t="inlineStr">
+      <c r="C55" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -3963,13 +4241,18 @@
           <t>Deferred indefinitely.</t>
         </is>
       </c>
-      <c r="K55" s="13" t="inlineStr">
+      <c r="K55" s="14" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
       </c>
       <c r="L55" s="2" t="inlineStr"/>
       <c r="M55" s="3" t="inlineStr"/>
+      <c r="N55" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="45" customHeight="1">
       <c r="A56" s="2" t="n">
@@ -3980,7 +4263,7 @@
           <t>PERF-8-13</t>
         </is>
       </c>
-      <c r="C56" s="9" t="inlineStr">
+      <c r="C56" s="10" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4020,13 +4303,18 @@
           <t>Don't pre-implement.</t>
         </is>
       </c>
-      <c r="K56" s="13" t="inlineStr">
+      <c r="K56" s="14" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
       </c>
       <c r="L56" s="2" t="inlineStr"/>
       <c r="M56" s="3" t="inlineStr"/>
+      <c r="N56" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="45" customHeight="1">
       <c r="A57" s="2" t="n">
@@ -4077,13 +4365,18 @@
           <t>Agents skim and miss post-filter subset analysis.</t>
         </is>
       </c>
-      <c r="K57" s="14" t="inlineStr">
+      <c r="K57" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="3" t="inlineStr"/>
+      <c r="N57" s="8" t="inlineStr">
+        <is>
+          <t>n/a — rejected</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="90" customHeight="1">
       <c r="A58" s="2" t="n">
@@ -4094,7 +4387,7 @@
           <t>H1</t>
         </is>
       </c>
-      <c r="C58" s="12" t="inlineStr">
+      <c r="C58" s="13" t="inlineStr">
         <is>
           <t>P3</t>
         </is>
@@ -4134,7 +4427,7 @@
           <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
         </is>
       </c>
-      <c r="K58" s="14" t="inlineStr">
+      <c r="K58" s="15" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
@@ -4145,6 +4438,11 @@
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr"/>
+      <c r="N58" s="8" t="inlineStr">
+        <is>
+          <t>n/a — rejected</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -4168,143 +4466,143 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="15" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B1" s="15" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="C1" s="15" t="inlineStr">
+      <c r="C1" s="16" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="D1" s="15" t="inlineStr">
+      <c r="D1" s="16" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E1" s="15" t="inlineStr">
+      <c r="E1" s="16" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="16" t="inlineStr">
+      <c r="A2" s="17" t="inlineStr">
         <is>
           <t>OPEN</t>
         </is>
       </c>
-      <c r="B2" s="17" t="n">
+      <c r="B2" s="18" t="n">
         <v>3</v>
       </c>
-      <c r="C2" s="17" t="n">
+      <c r="C2" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D2" s="17" t="n">
+      <c r="D2" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="E2" s="17" t="n">
+      <c r="E2" s="18" t="n">
         <v>18</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="18" t="inlineStr">
+      <c r="A3" s="19" t="inlineStr">
         <is>
           <t>IN_PROGRESS</t>
         </is>
       </c>
-      <c r="B3" s="17" t="n">
+      <c r="B3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C3" s="17" t="n">
+      <c r="C3" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="D3" s="17" t="n">
+      <c r="D3" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E3" s="17" t="n">
+      <c r="E3" s="18" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="19" t="inlineStr">
+      <c r="A4" s="20" t="inlineStr">
         <is>
           <t>DONE</t>
         </is>
       </c>
-      <c r="B4" s="17" t="n">
+      <c r="B4" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="C4" s="17" t="n">
+      <c r="C4" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="D4" s="17" t="n">
+      <c r="D4" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="E4" s="17" t="n">
+      <c r="E4" s="18" t="n">
         <v>29</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="inlineStr">
+      <c r="A5" s="21" t="inlineStr">
         <is>
           <t>DEFERRED</t>
         </is>
       </c>
-      <c r="B5" s="17" t="n">
+      <c r="B5" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="17" t="n">
+      <c r="C5" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="17" t="n">
+      <c r="D5" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="E5" s="17" t="n">
+      <c r="E5" s="18" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
+      <c r="A6" s="22" t="inlineStr">
         <is>
           <t>REJECTED</t>
         </is>
       </c>
-      <c r="B6" s="17" t="n">
+      <c r="B6" s="18" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="17" t="n">
+      <c r="C6" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="17" t="n">
+      <c r="D6" s="18" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="17" t="n">
+      <c r="E6" s="18" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="22" t="inlineStr">
+      <c r="A7" s="23" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B7" s="22" t="n">
+      <c r="B7" s="23" t="n">
         <v>17</v>
       </c>
-      <c r="C7" s="22" t="n">
+      <c r="C7" s="23" t="n">
         <v>23</v>
       </c>
-      <c r="D7" s="22" t="n">
+      <c r="D7" s="23" t="n">
         <v>14</v>
       </c>
-      <c r="E7" s="22" t="n">
+      <c r="E7" s="23" t="n">
         <v>57</v>
       </c>
     </row>
@@ -4328,153 +4626,153 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="23" t="inlineStr">
+      <c r="A1" s="24" t="inlineStr">
         <is>
           <t>Step</t>
         </is>
       </c>
-      <c r="B1" s="23" t="inlineStr">
+      <c r="B1" s="24" t="inlineStr">
         <is>
           <t>Command</t>
         </is>
       </c>
-      <c r="C1" s="23" t="inlineStr">
+      <c r="C1" s="24" t="inlineStr">
         <is>
           <t>What it does</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="24" t="inlineStr">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B2" s="25" t="inlineStr">
+      <c r="B2" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py list</t>
         </is>
       </c>
-      <c r="C2" s="26" t="inlineStr">
+      <c r="C2" s="27" t="inlineStr">
         <is>
           <t>Show all items grouped by status</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="24" t="inlineStr">
+      <c r="A3" s="25" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="B3" s="25" t="inlineStr">
+      <c r="B3" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py list --open</t>
         </is>
       </c>
-      <c r="C3" s="26" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>Show only OPEN / IN_PROGRESS</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="25" t="inlineStr">
         <is>
           <t>3</t>
         </is>
       </c>
-      <c r="B4" s="25" t="inlineStr">
+      <c r="B4" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py done &lt;id&gt;</t>
         </is>
       </c>
-      <c r="C4" s="26" t="inlineStr">
+      <c r="C4" s="27" t="inlineStr">
         <is>
           <t>Mark item DONE (auto-fills today's date + HEAD commit)</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="24" t="inlineStr">
+      <c r="A5" s="25" t="inlineStr">
         <is>
           <t>4</t>
         </is>
       </c>
-      <c r="B5" s="25" t="inlineStr">
+      <c r="B5" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py done &lt;id&gt; --commit abc123 --date 2026-05-09</t>
         </is>
       </c>
-      <c r="C5" s="26" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Mark DONE with explicit commit/date</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="A6" s="25" t="inlineStr">
         <is>
           <t>5</t>
         </is>
       </c>
-      <c r="B6" s="25" t="inlineStr">
+      <c r="B6" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py status &lt;id&gt; IN_PROGRESS</t>
         </is>
       </c>
-      <c r="C6" s="26" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>Set arbitrary status (OPEN/IN_PROGRESS/DONE/DEFERRED/REJECTED)</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="24" t="inlineStr">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>6</t>
         </is>
       </c>
-      <c r="B7" s="25" t="inlineStr">
+      <c r="B7" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py add NEW-ID P1 "Section" "Item title" "What" "How"</t>
         </is>
       </c>
-      <c r="C7" s="26" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Add a new item to the registry</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="24" t="inlineStr">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>7</t>
         </is>
       </c>
-      <c r="B8" s="25" t="inlineStr">
+      <c r="B8" s="26" t="inlineStr">
         <is>
           <t>python3 scripts/update_open_items.py xlsx</t>
         </is>
       </c>
-      <c r="C8" s="26" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>Regenerate this Excel from data/open_items.json</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="24" t="inlineStr">
+      <c r="A9" s="25" t="inlineStr">
         <is>
           <t>8</t>
         </is>
       </c>
-      <c r="B9" s="25" t="inlineStr">
+      <c r="B9" s="26" t="inlineStr">
         <is>
           <t>edit data/open_items.json directly, then run xlsx</t>
         </is>
       </c>
-      <c r="C9" s="26" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Free-form edits — works too</t>
         </is>

</xml_diff>

<commit_message>
Open items: add MOD-A + MOD-B, document Q1-step5 acceptance failure
Two new umbrella entries marked DONE for tonight's frontend modularization:

  MOD-A · Phase A — split 5 main tabs into 28 sub-modules
    commits 9517bbbe9, 0d035d6cd, 733342cd3, cf5e0bb92, 7229d4ccb
    (performance / audit / elite / earnings / strategies)

  MOD-B · Phase B — split 5 elite-detail subtabs into 17 sub-modules
    commits 18ef1002e, 5c3497e6f, cb167a47b, 2a767ac98, 388c316c4
    (ruleengine / smc / insider / options / sentiment)

Q1-step5 notes refreshed with FAILED ACCEPTANCE BAR finding from 250d
backtest (0 BUYs over 3+ simulated months). Recovery path filed:
Variant F (f0a66543e) — regime-conditional TC kill in bull regime only;
verification still pending before declaring fix.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-10.xlsx
+++ b/cache/open_items_2026-05-10.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N63"/>
+  <dimension ref="A1:N65"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1684,7 +1684,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="105" customHeight="1">
+    <row r="17" ht="180" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
@@ -1730,7 +1730,7 @@
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first.</t>
+          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first. / FAILED ACCEPTANCE BAR (2026-05-10): 250d backtest produced 0 BUYs across 3+ simulated months. Q1 multipliers + threshold combo demoted every qualifying signal. Sibling commit a18282d28 (Q1-step5 250d FINAL) logged the failure; recovery path was Variant F (commit f0a66543e) — regime-conditional TC kill ONLY in bull regime (not all 4 regimes). 250d Variant F backtest pending verification before declaring real fix.</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
@@ -3916,51 +3916,47 @@
         </is>
       </c>
     </row>
-    <row r="49" ht="60" customHeight="1">
+    <row r="49" ht="105" customHeight="1">
       <c r="A49" s="2" t="n">
         <v>48</v>
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="C49" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-A</t>
+        </is>
+      </c>
+      <c r="C49" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md with new tools</t>
+          <t>Split 5 main tabs into sub-function modules (Phase A)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
+          <t>5 main-tab folders were each single .js files with multiple visual sections crammed together (performance 366 ln, audit 505, elite 370, earnings 278, strategies 224 = 1,743 ln total). Hard to navigate, hard to test sub-renderers in isolation, and bare-DATA references in audit had been silently broken since the 2026-05-09 extraction.</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
-        </is>
-      </c>
-      <c r="H49" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I49" s="5" t="inlineStr">
-        <is>
-          <t>Win: future Claude sessions discover new tools.</t>
-        </is>
-      </c>
-      <c r="J49" s="5" t="inlineStr"/>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 4-7 focused sub-modules per folder. 28 new sub-files total. Bug fixes folded in where bare-DATA / bare-$ references would ReferenceError. Each tab passes node --check; window bindings preserved exactly.</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="5" t="inlineStr"/>
+      <c r="J49" s="5" t="inlineStr">
+        <is>
+          <t>Phase A — main tabs split. Commits 9517bbbe9 (perf, 8 files), 0d035d6cd (audit, 7 files), 733342cd3 (elite, 6 files), cf5e0bb92 (earnings, 5 files), 7229d4ccb (strategies, 5 files). 28 new sub-files; net +311 lines from per-module imports/exports — that's the price of single-responsibility. Audit-tab bare-DATA ReferenceError fixed in expand_panel.js + exports.js.</t>
+        </is>
+      </c>
       <c r="K49" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -3968,67 +3964,59 @@
       </c>
       <c r="L49" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>9517bbbe9..7229d4ccb</t>
         </is>
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
-          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="75" customHeight="1">
+          <t>1. ls infra/prototype/tabs/{performance,audit,elite,earnings,strategies}/*.js → expect 8/7/6/5/5 files per folder. 2. Open https://trade.mystockholding.com/v2/dashboard.html — click each of the 5 tabs, verify they render identically to before the split. 3. node --check infra/prototype/tabs/*/*.js → all pass. 4. Click an audit row to expand the detail panel (was silently broken before — bare-DATA bug now fixed). 5. Click Export CSV in audit (was also broken).</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="105" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
-        </is>
-      </c>
-      <c r="C50" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-B</t>
+        </is>
+      </c>
+      <c r="C50" s="9" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
+          <t>Split 5 elite-detail subtabs into sub-function modules (Phase B)</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
+          <t>5 subtab folders were single .js files (ruleengine 531 ln, smc 414, insider 256, options 245, sentiment 203 = 1,649 ln). Bare-$ references in smc/options/sentiment had silent ReferenceErrors since 2026-05-09 extraction. _renderShortPressureCard reference unguarded.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I50" s="5" t="inlineStr">
-        <is>
-          <t>Win: clear activation procedure before flipping live.</t>
-        </is>
-      </c>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 2-3 focused sub-modules per folder. 17 new sub-files total. Bare-$ → document.getElementById fixed. _renderShortPressureCard wrapped in typeof guard. All files pass node --check.</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="inlineStr">
         <is>
-          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
+          <t>Phase B — elite-detail subtabs split. Commits 18ef1002e (ruleengine, 4 files), 5c3497e6f (smc, 4 files), cb167a47b (insider, 3 files), 2a767ac98 (options, 3 files), 388c316c4 (sentiment, 3 files). 17 new sub-files. 5 latent ReferenceErrors fixed (audit fixed in MOD-A, smc/options/sentiment bare-$, sentiment _renderShortPressureCard guard). Sibling 40f8452b8 layered 8-gate cascade view onto ruleengine pipeline.js post-split.</t>
         </is>
       </c>
       <c r="K50" s="12" t="inlineStr">
@@ -4038,27 +4026,27 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>18ef1002e..388c316c4</t>
         </is>
       </c>
       <c r="N50" s="8" t="inlineStr">
         <is>
-          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="45" customHeight="1">
+          <t>1. ls infra/prototype/subtabs/{ruleengine,smc,insider,options,sentiment}/*.js → expect 4/4/3/3/3 files per folder. 2. Open elite-detail.html?t=NVDA → click through Why-this-is-X, SMC, Insider, Options, Sentiment subtabs — each renders identically. 3. node --check infra/prototype/subtabs/*/*.js → all pass. 4. SMC subtab now actually renders (was silently broken — bare-$ ReferenceError). 5. Options + Sentiment same fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="60" customHeight="1">
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C51" s="10" t="inlineStr">
@@ -4068,22 +4056,22 @@
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Git committer.email set globally</t>
+          <t>Update CLAUDE.md with new tools</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
+          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
+          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -4093,7 +4081,7 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Win: clean attribution in git log.</t>
+          <t>Win: future Claude sessions discover new tools.</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr"/>
@@ -4109,12 +4097,12 @@
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
-          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
         </is>
       </c>
     </row>
@@ -4124,7 +4112,7 @@
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C52" s="10" t="inlineStr">
@@ -4134,22 +4122,22 @@
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
+          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4159,12 +4147,12 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
+          <t>Win: clear activation procedure before flipping live.</t>
         </is>
       </c>
       <c r="J52" s="5" t="inlineStr">
         <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
+          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
         </is>
       </c>
       <c r="K52" s="12" t="inlineStr">
@@ -4179,22 +4167,22 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N52" s="8" t="inlineStr">
         <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="60" customHeight="1">
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="45" customHeight="1">
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C53" s="10" t="inlineStr">
@@ -4204,39 +4192,35 @@
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Git committer.email set globally</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr">
-        <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
-        </is>
-      </c>
+          <t>Win: clean attribution in git log.</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr"/>
       <c r="K53" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4244,27 +4228,27 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="60" customHeight="1">
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="75" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C54" s="10" t="inlineStr">
@@ -4274,37 +4258,37 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K54" s="12" t="inlineStr">
@@ -4314,17 +4298,17 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
         </is>
       </c>
     </row>
@@ -4334,7 +4318,7 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C55" s="10" t="inlineStr">
@@ -4349,32 +4333,32 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K55" s="12" t="inlineStr">
@@ -4394,7 +4378,7 @@
       </c>
       <c r="N55" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -4404,7 +4388,7 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C56" s="10" t="inlineStr">
@@ -4419,32 +4403,32 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K56" s="12" t="inlineStr">
@@ -4454,27 +4438,27 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N56" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="150" customHeight="1">
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="60" customHeight="1">
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OPS-4</t>
         </is>
       </c>
       <c r="C57" s="10" t="inlineStr">
@@ -4484,29 +4468,37 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
-        </is>
-      </c>
-      <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="5" t="inlineStr"/>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr">
+        <is>
+          <t>2 hrs</t>
+        </is>
+      </c>
+      <c r="I57" s="5" t="inlineStr">
+        <is>
+          <t>Win: visibility into RBAC changes.</t>
+        </is>
+      </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K57" s="12" t="inlineStr">
@@ -4521,62 +4513,62 @@
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N57" s="8" t="inlineStr">
         <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C58" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>OPS-5</t>
+        </is>
+      </c>
+      <c r="C58" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I58" s="5" t="inlineStr">
         <is>
-          <t>Win: persistence works; no silent overwrites.</t>
+          <t>Win: fast iteration on report templates.</t>
         </is>
       </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
+          <t>Trivial CLI wrapper.</t>
         </is>
       </c>
       <c r="K58" s="12" t="inlineStr">
@@ -4589,60 +4581,56 @@
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="M58" s="3" t="inlineStr"/>
+      <c r="M58" s="3" t="inlineStr">
+        <is>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
       <c r="N58" s="8" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="45" customHeight="1">
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="150" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="C59" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>PERF-7b</t>
+        </is>
+      </c>
+      <c r="C59" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr">
-        <is>
-          <t>verified (no change needed)</t>
-        </is>
-      </c>
-      <c r="I59" s="5" t="inlineStr">
-        <is>
-          <t>Win: confirms infrastructure still healthy.</t>
-        </is>
-      </c>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="5" t="inlineStr"/>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
         </is>
       </c>
       <c r="K59" s="12" t="inlineStr">
@@ -4652,13 +4640,17 @@
       </c>
       <c r="L59" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M59" s="3" t="inlineStr"/>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr">
+        <is>
+          <t>cf30df858</t>
+        </is>
+      </c>
       <c r="N59" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
         </is>
       </c>
     </row>
@@ -4668,59 +4660,63 @@
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
-        </is>
-      </c>
-      <c r="C60" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="C60" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>5 min after answer</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Win: -671 lines.</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K60" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L60" s="2" t="inlineStr"/>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
+        </is>
+      </c>
+      <c r="K60" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
       <c r="M60" s="3" t="inlineStr"/>
       <c r="N60" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
         </is>
       </c>
     </row>
@@ -4730,59 +4726,63 @@
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
-        </is>
-      </c>
-      <c r="C61" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>I4</t>
+        </is>
+      </c>
+      <c r="C61" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Win: confirms infrastructure still healthy.</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
-        </is>
-      </c>
-      <c r="K61" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L61" s="2" t="inlineStr"/>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
+      <c r="K61" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
       <c r="M61" s="3" t="inlineStr"/>
       <c r="N61" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
         </is>
       </c>
     </row>
@@ -4792,123 +4792,247 @@
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C62" s="4" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>CLEAN-2</t>
+        </is>
+      </c>
+      <c r="C62" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>5 min after answer</t>
         </is>
       </c>
       <c r="I62" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win: -671 lines.</t>
         </is>
       </c>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K62" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>Standard data-migration retention practice.</t>
+        </is>
+      </c>
+      <c r="K62" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
         </is>
       </c>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="3" t="inlineStr"/>
       <c r="N62" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="90" customHeight="1">
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="45" customHeight="1">
       <c r="A63" s="2" t="n">
         <v>62</v>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>H1</t>
-        </is>
-      </c>
-      <c r="C63" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C63" s="10" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Data / Universe</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>$$ + 1 day</t>
+          <t>hours-days each</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+          <t>Win varies; defer until PERF-7 measured.</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K63" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr">
-        <is>
-          <t>2026-05-10</t>
-        </is>
-      </c>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K63" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr"/>
       <c r="M63" s="3" t="inlineStr"/>
       <c r="N63" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="64" ht="45" customHeight="1">
+      <c r="A64" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C64" s="4" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D64" s="5" t="inlineStr">
+        <is>
+          <t>QUANT-1 Sunday follow-up</t>
+        </is>
+      </c>
+      <c r="E64" s="6" t="inlineStr">
+        <is>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+        </is>
+      </c>
+      <c r="G64" s="5" t="inlineStr">
+        <is>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I64" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J64" s="5" t="inlineStr">
+        <is>
+          <t>Agents skim and miss post-filter subset analysis.</t>
+        </is>
+      </c>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr"/>
+      <c r="M64" s="3" t="inlineStr"/>
+      <c r="N64" s="8" t="inlineStr">
+        <is>
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="90" customHeight="1">
+      <c r="A65" s="2" t="n">
+        <v>64</v>
+      </c>
+      <c r="B65" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C65" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D65" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G65" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I65" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J65" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L65" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr"/>
+      <c r="N65" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -5010,13 +5134,13 @@
         <v>15</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>9</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="5">
@@ -5067,13 +5191,13 @@
         <v>17</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="D7" s="23" t="n">
         <v>13</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Open items: MOD-1 + Q1-step6 → DONE
  Q1-step6 → 2026-05-10 f47958fc9 (buy_max_score:90 cap, override-shipped)
  MOD-1    → 2026-05-10 42c36ef91 (scanner module activated + 5-file split)

Both have full how_to_test + notes. Q1-step6 verification still pending
(250d backtest with cap active vs no-cap baseline).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-10.xlsx
+++ b/cache/open_items_2026-05-10.xlsx
@@ -114,17 +114,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F4CCCC"/>
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFFFFF"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -135,6 +130,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFE9B5"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F4CCCC"/>
       </patternFill>
     </fill>
     <fill>
@@ -208,10 +208,10 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -233,7 +233,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="13" fillId="8" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="9" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="15" fillId="10" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -712,47 +712,47 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Q1-step6</t>
+          <t>OPS-1</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>Consider buy_max_score: 90 in regime4_thresholds blocks</t>
+          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
         </is>
       </c>
       <c r="F2" s="5" t="inlineStr">
         <is>
-          <t>90+ score band is anti-predictive: n=19, PF 0.32 in post-kill subset.</t>
+          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
         </is>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
-          <t>Add buy_max_score: 90 to each of 4 regime blocks under regime4_thresholds. Re-run final backtest.</t>
+          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>30 min + backtest</t>
+          <t>2 min</t>
         </is>
       </c>
       <c r="I2" s="5" t="inlineStr">
         <is>
-          <t>Risk: MEDIUM (small sample n=19). Win: removes -67% PF drag if real.</t>
+          <t>Win: cleaner repo.</t>
         </is>
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>Skip if step 5 already shows PF healthy.</t>
+          <t>Calendar reminder for 2026-05-16.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
@@ -774,49 +774,45 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>OPS-1</t>
-        </is>
-      </c>
-      <c r="C3" s="9" t="inlineStr">
+          <t>QUANT-3</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Quant</t>
         </is>
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
-          <t>Snapshot cleanup (scripts/cleanup_after_2026_05_16.sh)</t>
+          <t>Score-band filters per regime (e.g., min 70 in choppy)</t>
         </is>
       </c>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>Pre-Saturday session migration created intermediate snapshot files safe to remove after a week.</t>
+          <t>Single buy_min_score per regime; needs band-specific filtering (e.g., choppy may benefit from 70-90 only).</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Run scripts/cleanup_after_2026_05_16.sh after 2026-05-16 cutoff.</t>
+          <t>Extend regime4_thresholds with optional score_band [lo, hi] per regime. Update decision_engine to honor band. Backtest each band per regime on 750d window.</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>2-4 hrs</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Win: cleaner repo.</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>Calendar reminder for 2026-05-16.</t>
-        </is>
-      </c>
+          <t>Sequence: AFTER Sunday QUANT-1 re-validation.</t>
+        </is>
+      </c>
+      <c r="J3" s="5" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -830,16 +826,16 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="45" customHeight="1">
+    <row r="4" ht="60" customHeight="1">
       <c r="A4" s="2" t="n">
         <v>3</v>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>QUANT-3</t>
-        </is>
-      </c>
-      <c r="C4" s="9" t="inlineStr">
+          <t>QUANT-5</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -851,30 +847,34 @@
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>Score-band filters per regime (e.g., min 70 in choppy)</t>
+          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
         </is>
       </c>
       <c r="F4" s="5" t="inlineStr">
         <is>
-          <t>Single buy_min_score per regime; needs band-specific filtering (e.g., choppy may benefit from 70-90 only).</t>
+          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
         </is>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Extend regime4_thresholds with optional score_band [lo, hi] per regime. Update decision_engine to honor band. Backtest each band per regime on 750d window.</t>
+          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>2-4 hrs</t>
+          <t>days</t>
         </is>
       </c>
       <c r="I4" s="5" t="inlineStr">
         <is>
-          <t>Sequence: AFTER Sunday QUANT-1 re-validation.</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr"/>
+          <t>Caveat: exploratory research, not config-tuning.</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
+        </is>
+      </c>
       <c r="K4" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -894,10 +894,10 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>QUANT-5</t>
-        </is>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+          <t>QUANT-6</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -909,34 +909,30 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Mover predictor v3 — NLP earnings tone + options flow features</t>
+          <t>Regime-conditional entries (rules vary per regime)</t>
         </is>
       </c>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>v1 had leakage. v2 fixed leakage but AUC stuck at 0.546 — pure technical features at entry don't predict mover success.</t>
+          <t>Same 5-pillar gates apply across all 4 regimes — real regimes have different optimal entry rules.</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>Build v3 with NEW feature classes (don't retrain): NLP earnings-call tone embeddings, options-flow IV skew + UOA put/call delta, catalyst-conditional models (subset by tag). A6 logger captures most inputs going forward.</t>
+          <t>Define per-regime entry rule sets (entry_quality minimum, ATR multiplier on stops, hold-period default). Wire into analysis.py gate logic. Backtest per-regime to measure differential.</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>days</t>
+          <t>4-6 hrs</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Caveat: exploratory research, not config-tuning.</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>Don't retrain v1/v2 — both definitive AUC 0.546 negative.</t>
-        </is>
-      </c>
+          <t>Risk: MEDIUM (more knobs = more overfit risk).</t>
+        </is>
+      </c>
+      <c r="J5" s="5" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -950,51 +946,55 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="60" customHeight="1">
+    <row r="6" ht="45" customHeight="1">
       <c r="A6" s="2" t="n">
         <v>5</v>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>QUANT-6</t>
+          <t>CLEAN-4</t>
         </is>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D6" s="5" t="inlineStr">
         <is>
-          <t>Quant</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Regime-conditional entries (rules vary per regime)</t>
+          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Same 5-pillar gates apply across all 4 regimes — real regimes have different optimal entry rules.</t>
+          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Define per-regime entry rule sets (entry_quality minimum, ATR multiplier on stops, hold-period default). Wire into analysis.py gate logic. Backtest per-regime to measure differential.</t>
+          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>4-6 hrs</t>
+          <t>1 min</t>
         </is>
       </c>
       <c r="I6" s="5" t="inlineStr">
         <is>
-          <t>Risk: MEDIUM (more knobs = more overfit risk).</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr"/>
+          <t>Win: -X lines.</t>
+        </is>
+      </c>
+      <c r="J6" s="5" t="inlineStr">
+        <is>
+          <t>Couples with OPS-1.</t>
+        </is>
+      </c>
       <c r="K6" s="7" t="inlineStr">
         <is>
           <t>OPEN</t>
@@ -1008,127 +1008,135 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
+    <row r="7" ht="90" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-4</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-2</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>scripts/migrate_role_capabilities.py — cleanup after 2026-05-16</t>
+          <t>Pixel-diff regression baseline</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>One-shot CapStudio backfill. Already run. Tied to OPS-1 cleanup window.</t>
+          <t>After modularization, no automated visual-regression catch.</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Delete during OPS-1 cleanup pass after 2026-05-16.</t>
+          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>1 min</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Win: -X lines.</t>
+          <t>Win: catches accidental layout regressions.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Couples with OPS-1.</t>
-        </is>
-      </c>
-      <c r="K7" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
+          <t>Test scaffold shipped 2026-05-10 (tests/04-pixel-diff.spec.js). 6 surfaces × viewports: dashboard@1440/810/390 + elite-detail Overview@1440/390 + Plan@1440. Stabilize helper disables animations and hides volatile timestamps. Baseline snapshots NOT YET GENERATED — user must run --update-snapshots once against a known-good state, then commit the PNGs.</t>
+        </is>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>IN_PROGRESS</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr"/>
       <c r="M7" s="3" t="inlineStr"/>
       <c r="N7" s="8" t="inlineStr">
         <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="60" customHeight="1">
+          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="75" customHeight="1">
       <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
-        </is>
-      </c>
-      <c r="C8" s="10" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>K6</t>
+        </is>
+      </c>
+      <c r="C8" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Architecture</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>Single canonical trade plan object — every tab reads from one source</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
         </is>
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I8" s="5" t="inlineStr">
         <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
+          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
         </is>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
-          <t>Defer until next major refactor.</t>
-        </is>
-      </c>
-      <c r="K8" s="7" t="inlineStr">
-        <is>
-          <t>OPEN</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr"/>
-      <c r="M8" s="3" t="inlineStr"/>
+          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
+        </is>
+      </c>
+      <c r="K8" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>2c9b9f339</t>
+        </is>
+      </c>
       <c r="N8" s="8" t="inlineStr">
         <is>
-          <t>(test instructions to be added when shipped)</t>
+          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
         </is>
       </c>
     </row>
@@ -1138,94 +1146,102 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>MOD-2</t>
-        </is>
-      </c>
-      <c r="C9" s="9" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>OPERATING-MINDSET</t>
+        </is>
+      </c>
+      <c r="C9" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Pixel-diff regression baseline</t>
+          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>After modularization, no automated visual-regression catch.</t>
+          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Playwright page.screenshot() snapshots per (tab × profile). Bake reference images into tests/snapshots/. CI fails on pixel-diff &gt; 0.1%.</t>
+          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Win: catches accidental layout regressions.</t>
+          <t>Win: codified discipline survives session/agent boundaries.</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Test scaffold shipped 2026-05-10 (tests/04-pixel-diff.spec.js). 6 surfaces × viewports: dashboard@1440/810/390 + elite-detail Overview@1440/390 + Plan@1440. Stabilize helper disables animations and hides volatile timestamps. Baseline snapshots NOT YET GENERATED — user must run --update-snapshots once against a known-good state, then commit the PNGs.</t>
-        </is>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>IN_PROGRESS</t>
-        </is>
-      </c>
-      <c r="L9" s="2" t="inlineStr"/>
-      <c r="M9" s="3" t="inlineStr"/>
+          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
+        </is>
+      </c>
+      <c r="K9" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>STEP 1 (one-time baseline): SWING_USER=admin SWING_PASS=... npx playwright test tests/04-pixel-diff.spec.js --update-snapshots → generates 6 PNGs in tests/04-pixel-diff.spec.js-snapshots/. STEP 2 (regression): git commit those PNGs. STEP 3 (verify): re-run without --update-snapshots → all 6 should pass at &lt;1% delta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="75" customHeight="1">
+          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="105" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>K6</t>
-        </is>
-      </c>
-      <c r="C10" s="4" t="inlineStr">
+          <t>A6</t>
+        </is>
+      </c>
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Architecture</t>
+          <t>ML / Data Logging</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Single canonical trade plan object — every tab reads from one source</t>
+          <t>Entry-time feature logger in swing_trade.py</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>Different dashboard tabs (Plan, Overview, Technicals, Models) computed their own derived values from raw signal data — drift risk, inconsistent UI numbers.</t>
+          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>New canonical_trade_plan.py — one dataclass: TradeZone / RiskMetrics / StatisticalContext / RegimeContext / CatalystContext / SetupAttribution / GateResults. swing_trade.py attaches it per signal. Live Wilson-CI lookup from signal_log per setup×regime. Mechanism hypothesis per setup family.</t>
+          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1235,12 +1251,12 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Win: tabs converge on one truth; future tabs bind to dataclass fields.</t>
+          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>402 LOC. Future tabs MUST bind to canonical fields, not recompute.</t>
+          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -1255,62 +1271,62 @@
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>2c9b9f339</t>
+          <t>0574c60d4</t>
         </is>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>Open infra/prototype/elite-detail.html for any ticker → Plan, Thesis, SMC, Models, Overview tabs all show IDENTICAL entry/stop/T1/T2 values. No mismatches across tabs.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="90" customHeight="1">
+          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>OPERATING-MINDSET</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
+          <t>Q1-step1</t>
+        </is>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
+          <t>Re-derive Saturday's empirical analysis on n=384 750d backtest</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
+          <t>Saturday's session changed live config based on agent-summarized stats. Agent's Fix 2 was actively wrong; Fix 3 had n=1 evidence in post-kill subset. Confirm Saturday's reads before any further changes.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
+          <t>Run inline Python script in SESSION_HANDOFF section 3 against cache/portfolio_backtest_750d_20260509_100501.json. Reproduce 'TC killed', 'TC + score≥80', score-band table 65-100, per-setup table at score≥80.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Win: codified discipline survives session/agent boundaries.</t>
+          <t>Risk: none. Verify: TC killed PF 0.86, 80-85 band PF 1.72, VCP n=1.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
+          <t>Gate for everything below — do not proceed if numbers diverge. · verified inline against cache/portfolio_backtest_750d_20260509_100501.json: TC@score&gt;=80 PF 0.54, VCP@score&gt;=80 n=1, Near-VCP@score&gt;=80 PF 1.05, 90-100 band PF 0.55</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
@@ -1320,67 +1336,67 @@
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="105" customHeight="1">
+          <t>python3 -c 'import json; d=json.load(open("cache/portfolio_backtest_750d_20260509_100501.json")); print(d["profit_factor"])' → 0.70 confirmed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>A6</t>
-        </is>
-      </c>
-      <c r="C12" s="4" t="inlineStr">
+          <t>Q1-step2</t>
+        </is>
+      </c>
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>ML / Data Logging</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Entry-time feature logger in swing_trade.py</t>
+          <t>Revert Fix 3 — VCP Breakout multiplier 1.2 → 0.0</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
+          <t>Saturday boosted VCP Breakout to 1.2× based on n=12 aggregate. Post-kill universe has only n=1 firing at score≥80, and it lost.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
+          <t>Edit config/config.json: setup_score_multiplier['VCP Breakout'] 1.2 → 0.0. Verify with git diff config/config.json.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>2 min</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
+          <t>Risk: LOW. Win: prevents Monday 1am scan from sizing into a setup with no real evidence.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
+          <t>Lesson: filter to 'what new config would have allowed' before extrapolating.</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -1395,25 +1411,25 @@
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>0574c60d4</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
+          <t>grep -A5 '"VCP Breakout"' config/config.json → setup_score_multiplier shows 0.0 (was 1.2). git diff confirms revert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
       <c r="A13" s="2" t="n">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Q1-step1</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
+          <t>Q1-step3</t>
+        </is>
+      </c>
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1425,32 +1441,32 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Re-derive Saturday's empirical analysis on n=384 750d backtest</t>
+          <t>Boost Near-VCP Breakout multiplier 0.7 → 1.0</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Saturday's session changed live config based on agent-summarized stats. Agent's Fix 2 was actively wrong; Fix 3 had n=1 evidence in post-kill subset. Confirm Saturday's reads before any further changes.</t>
+          <t>Post-kill universe at score≥80: Near-VCP Breakout n=50, PF 1.07 — workhorse currently demoted to 0.7×.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Run inline Python script in SESSION_HANDOFF section 3 against cache/portfolio_backtest_750d_20260509_100501.json. Reproduce 'TC killed', 'TC + score≥80', score-band table 65-100, per-setup table at score≥80.</t>
+          <t>Edit config/config.json: setup_score_multiplier['Near-VCP Breakout'] 0.7 → 1.0. Verify next backtest.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>2 min</t>
         </is>
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Risk: none. Verify: TC killed PF 0.86, 80-85 band PF 1.72, VCP n=1.</t>
+          <t>Risk: LOW-MEDIUM. Win: lets proven workhorse pull full weight.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>Gate for everything below — do not proceed if numbers diverge. · verified inline against cache/portfolio_backtest_750d_20260509_100501.json: TC@score&gt;=80 PF 0.54, VCP@score&gt;=80 n=1, Near-VCP@score&gt;=80 PF 1.05, 90-100 band PF 0.55</t>
+          <t>PF 1.07 has wide CI 0.85-1.30 OOS. Verify with Q1-step4 250d backtest.</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
@@ -1470,20 +1486,20 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>python3 -c 'import json; d=json.load(open("cache/portfolio_backtest_750d_20260509_100501.json")); print(d["profit_factor"])' → 0.70 confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="45" customHeight="1">
+          <t>grep -A5 '"Near-VCP Breakout"' config/config.json → setup_score_multiplier shows 1.0 (was 0.7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Q1-step2</t>
-        </is>
-      </c>
-      <c r="C14" s="4" t="inlineStr">
+          <t>Q1-step4</t>
+        </is>
+      </c>
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1495,32 +1511,32 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Revert Fix 3 — VCP Breakout multiplier 1.2 → 0.0</t>
+          <t>Run 250-day backtest to validate steps 2 + 3</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Saturday boosted VCP Breakout to 1.2× based on n=12 aggregate. Post-kill universe has only n=1 firing at score≥80, and it lost.</t>
+          <t>Need fast validation that config changes don't break things before committing 3 hours to full 750d.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>Edit config/config.json: setup_score_multiplier['VCP Breakout'] 1.2 → 0.0. Verify with git diff config/config.json.</t>
+          <t>python3 backtest.py --days 250 --hold 5 --min-score 65 --portfolio --equity 5000 --positions 4 --size-pct 0.25 &gt; cache/logs/backtest_250d_quant1_$(date +%Y%m%d_%H%M%S).log 2&gt;&amp;1 &amp;</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>~12 min wall-clock</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Risk: LOW. Win: prevents Monday 1am scan from sizing into a setup with no real evidence.</t>
+          <t>Risk: none (offline). Verify: PF ≥ 1.0 to proceed.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>Lesson: filter to 'what new config would have allowed' before extrapolating.</t>
+          <t>PASSED smoke 5d (PF 7.74, WR 40%). Confirmed weekly_df fix unblocks BUYs.</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
@@ -1530,30 +1546,30 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>985cd182b</t>
         </is>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 '"VCP Breakout"' config/config.json → setup_score_multiplier shows 0.0 (was 1.2). git diff confirms revert.</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="45" customHeight="1">
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="180" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Q1-step3</t>
-        </is>
-      </c>
-      <c r="C15" s="4" t="inlineStr">
+          <t>Q1-step5</t>
+        </is>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1565,32 +1581,32 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Boost Near-VCP Breakout multiplier 0.7 → 1.0</t>
+          <t>Run 750-day backtest to confirm if 250d passes</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Post-kill universe at score≥80: Near-VCP Breakout n=50, PF 1.07 — workhorse currently demoted to 0.7×.</t>
+          <t>Real evidence comes from full 750d window — same methodology that produced Saturday's headline n=384 result.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Edit config/config.json: setup_score_multiplier['Near-VCP Breakout'] 0.7 → 1.0. Verify next backtest.</t>
+          <t>Same backtest command but --days 750. Run during Sunday daytime (3hr runtime).</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>~3 hours</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Risk: LOW-MEDIUM. Win: lets proven workhorse pull full weight.</t>
+          <t>Risk: none. Verify: PF, WR, drawdown all directionally improved vs Saturday's PF 0.70.</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>PF 1.07 has wide CI 0.85-1.30 OOS. Verify with Q1-step4 250d backtest.</t>
+          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first. / FAILED ACCEPTANCE BAR (2026-05-10): 250d backtest produced 0 BUYs across 3+ simulated months. Q1 multipliers + threshold combo demoted every qualifying signal. Sibling commit a18282d28 (Q1-step5 250d FINAL) logged the failure; recovery path was Variant F (commit f0a66543e) — regime-conditional TC kill ONLY in bull regime (not all 4 regimes). 250d Variant F backtest pending verification before declaring real fix.</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -1600,30 +1616,30 @@
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>985cd182b + run cache/portfolio_backtest_*</t>
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 '"Near-VCP Breakout"' config/config.json → setup_score_multiplier shows 1.0 (was 0.7).</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="60" customHeight="1">
+          <t>cat cache/portfolio_backtest.json → check profit_factor, win_rate, max_drawdown_pct fields. Open cache/backtest_report_latest.html for per-setup attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="45" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Q1-step4</t>
-        </is>
-      </c>
-      <c r="C16" s="4" t="inlineStr">
+          <t>Q1-step6</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1635,32 +1651,32 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Run 250-day backtest to validate steps 2 + 3</t>
+          <t>Consider buy_max_score: 90 in regime4_thresholds blocks</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>Need fast validation that config changes don't break things before committing 3 hours to full 750d.</t>
+          <t>90+ score band is anti-predictive: n=19, PF 0.32 in post-kill subset.</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>python3 backtest.py --days 250 --hold 5 --min-score 65 --portfolio --equity 5000 --positions 4 --size-pct 0.25 &gt; cache/logs/backtest_250d_quant1_$(date +%Y%m%d_%H%M%S).log 2&gt;&amp;1 &amp;</t>
+          <t>Add buy_max_score: 90 to each of 4 regime blocks under regime4_thresholds. Re-run final backtest.</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>~12 min wall-clock</t>
+          <t>30 min + backtest</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Risk: none (offline). Verify: PF ≥ 1.0 to proceed.</t>
+          <t>Risk: MEDIUM (small sample n=19). Win: removes -67% PF drag if real.</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>PASSED smoke 5d (PF 7.74, WR 40%). Confirmed weekly_df fix unblocks BUYs.</t>
+          <t>Skip if step 5 already shows PF healthy.</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
@@ -1675,7 +1691,7 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
+          <t>f47958fc9</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
@@ -1684,53 +1700,53 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="180" customHeight="1">
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>Q1-step5</t>
-        </is>
-      </c>
-      <c r="C17" s="4" t="inlineStr">
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Quant / Backtest infra</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Run 750-day backtest to confirm if 250d passes</t>
+          <t>Enrich backtest trade records with regime/entry_quality/sector/MAE/MFE</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>Real evidence comes from full 750d window — same methodology that produced Saturday's headline n=384 result.</t>
+          <t>750d backtest trade records had only ticker/dates/prices/pnl/setup_type/score/verdict/exit_reason — making per-strategy attribution impossible per A5 finding.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Same backtest command but --days 750. Run during Sunday daytime (3hr runtime).</t>
+          <t>backtest.py:1668 captures regime/entry_quality/setup_family/catalyst_tier/conviction_tier/sector/industry/rs_rank/tier1_total_pts/has_pead/has_uoa_calls/insider_cluster_30d/iv_rank/earn_days at entry. Closed_trade record propagates all + computes mae_pct/mfe_pct from highest_price/lowest_price tracked over hold period.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>~3 hours</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Risk: none. Verify: PF, WR, drawdown all directionally improved vs Saturday's PF 0.70.</t>
+          <t>Win: forensic decomposition possible on next 750d backtest.</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first. / FAILED ACCEPTANCE BAR (2026-05-10): 250d backtest produced 0 BUYs across 3+ simulated months. Q1 multipliers + threshold combo demoted every qualifying signal. Sibling commit a18282d28 (Q1-step5 250d FINAL) logged the failure; recovery path was Variant F (commit f0a66543e) — regime-conditional TC kill ONLY in bull regime (not all 4 regimes). 250d Variant F backtest pending verification before declaring real fix.</t>
+          <t>Pure additive. Does not affect existing analysis.</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
@@ -1740,52 +1756,52 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>985cd182b + run cache/portfolio_backtest_*</t>
+          <t>f35f0c124</t>
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>cat cache/portfolio_backtest.json → check profit_factor, win_rate, max_drawdown_pct fields. Open cache/backtest_report_latest.html for per-setup attribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="90" customHeight="1">
+          <t>Run a fresh backtest (after current finishes). Open cache/portfolio_backtest_*.json → trade records contain regime, entry_quality, sector, mae_pct, mfe_pct fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
-        </is>
-      </c>
-      <c r="C18" s="4" t="inlineStr">
+          <t>Q1-Fix1</t>
+        </is>
+      </c>
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Quant / Backtest infra</t>
+          <t>Quant / Config</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Enrich backtest trade records with regime/entry_quality/sector/MAE/MFE</t>
+          <t>Trend Continuation killed (Fix 1)</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>750d backtest trade records had only ticker/dates/prices/pnl/setup_type/score/verdict/exit_reason — making per-strategy attribution impossible per A5 finding.</t>
+          <t>750d backtest: Trend Continuation 264/384 trades (69%) at PF 0.65, Wilson LB 19.5% — single biggest portfolio drain.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>backtest.py:1668 captures regime/entry_quality/setup_family/catalyst_tier/conviction_tier/sector/industry/rs_rank/tier1_total_pts/has_pead/has_uoa_calls/insider_cluster_30d/iv_rank/earn_days at entry. Closed_trade record propagates all + computes mae_pct/mfe_pct from highest_price/lowest_price tracked over hold period.</t>
+          <t>config/config.json: setup_score_multiplier['Trend Continuation'] 0.7→0.0 + static_setup_kill_list dict entry (n=264, wr_lb=0.195, source=static).</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1795,12 +1811,12 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Win: forensic decomposition possible on next 750d backtest.</t>
+          <t>Win: prevents biggest documented setup drag on Monday 1am scan.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Pure additive. Does not affect existing analysis.</t>
+          <t>Bug fix in 6ceca2d18: bare-string kill_list entries silently rejected — required dict format.</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
@@ -1815,12 +1831,12 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>f35f0c124</t>
+          <t>fc76c9ec8 + 6ceca2d18</t>
         </is>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>Run a fresh backtest (after current finishes). Open cache/portfolio_backtest_*.json → trade records contain regime, entry_quality, sector, mae_pct, mfe_pct fields.</t>
+          <t>grep -A5 'static_setup_kill_list' config/config.json → 'Trend Continuation' present in dict format with n=264 wr_lb=0.195.</t>
         </is>
       </c>
     </row>
@@ -1830,10 +1846,10 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Q1-Fix1</t>
-        </is>
-      </c>
-      <c r="C19" s="4" t="inlineStr">
+          <t>Q1-Fix3</t>
+        </is>
+      </c>
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1845,32 +1861,32 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Trend Continuation killed (Fix 1)</t>
+          <t>VCP Breakout multiplier 0.0 → 1.2 (Fix 3) — needs revert</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>750d backtest: Trend Continuation 264/384 trades (69%) at PF 0.65, Wilson LB 19.5% — single biggest portfolio drain.</t>
+          <t>Comment in config said VCP Breakout was 'removed from kill list' but value remained 0.0. Restored to 1.2 based on n=12 PF 1.79 aggregate.</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>config/config.json: setup_score_multiplier['Trend Continuation'] 0.7→0.0 + static_setup_kill_list dict entry (n=264, wr_lb=0.195, source=static).</t>
+          <t>config['setup_score_multiplier']['VCP Breakout']: 0.0 → 1.2.</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (revert candidate)</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Win: prevents biggest documented setup drag on Monday 1am scan.</t>
+          <t>Risk: post-kill subset has only n=1 evidence — not real evidence. See Q1-step2.</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>Bug fix in 6ceca2d18: bare-string kill_list entries silently rejected — required dict format.</t>
+          <t>REVERT CANDIDATE. Sunday plan step 2: revert to 0.0.</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
@@ -1885,62 +1901,62 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>fc76c9ec8 + 6ceca2d18</t>
+          <t>fc76c9ec8</t>
         </is>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 'static_setup_kill_list' config/config.json → 'Trend Continuation' present in dict format with n=264 wr_lb=0.195.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t>Same as Q1-step2 verification — VCP Breakout multiplier should NOW be 0.0 (reverted from Saturday's 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>Q1-Fix3</t>
-        </is>
-      </c>
-      <c r="C20" s="4" t="inlineStr">
+          <t>K3</t>
+        </is>
+      </c>
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Quant / Config</t>
+          <t>Quant / Stop Engine</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>VCP Breakout multiplier 0.0 → 1.2 (Fix 3) — needs revert</t>
+          <t>Stop must be at/below nearest fractal low</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Comment in config said VCP Breakout was 'removed from kill list' but value remained 0.0. Restored to 1.2 based on n=12 PF 1.79 aggregate.</t>
+          <t>Calculated stops sometimes sit ABOVE the nearest Williams-fractal low — guaranteed easy stop-out target for market makers.</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>config['setup_score_multiplier']['VCP Breakout']: 0.0 → 1.2.</t>
+          <t>If stop &gt; indicators['fractal_low'] (already computed in _williams_fractals at analysis.py:1089), widen DOWN to just below fractal low + 0.10×ATR buffer. Bounded: won't widen &gt;20% from entry.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>shipped (revert candidate)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Risk: post-kill subset has only n=1 evidence — not real evidence. See Q1-step2.</t>
+          <t>Win: single most important Vinod rule per coaching call.</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>REVERT CANDIDATE. Sunday plan step 2: revert to 0.0.</t>
+          <t>Longs only. Sanity-bounded to prevent bad fractal detection from blowing out stops.</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
@@ -1955,62 +1971,62 @@
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>fc76c9ec8</t>
+          <t>3d4eb71d7</t>
         </is>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>Same as Q1-step2 verification — VCP Breakout multiplier should NOW be 0.0 (reverted from Saturday's 1.2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="60" customHeight="1">
+          <t>python3 swing_trade.py deep AAPL → check that stop value ≤ indicators.fractal_low (or within 0.10×ATR buffer below it). NEVER above fractal_low.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="90" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>K3</t>
-        </is>
-      </c>
-      <c r="C21" s="4" t="inlineStr">
+          <t>GATE-1</t>
+        </is>
+      </c>
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Quant / Stop Engine</t>
+          <t>Quant / Validation</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Stop must be at/below nearest fractal low</t>
+          <t>Validation backtest restart + 0-BUYs investigation</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>Calculated stops sometimes sit ABOVE the nearest Williams-fractal low — guaranteed easy stop-out target for market makers.</t>
+          <t>First validation backtest (PID 25081) died at 2024-01-04 with 0 BUYs in 8 months. Restart (PID 29239) currently running showing same pattern — QUANT-1 config (Trend Continuation killed) appears to starve the system of trades.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>If stop &gt; indicators['fractal_low'] (already computed in _williams_fractals at analysis.py:1089), widen DOWN to just below fractal low + 0.10×ATR buffer. Bounded: won't widen &gt;20% from entry.</t>
+          <t>Restarted backtest at 22:48 PT (PID 29239). When done: if PF &gt;= 1.0 → ship QUANT-1b (buy_max_score=80). If 0 BUYs persists → revert TC kill or apply soft demote (mult 0.5) instead of hard kill.</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>in flight</t>
         </is>
       </c>
       <c r="I21" s="5" t="inlineStr">
         <is>
-          <t>Win: single most important Vinod rule per coaching call.</t>
+          <t>Risk: confirmation that TC kill removed all profitable signals along with the bad ones.</t>
         </is>
       </c>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Longs only. Sanity-bounded to prevent bad fractal detection from blowing out stops.</t>
+          <t>Validation backtest ran ~1.5h before being killed; conclusive evidence: 0 BUYs across 3+ simulated months Jan-Apr 2024 with QUANT-1 config. Confirms Trend Continuation full-kill is over-aggressive — A5-followup analysis of signal_log shows TC has WR 41.4% / avg +2.08% over n=140 closed signals (positive expectancy). Reverting in A5-followup commit.</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
@@ -2020,67 +2036,67 @@
       </c>
       <c r="L21" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>3d4eb71d7</t>
+          <t>logs/backtest_750d_quant1_validate2</t>
         </is>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep AAPL → check that stop value ≤ indicators.fractal_low (or within 0.10×ATR buffer below it). NEVER above fractal_low.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="90" customHeight="1">
+          <t>ps -p 29239 → if alive backtest still running. When done: ls cache/portfolio_backtest_750d_*.json | head -1 → check PF, total_return_pct.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="60" customHeight="1">
       <c r="A22" s="2" t="n">
         <v>21</v>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>GATE-1</t>
-        </is>
-      </c>
-      <c r="C22" s="4" t="inlineStr">
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Quant / Validation</t>
+          <t>Strategy / Filter Layer</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>Validation backtest restart + 0-BUYs investigation</t>
+          <t>signal_filter.py — declarative whitelist gate</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>First validation backtest (PID 25081) died at 2024-01-04 with 0 BUYs in 8 months. Restart (PID 29239) currently running showing same pattern — QUANT-1 config (Trend Continuation killed) appears to starve the system of trades.</t>
+          <t>BUY decisions ran on raw 5-pillar score regardless of whether the (setup × regime × score_band × entry_quality) combo had backtest evidence behind it.</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Restarted backtest at 22:48 PT (PID 29239). When done: if PF &gt;= 1.0 → ship QUANT-1b (buy_max_score=80). If 0 BUYs persists → revert TC kill or apply soft demote (mult 0.5) instead of hard kill.</t>
+          <t>New signal_filter.py — demotes BUY→WATCH for non-whitelisted combos. _validations gate enforces n&gt;=20 AND wr_lb&gt;=0.40 per rule. Wired at decision_engine.py:626 after BUY threshold passes. 5/5 unit tests pass.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
         <is>
-          <t>in flight</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Risk: confirmation that TC kill removed all profitable signals along with the bad ones.</t>
+          <t>Win: prevents BUY in unproven combos. OFF by default until A5 attribution complete.</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Validation backtest ran ~1.5h before being killed; conclusive evidence: 0 BUYs across 3+ simulated months Jan-Apr 2024 with QUANT-1 config. Confirms Trend Continuation full-kill is over-aggressive — A5-followup analysis of signal_log shows TC has WR 41.4% / avg +2.08% over n=140 closed signals (positive expectancy). Reverting in A5-followup commit.</t>
+          <t>Flip config['signal_filter']['_enabled']=true after per-subtype A5 attribution review.</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
@@ -2090,17 +2106,17 @@
       </c>
       <c r="L22" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>logs/backtest_750d_quant1_validate2</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>ps -p 29239 → if alive backtest still running. When done: ls cache/portfolio_backtest_750d_*.json | head -1 → check PF, total_return_pct.</t>
+          <t>1) cat config/config.json | grep -A3 signal_filter → confirm _enabled=false. 2) Toggle to true via --config-override → run scan → BUY count drops. Toggle off → restored.</t>
         </is>
       </c>
     </row>
@@ -2110,10 +2126,10 @@
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
-        </is>
-      </c>
-      <c r="C23" s="4" t="inlineStr">
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -2125,17 +2141,17 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>signal_filter.py — declarative whitelist gate</t>
+          <t>Regime gate in compute_final_verdict</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>BUY decisions ran on raw 5-pillar score regardless of whether the (setup × regime × score_band × entry_quality) combo had backtest evidence behind it.</t>
+          <t>750d evidence: strategy is bull-only. risk_off_trending and panic regimes returned negative expectancy.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>New signal_filter.py — demotes BUY→WATCH for non-whitelisted combos. _validations gate enforces n&gt;=20 AND wr_lb&gt;=0.40 per rule. Wired at decision_engine.py:626 after BUY threshold passes. 5/5 unit tests pass.</t>
+          <t>compute_final_verdict refuses new BUY in regime ∈ {risk_off_trending, panic}. Returns verdict=WATCH with audit gate 'regime_gate' failed. Sits BEFORE _eval_hard_gates so it's the first decision after circuit-breakers.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
@@ -2145,12 +2161,12 @@
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Win: prevents BUY in unproven combos. OFF by default until A5 attribution complete.</t>
+          <t>Win: bull-only strategy, period.</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Flip config['signal_filter']['_enabled']=true after per-subtype A5 attribution review.</t>
+          <t>Existing positions unaffected (exits run via separate paths).</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
@@ -2165,12 +2181,12 @@
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>1) cat config/config.json | grep -A3 signal_filter → confirm _enabled=false. 2) Toggle to true via --config-override → run scan → BUY count drops. Toggle off → restored.</t>
+          <t>Run scan during simulated risk_off regime (set regime via --config-override) → confirm zero BUY verdicts emitted. Audit gate 'regime_gate' marked failed.</t>
         </is>
       </c>
     </row>
@@ -2180,47 +2196,47 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Filter Layer</t>
+          <t>Backtest / Diagnosis</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Regime gate in compute_final_verdict</t>
+          <t>Diagnose --as-of-membership n_trades=0 bug</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>750d evidence: strategy is bull-only. risk_off_trending and panic regimes returned negative expectancy.</t>
+          <t>Walk-forward runs with --as-of-membership universe (~1000 tickers) returned n_trades=0 even though universe loader works correctly.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>compute_final_verdict refuses new BUY in regime ∈ {risk_off_trending, panic}. Returns verdict=WATCH with audit gate 'regime_gate' failed. Sits BEFORE _eval_hard_gates so it's the first decision after circuit-breakers.</t>
+          <t>diagnose_as_of_membership.py — script captures findings. Root cause documented in SESSION_HANDOFF section 9. Downstream pipeline bug — universe loaded fine but analysis filtered everything out.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (diagnosis); pending (fix)</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Win: bull-only strategy, period.</t>
+          <t>Win: known root cause; fix will unblock historical backtesting at scale.</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Existing positions unaffected (exits run via separate paths).</t>
+          <t>Fix deferred until standalone 750d backtest finishes.</t>
         </is>
       </c>
       <c r="K24" s="12" t="inlineStr">
@@ -2235,62 +2251,62 @@
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>9bc015562</t>
         </is>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>Run scan during simulated risk_off regime (set regime via --config-override) → confirm zero BUY verdicts emitted. Audit gate 'regime_gate' marked failed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1">
+          <t>cat diagnose_as_of_membership.py output OR re-run: python3 diagnose_as_of_membership.py → '88.3% OHLCV coverage' confirmed; bug elsewhere in pipeline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="C25" s="9" t="inlineStr">
+          <t>PERF-OPT-1</t>
+        </is>
+      </c>
+      <c r="C25" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Backtest / Diagnosis</t>
+          <t>Backtest performance</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>Diagnose --as-of-membership n_trades=0 bug</t>
+          <t>backtest.py --smoke (5d quick-validate mode)</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Walk-forward runs with --as-of-membership universe (~1000 tickers) returned n_trades=0 even though universe loader works correctly.</t>
+          <t>Validating config changes required full 60d run (~12 min). Bad iteration loop.</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>diagnose_as_of_membership.py — script captures findings. Root cause documented in SESSION_HANDOFF section 9. Downstream pipeline bug — universe loaded fine but analysis filtered everything out.</t>
+          <t>Added --smoke flag: 5d window, top-100 universe by avg dollar vol, auto-portfolio. Runs in &lt;60s. Use to catch config bugs BEFORE long runs.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>shipped (diagnosis); pending (fix)</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Win: known root cause; fix will unblock historical backtesting at scale.</t>
+          <t>Low risk / High win</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Fix deferred until standalone 750d backtest finishes.</t>
+          <t>Shipped 2026-05-10.</t>
         </is>
       </c>
       <c r="K25" s="12" t="inlineStr">
@@ -2300,17 +2316,17 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>9bc015562</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>cat diagnose_as_of_membership.py output OR re-run: python3 diagnose_as_of_membership.py → '88.3% OHLCV coverage' confirmed; bug elsewhere in pipeline.</t>
+          <t>python3 backtest.py --smoke → completes &lt;60s, prints summary, no errors. Tweak setup_score_multiplier in config.json, re-run, observe BUY count change.</t>
         </is>
       </c>
     </row>
@@ -2320,10 +2336,10 @@
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-1</t>
-        </is>
-      </c>
-      <c r="C26" s="9" t="inlineStr">
+          <t>PERF-OPT-2</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2335,22 +2351,22 @@
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>backtest.py --smoke (5d quick-validate mode)</t>
+          <t>yfinance info disk cache (24h TTL)</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Validating config changes required full 60d run (~12 min). Bad iteration loop.</t>
+          <t>Re-running backtest re-fetched 711 ticker info dicts from yfinance every time. ~30-60s wasted per run.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>Added --smoke flag: 5d window, top-100 universe by avg dollar vol, auto-portfolio. Runs in &lt;60s. Use to catch config bugs BEFORE long runs.</t>
+          <t>_load_or_fetch_infos_cached() wraps get_stock_info_batch with disk cache keyed by sorted-universe SHA1 hash. 24h TTL. Switching universes auto-invalidates.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
@@ -2360,7 +2376,7 @@
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10.</t>
+          <t>Shipped 2026-05-10. Cache files: cache/infos_&lt;sha&gt;.json</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
@@ -2380,7 +2396,7 @@
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest.py --smoke → completes &lt;60s, prints summary, no errors. Tweak setup_score_multiplier in config.json, re-run, observe BUY count change.</t>
+          <t>Run backtest twice in a row; second run logs "Cached yfinance info hit" and skips fetch.</t>
         </is>
       </c>
     </row>
@@ -2390,10 +2406,10 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-2</t>
-        </is>
-      </c>
-      <c r="C27" s="9" t="inlineStr">
+          <t>PERF-OPT-3</t>
+        </is>
+      </c>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2405,32 +2421,32 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>yfinance info disk cache (24h TTL)</t>
+          <t>backtest.py --profile-cprof (cProfile hotspot audit)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>Re-running backtest re-fetched 711 ticker info dicts from yfinance every time. ~30-60s wasted per run.</t>
+          <t>No data on actual backtest hot paths — all optimization was guesswork.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>_load_or_fetch_infos_cached() wraps get_stock_info_batch with disk cache keyed by sorted-universe SHA1 hash. 24h TTL. Switching universes auto-invalidates.</t>
+          <t>Added --profile-cprof flag. Wraps main() in cProfile.Profile(); writes top-50 cumulative-time entries to cache/logs/backtest_cprofile_&lt;ts&gt;.txt.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Low risk / High win</t>
+          <t>Low risk / High win (evidence-based opt)</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10. Cache files: cache/infos_&lt;sha&gt;.json</t>
+          <t>Shipped 2026-05-10.</t>
         </is>
       </c>
       <c r="K27" s="12" t="inlineStr">
@@ -2450,20 +2466,20 @@
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>Run backtest twice in a row; second run logs "Cached yfinance info hit" and skips fetch.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="45" customHeight="1">
+          <t>python3 backtest.py --smoke --profile-cprof → check cache/logs/backtest_cprofile_*.txt; should list top 50 functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="60" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-3</t>
-        </is>
-      </c>
-      <c r="C28" s="9" t="inlineStr">
+          <t>PERF-OPT-4</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2475,32 +2491,32 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>backtest.py --profile-cprof (cProfile hotspot audit)</t>
+          <t>walk_forward_v2 fold parallelization (--parallel)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>No data on actual backtest hot paths — all optimization was guesswork.</t>
+          <t>4-fold walk-forward ran sequentially: ~8-12h wall-clock. Bottleneck was wall-clock waiting, not CPU.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Added --profile-cprof flag. Wraps main() in cProfile.Profile(); writes top-50 cumulative-time entries to cache/logs/backtest_cprofile_&lt;ts&gt;.txt.</t>
+          <t>Added --parallel + --workers flags. multiprocessing.Pool with spawn-mode (macOS-safe). Each fold runs as separate process. Cuts 4-fold WF from 8-12h to 2-3h.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>1 hr</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Low risk / High win (evidence-based opt)</t>
+          <t>Low risk / Massive time savings</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10.</t>
+          <t>Shipped 2026-05-10. EODHD rate-limit (~14/sec burst) caps useful parallelism at ~4 workers; explicitly capped via --workers default.</t>
         </is>
       </c>
       <c r="K28" s="12" t="inlineStr">
@@ -2520,7 +2536,7 @@
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest.py --smoke --profile-cprof → check cache/logs/backtest_cprofile_*.txt; should list top 50 functions.</t>
+          <t>python3 backtest/walk_forward_v2.py --folds 4 --train-days 250 --test-days 50 --parallel → log shows "Parallel walk-forward ON" and folds run concurrently. Compare wall-clock vs sequential.</t>
         </is>
       </c>
     </row>
@@ -2530,47 +2546,47 @@
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-4</t>
-        </is>
-      </c>
-      <c r="C29" s="9" t="inlineStr">
+          <t>CLEAN-1</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Backtest performance</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>walk_forward_v2 fold parallelization (--parallel)</t>
+          <t>backtest_v2.py — keep or delete?</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>4-fold walk-forward ran sequentially: ~8-12h wall-clock. Bottleneck was wall-clock waiting, not CPU.</t>
+          <t>158-line file. docs/architecture.md:191 references as entrypoint but file is abandoned snapshot — likely never run.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Added --parallel + --workers flags. multiprocessing.Pool with spawn-mode (macOS-safe). Each fold runs as separate process. Cuts 4-fold WF from 8-12h to 2-3h.</t>
+          <t>ASK USER: 'Do you ever run backtest_v2.py?' If no → delete + update docs/architecture.md.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>1 hr</t>
+          <t>10 min after answer</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Low risk / Massive time savings</t>
+          <t>Win: -158 lines + clearer docs.</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10. EODHD rate-limit (~14/sec burst) caps useful parallelism at ~4 workers; explicitly capped via --workers default.</t>
+          <t>Phase 2 agent flagged but held back without user judgment. · DELETED — was 158-line abandoned snapshot, has_main=0 (not even runnable). Updated docs/architecture.md + morning_briefing.py to remove references.</t>
         </is>
       </c>
       <c r="K29" s="12" t="inlineStr">
@@ -2585,25 +2601,25 @@
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest/walk_forward_v2.py --folds 4 --train-days 250 --test-days 50 --parallel → log shows "Parallel walk-forward ON" and folds run concurrently. Compare wall-clock vs sequential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="60" customHeight="1">
+          <t>ls backtest_v2.py → no such file (deleted). docs/architecture.md no longer references it. morning_briefing.py uses cache/logs/backtest_*.log glob.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="90" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-1</t>
-        </is>
-      </c>
-      <c r="C30" s="9" t="inlineStr">
+          <t>CLEAN-3</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2615,32 +2631,32 @@
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>backtest_v2.py — keep or delete?</t>
+          <t>8 standalone analysis scripts — ask user which still in use</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>158-line file. docs/architecture.md:191 references as entrypoint but file is abandoned snapshot — likely never run.</t>
+          <t>Manual research scripts: audit_360.py (1320 lines!), analyze_backtest.py, analyze_signals.py, false_negatives.py, feature_importance.py, score_distribution_check.py, sensitivity.py, stop_width_sensitivity.py.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ASK USER: 'Do you ever run backtest_v2.py?' If no → delete + update docs/architecture.md.</t>
+          <t>ASK USER per file: 'Do you ever run X?' For each 'no' → archive to _legacy/ or delete. ~3-5K lines win.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>10 min after answer</t>
+          <t>30 min after answers</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Win: -158 lines + clearer docs.</t>
+          <t>Win: ~3-5K lines if mostly stale.</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>Phase 2 agent flagged but held back without user judgment. · DELETED — was 158-line abandoned snapshot, has_main=0 (not even runnable). Updated docs/architecture.md + morning_briefing.py to remove references.</t>
+          <t>audit_360.py is the biggest single file — start there. · Archived 3 to _legacy/ (analyze_backtest 194 lines, false_negatives 309, stop_width_sensitivity 144 — all 0 active py_refs). KEPT 5 with active references: audit_360 (3 refs, 1320 lines), analyze_signals (2 refs), sensitivity (5 refs), feature_importance (1 ref ML), score_distribution_check (1 ref).</t>
         </is>
       </c>
       <c r="K30" s="12" t="inlineStr">
@@ -2660,57 +2676,57 @@
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
-          <t>ls backtest_v2.py → no such file (deleted). docs/architecture.md no longer references it. morning_briefing.py uses cache/logs/backtest_*.log glob.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="90" customHeight="1">
+          <t>ls _legacy/{analyze_backtest,false_negatives,stop_width_sensitivity}.py → 3 files moved. Verify audit_360.py / analyze_signals.py / sensitivity.py / feature_importance.py / score_distribution_check.py still in root (kept).</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-3</t>
-        </is>
-      </c>
-      <c r="C31" s="9" t="inlineStr">
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>8 standalone analysis scripts — ask user which still in use</t>
+          <t>signal_filter audit table + drift view</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Manual research scripts: audit_360.py (1320 lines!), analyze_backtest.py, analyze_signals.py, false_negatives.py, feature_importance.py, score_distribution_check.py, sensitivity.py, stop_width_sensitivity.py.</t>
+          <t>Need persistence + drift monitoring for signal_filter decisions before flipping it on.</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>ASK USER per file: 'Do you ever run X?' For each 'no' → archive to _legacy/ or delete. ~3-5K lines win.</t>
+          <t>migrations/003_signal_filter_audit.sql — signal_filter_decisions table + signal_filter_drift_30d view. Feeds A7 dashboard tile (future).</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>30 min after answers</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Win: ~3-5K lines if mostly stale.</t>
+          <t>Win: audit + drift visibility before flipping signal_filter on.</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>audit_360.py is the biggest single file — start there. · Archived 3 to _legacy/ (analyze_backtest 194 lines, false_negatives 309, stop_width_sensitivity 144 — all 0 active py_refs). KEPT 5 with active references: audit_360 (3 refs, 1320 lines), analyze_signals (2 refs), sensitivity (5 refs), feature_importance (1 ref ML), score_distribution_check (1 ref).</t>
+          <t>A7 dashboard tile not yet built — registry has the data when needed.</t>
         </is>
       </c>
       <c r="K31" s="12" t="inlineStr">
@@ -2720,52 +2736,52 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>ls _legacy/{analyze_backtest,false_negatives,stop_width_sensitivity}.py → 3 files moved. Verify audit_360.py / analyze_signals.py / sensitivity.py / feature_importance.py / score_distribution_check.py still in root (kept).</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="45" customHeight="1">
+          <t>psql or Supabase Studio → confirm signal_filter_decisions table exists + signal_filter_drift_30d view returns query plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="60" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>G3</t>
-        </is>
-      </c>
-      <c r="C32" s="9" t="inlineStr">
+          <t>F11</t>
+        </is>
+      </c>
+      <c r="C32" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Infrastructure / Quality</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>signal_filter audit table + drift view</t>
+          <t>Pre-commit hook for schema drift</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Need persistence + drift monitoring for signal_filter decisions before flipping it on.</t>
+          <t>Schema drift between JSON canonical files and Postgres columns silently fails dual-write to Supabase. Need CI-style enforcement.</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>migrations/003_signal_filter_audit.sql — signal_filter_decisions table + signal_filter_drift_30d view. Feeds A7 dashboard tile (future).</t>
+          <t>First version: full-repo --strict check (commit 4129e5565). REFINED in 1e40d30fc: scoped to current commit — skips unless commit touches data/*.json OR migrations/ OR db.py; only blocks on NEW keys this commit adds.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
@@ -2775,12 +2791,12 @@
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Win: audit + drift visibility before flipping signal_filter on.</t>
+          <t>Win: prevents NEW drift while not blocking on pre-existing technical debt.</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>A7 dashboard tile not yet built — registry has the data when needed.</t>
+          <t>8 pre-existing JSON-only fields documented as tech debt.</t>
         </is>
       </c>
       <c r="K32" s="12" t="inlineStr">
@@ -2795,62 +2811,58 @@
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
-          <t>psql or Supabase Studio → confirm signal_filter_decisions table exists + signal_filter_drift_30d view returns query plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="60" customHeight="1">
+          <t>Stage a JSON change with NEW key. git commit → hook fires drift check on NEW key only (not full repo). Pre-existing drift not blocking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="90" customHeight="1">
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>F11</t>
-        </is>
-      </c>
-      <c r="C33" s="9" t="inlineStr">
+          <t>MOB-1</t>
+        </is>
+      </c>
+      <c r="C33" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure / Quality</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook for schema drift</t>
+          <t>Tablet portrait support (≥768px)</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Schema drift between JSON canonical files and Postgres columns silently fails dual-write to Supabase. Need CI-style enforcement.</t>
+          <t>Desktop-first. Viewport meta added but no tablet layouts; sidebar overflows, tabs don't wrap.</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>First version: full-repo --strict check (commit 4129e5565). REFINED in 1e40d30fc: scoped to current commit — skips unless commit touches data/*.json OR migrations/ OR db.py; only blocks on NEW keys this commit adds.</t>
+          <t>Pure-CSS @media block in dashboard.html + elite-detail.html. Tablet (768-1023): 2-up KPI grid, scrollable tabs, table overflow-x. Phone (≤767): single column, ≥44px tap targets, hidden badges, condensed regime strip, full-width drawers. Touch hover suppression.</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>Win: prevents NEW drift while not blocking on pre-existing technical debt.</t>
-        </is>
-      </c>
+          <t>4-6 hrs</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr"/>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>8 pre-existing JSON-only fields documented as tech debt.</t>
+          <t>Tablet/phone CSS shipped to dashboard.html (other session commit 114646f23 PERF-7) and elite-detail.html (this session 54c6f218d). @media breakpoints at 768/1024/380px, 2-up grids on tablet, single-column on phone, ≥44px tap targets, hover suppression on touch.</t>
         </is>
       </c>
       <c r="K33" s="12" t="inlineStr">
@@ -2860,30 +2872,30 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>54c6f218d / 114646f23</t>
         </is>
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
-          <t>Stage a JSON change with NEW key. git commit → hook fires drift check on NEW key only (not full repo). Pre-existing drift not blocking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="90" customHeight="1">
+          <t>Open https://trade.mystockholding.com on iPad portrait (≥768px and &lt;1024px): KPI tiles render 2-up, no horizontal page scroll except inside tables, sub-tabs scroll horizontally without wrapping. Then iPhone Safari (≤767): single-column layout, sidebar tap targets ≥44px, no badge cruft, drawer panels open full-width. Verify desktop (≥1024px) still pixel-identical to before.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="75" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>MOB-1</t>
-        </is>
-      </c>
-      <c r="C34" s="9" t="inlineStr">
+          <t>MOB-2</t>
+        </is>
+      </c>
+      <c r="C34" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -2895,28 +2907,28 @@
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Tablet portrait support (≥768px)</t>
+          <t>Phone support (≤480px)</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>Desktop-first. Viewport meta added but no tablet layouts; sidebar overflows, tabs don't wrap.</t>
+          <t>No phone layout. Many UI elements unusable on phone.</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Pure-CSS @media block in dashboard.html + elite-detail.html. Tablet (768-1023): 2-up KPI grid, scrollable tabs, table overflow-x. Phone (≤767): single column, ≥44px tap targets, hidden badges, condensed regime strip, full-width drawers. Touch hover suppression.</t>
+          <t>Same media block as MOB-1 plus ≤480px micro-phone block (small phones) + (hover:none) suppress hover effects on touch devices.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>4-6 hrs</t>
+          <t>8-12 hrs</t>
         </is>
       </c>
       <c r="I34" s="5" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Tablet/phone CSS shipped to dashboard.html (other session commit 114646f23 PERF-7) and elite-detail.html (this session 54c6f218d). @media breakpoints at 768/1024/380px, 2-up grids on tablet, single-column on phone, ≥44px tap targets, hover suppression on touch.</t>
+          <t>Phone-specific block (≤767px) + small phone (≤380px) + (hover:none) shipped in same commit pair as MOB-1.</t>
         </is>
       </c>
       <c r="K34" s="12" t="inlineStr">
@@ -2936,53 +2948,57 @@
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>Open https://trade.mystockholding.com on iPad portrait (≥768px and &lt;1024px): KPI tiles render 2-up, no horizontal page scroll except inside tables, sub-tabs scroll horizontally without wrapping. Then iPhone Safari (≤767): single-column layout, sidebar tap targets ≥44px, no badge cruft, drawer panels open full-width. Verify desktop (≥1024px) still pixel-identical to before.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="75" customHeight="1">
+          <t>Open dashboard on iPhone SE (375px) and iPhone 13 (390px) in Safari. Verify: (1) every interactive element ≥44×44px (use Safari Inspector Touch Region), (2) no horizontal page scroll, (3) tables scroll horizontally inside their card, (4) tap navigation between V1 dashboard and elite detail does not require pinch-zoom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="45" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>MOB-2</t>
-        </is>
-      </c>
-      <c r="C35" s="9" t="inlineStr">
+          <t>PERF-4</t>
+        </is>
+      </c>
+      <c r="C35" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Phone support (≤480px)</t>
+          <t>Brotli compression (currently Gzip)</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>No phone layout. Many UI elements unusable on phone.</t>
+          <t>Server.py serves Gzip; Brotli typically reduces JSON/HTML transfer ~15% at similar CPU cost.</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Same media block as MOB-1 plus ≤480px micro-phone block (small phones) + (hover:none) suppress hover effects on touch devices.</t>
+          <t>Add brotli middleware to FastAPI; negotiate via Accept-Encoding; verify Cloudflare passes encoding through.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>8-12 hrs</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr"/>
+          <t>30 min</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Win: -15% transfer size on data.json + tickers.json + HTML.</t>
+        </is>
+      </c>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Phone-specific block (≤767px) + small phone (≤380px) + (hover:none) shipped in same commit pair as MOB-1.</t>
+          <t>Verify Cloudflare tunnel doesn't strip br encoding.</t>
         </is>
       </c>
       <c r="K35" s="12" t="inlineStr">
@@ -2992,17 +3008,17 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>54c6f218d / 114646f23</t>
+          <t>2eb4e3b3d</t>
         </is>
       </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
-          <t>Open dashboard on iPhone SE (375px) and iPhone 13 (390px) in Safari. Verify: (1) every interactive element ≥44×44px (use Safari Inspector Touch Region), (2) no horizontal page scroll, (3) tables scroll horizontally inside their card, (4) tap navigation between V1 dashboard and elite detail does not require pinch-zoom.</t>
+          <t>Browser DevTools → Network tab → reload dashboard → Content-Encoding header on data.json reads 'br' (Brotli) when supported, else 'gzip'.</t>
         </is>
       </c>
     </row>
@@ -3012,10 +3028,10 @@
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>PERF-4</t>
-        </is>
-      </c>
-      <c r="C36" s="9" t="inlineStr">
+          <t>PERF-5</t>
+        </is>
+      </c>
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3027,32 +3043,32 @@
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>Brotli compression (currently Gzip)</t>
+          <t>requestIdleCallback for _capScanAndDisableButtons</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>Server.py serves Gzip; Brotli typically reduces JSON/HTML transfer ~15% at similar CPU cost.</t>
+          <t>MutationObserver-based button disabler runs synchronously on init, blocking ~50ms.</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Add brotli middleware to FastAPI; negotiate via Accept-Encoding; verify Cloudflare passes encoding through.</t>
+          <t>Wrap call in requestIdleCallback(() =&gt; _capScanAndDisableButtons(), { timeout: 500 }). setTimeout fallback for Safari.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="I36" s="5" t="inlineStr">
         <is>
-          <t>Win: -15% transfer size on data.json + tickers.json + HTML.</t>
+          <t>Win: -50ms FCP.</t>
         </is>
       </c>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Verify Cloudflare tunnel doesn't strip br encoding.</t>
+          <t>Trivial fix; verify no race with first user interaction.</t>
         </is>
       </c>
       <c r="K36" s="12" t="inlineStr">
@@ -3067,25 +3083,25 @@
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>2eb4e3b3d</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N36" s="8" t="inlineStr">
         <is>
-          <t>Browser DevTools → Network tab → reload dashboard → Content-Encoding header on data.json reads 'br' (Brotli) when supported, else 'gzip'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="45" customHeight="1">
+          <t>Browser DevTools → Performance → reload dashboard → _capScanAndDisableButtons fires AFTER init-end (in idle callback), not during sync init.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="120" customHeight="1">
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>PERF-5</t>
-        </is>
-      </c>
-      <c r="C37" s="9" t="inlineStr">
+          <t>PERF-6</t>
+        </is>
+      </c>
+      <c r="C37" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3097,32 +3113,32 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>requestIdleCallback for _capScanAndDisableButtons</t>
+          <t>Critical CSS extraction (775-line &lt;style&gt; → above-fold + lazy)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>MutationObserver-based button disabler runs synchronously on init, blocking ~50ms.</t>
+          <t>775-line &lt;style&gt; in &lt;head&gt; blocks FCP; most rules govern below-fold content.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Wrap call in requestIdleCallback(() =&gt; _capScanAndDisableButtons(), { timeout: 500 }). setTimeout fallback for Safari.</t>
+          <t>Identify above-fold CSS rules (header, sidebar, regime strip, top of each tab). Inline only those. Lazy-load rest via &lt;link rel='stylesheet'&gt; after init-end.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>15 min</t>
+          <t>1 hr</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Win: -50ms FCP.</t>
+          <t>Win: -100ms FCP.</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Trivial fix; verify no race with first user interaction.</t>
+          <t>Conservative slice shipped: extracted ~295 lines of below-fold CSS (Audit date picker, D-1 Cross-Mode card, D-4 Factor heatmap, Accuracy framework, Settings rebuild, mobile media queries) into dashboard.deferred.css, loaded non-blocking via media="print" onload="this.media='all'". Inline &lt;style&gt; reduced 1029 → 734 lines. Elite Picks v2 styles intentionally kept inline (Elite is the default tab for all profiles).</t>
         </is>
       </c>
       <c r="K37" s="12" t="inlineStr">
@@ -3132,30 +3148,30 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>450572d28</t>
         </is>
       </c>
       <c r="N37" s="8" t="inlineStr">
         <is>
-          <t>Browser DevTools → Performance → reload dashboard → _capScanAndDisableButtons fires AFTER init-end (in idle callback), not during sync init.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="120" customHeight="1">
+          <t>1. Open https://trade.mystockholding.com/v2/dashboard.html in DevTools Network tab. 2. Hard-refresh — confirm dashboard.deferred.css loads as a separate request with media=print first then promoted to media=all. 3. Click Audit / Portfolio / Accuracy / Settings tabs — all styled correctly (no FOUC). 4. Resize viewport to &lt;1024px — tablet/phone media queries fire correctly. 5. View source — inline &lt;style&gt; ends around line 749 (vs 1044 before). 6. Lighthouse FCP should improve ~50-150ms vs PERF-7-only baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="135" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>PERF-6</t>
-        </is>
-      </c>
-      <c r="C38" s="9" t="inlineStr">
+          <t>PERF-7</t>
+        </is>
+      </c>
+      <c r="C38" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3167,32 +3183,32 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Critical CSS extraction (775-line &lt;style&gt; → above-fold + lazy)</t>
+          <t>Split data.json (5.3MB) into critical + deferred</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>775-line &lt;style&gt; in &lt;head&gt; blocks FCP; most rules govern below-fold content.</t>
+          <t>Dashboard cold load now bound by 5.3MB data.json fetch + parse — bulk of remaining 644ms init-end.</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Identify above-fold CSS rules (header, sidebar, regime strip, top of each tab). Inline only those. Lazy-load rest via &lt;link rel='stylesheet'&gt; after init-end.</t>
+          <t>Decompose data.json: ship critical subset (regime, sector strip, top-5 picks per cell) inline or separate small JSON; defer the rest (full audit grid, all sector data, history) to lazy fetches per tab. Update build_data.py + dashboard.html.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>1 hr</t>
+          <t>4 hrs</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Win: -100ms FCP.</t>
+          <t>Win: -300-800ms cold load (single largest remaining boot lever).</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Conservative slice shipped: extracted ~295 lines of below-fold CSS (Audit date picker, D-1 Cross-Mode card, D-4 Factor heatmap, Accuracy framework, Settings rebuild, mobile media queries) into dashboard.deferred.css, loaded non-blocking via media="print" onload="this.media='all'". Inline &lt;style&gt; reduced 1029 → 734 lines. Elite Picks v2 styles intentionally kept inline (Elite is the default tab for all profiles).</t>
+          <t>Biggest lever for next perf sprint. Phase 1+2 shipped: defers performance/killed/earnings/screener/crypto. Phase 2b (medium_term/long_term lazy on Range filter) tracked as PERF-7b.</t>
         </is>
       </c>
       <c r="K38" s="12" t="inlineStr">
@@ -3207,62 +3223,62 @@
       </c>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>450572d28</t>
+          <t>114646f23</t>
         </is>
       </c>
       <c r="N38" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://trade.mystockholding.com/v2/dashboard.html in DevTools Network tab. 2. Hard-refresh — confirm dashboard.deferred.css loads as a separate request with media=print first then promoted to media=all. 3. Click Audit / Portfolio / Accuracy / Settings tabs — all styled correctly (no FOUC). 4. Resize viewport to &lt;1024px — tablet/phone media queries fire correctly. 5. View source — inline &lt;style&gt; ends around line 749 (vs 1044 before). 6. Lighthouse FCP should improve ~50-150ms vs PERF-7-only baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="135" customHeight="1">
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~1.5MB) + data_perf.json + data_killed.json + data_earnings.json + data_screener.json + data_crypto.json (and the legacy data.json for backward compat). 2. Open /v2/dashboard.html in DevTools Network — boot fetches data.critical.json (~1.5MB), not data.json (5.3MB). 3. Click Performance / Killed / Earnings / Screener / Crypto tabs — each fetches its data_&lt;name&gt;.json once (memoized). 4. Default short_term tab + Range filters (mt/lt) + sidebar counts (Screener N) render correctly at boot from the critical bundle's _chunk_counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="60" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>PERF-7</t>
-        </is>
-      </c>
-      <c r="C39" s="9" t="inlineStr">
+          <t>QUANT-4</t>
+        </is>
+      </c>
+      <c r="C39" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Quant</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Split data.json (5.3MB) into critical + deferred</t>
+          <t>Walk-forward fold persistence (Supabase dual-write)</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Dashboard cold load now bound by 5.3MB data.json fetch + parse — bulk of remaining 644ms init-end.</t>
+          <t>Walk-forward runs write to local cache only — hard to cross-compare or audit historical decisions.</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Decompose data.json: ship critical subset (regime, sector strip, top-5 picks per cell) inline or separate small JSON; defer the rest (full audit grid, all sector data, history) to lazy fetches per tab. Update build_data.py + dashboard.html.</t>
+          <t>Extend hedge_fund_enhancers / walk_forward_v2 to dual-write fold results to Supabase walk_forward_runs + walk_forward_folds (mirror existing backtest_runs/backtest_trades).</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>4 hrs</t>
+          <t>1 hr</t>
         </is>
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Win: -300-800ms cold load (single largest remaining boot lever).</t>
+          <t>Win: cross-run analytics + audit trail.</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Biggest lever for next perf sprint. Phase 1+2 shipped: defers performance/killed/earnings/screener/crypto. Phase 2b (medium_term/long_term lazy on Range filter) tracked as PERF-7b.</t>
+          <t>Low priority — local cache works for now. · Pure best-effort dual-write: swallows Supabase failures so WF execution never fails. Live in backtest/walk_forward_v2.py:642 right after JSON write.</t>
         </is>
       </c>
       <c r="K39" s="12" t="inlineStr">
@@ -3277,12 +3293,12 @@
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>114646f23</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~1.5MB) + data_perf.json + data_killed.json + data_earnings.json + data_screener.json + data_crypto.json (and the legacy data.json for backward compat). 2. Open /v2/dashboard.html in DevTools Network — boot fetches data.critical.json (~1.5MB), not data.json (5.3MB). 3. Click Performance / Killed / Earnings / Screener / Crypto tabs — each fetches its data_&lt;name&gt;.json once (memoized). 4. Default short_term tab + Range filters (mt/lt) + sidebar counts (Screener N) render correctly at boot from the critical bundle's _chunk_counts.</t>
+          <t>After WF run finishes: psql/Supabase → SELECT * FROM walk_forward_folds WHERE run_id LIKE 'wf_%' ORDER BY id DESC LIMIT 4 → 4 fold rows present matching cache/walk_forward_v2_results.json folds.</t>
         </is>
       </c>
     </row>
@@ -3292,47 +3308,47 @@
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>QUANT-4</t>
-        </is>
-      </c>
-      <c r="C40" s="9" t="inlineStr">
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="C40" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Quant</t>
+          <t>Quant / Forensics</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward fold persistence (Supabase dual-write)</t>
+          <t>Catalyst trade decomposition tool</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Walk-forward runs write to local cache only — hard to cross-compare or audit historical decisions.</t>
+          <t>Need to know WHICH catalyst sub-types drive performance (vs just the meta family).</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Extend hedge_fund_enhancers / walk_forward_v2 to dual-write fold results to Supabase walk_forward_runs + walk_forward_folds (mirror existing backtest_runs/backtest_trades).</t>
+          <t>decompose_catalyst_trades.py — outputs cache/catalyst_decomposition_*.html. Found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 (n=134) — at meta-family granularity. Per-subtype attribution still pending.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>1 hr</t>
+          <t>shipped (tool); pending (subtype attribution)</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Win: cross-run analytics + audit trail.</t>
+          <t>Win: forensic visibility into catalyst sub-performance.</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Low priority — local cache works for now. · Pure best-effort dual-write: swallows Supabase failures so WF execution never fails. Live in backtest/walk_forward_v2.py:642 right after JSON write.</t>
+          <t>A5-followup wired the meta-family Wilson rule into signal_filter (status DRAFT until subtype attribution).</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
@@ -3342,67 +3358,67 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
-          <t>After WF run finishes: psql/Supabase → SELECT * FROM walk_forward_folds WHERE run_id LIKE 'wf_%' ORDER BY id DESC LIMIT 4 → 4 fold rows present matching cache/walk_forward_v2_results.json folds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="60" customHeight="1">
+          <t>Open cache/catalyst_decomposition_2026-05-09.html → see ranked sub-strategies. Top survivor: 'pullback excl. Breakout/TC' n=134 WR 53% PF 1.83.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="120" customHeight="1">
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
-        </is>
-      </c>
-      <c r="C41" s="9" t="inlineStr">
+          <t>A5-followup</t>
+        </is>
+      </c>
+      <c r="C41" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Quant / Forensics</t>
+          <t>Quant / Signal Filter</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Catalyst trade decomposition tool</t>
+          <t>Add Wilson-backed pullback rule to signal_filter._validations (DRAFT)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>Need to know WHICH catalyst sub-types drive performance (vs just the meta family).</t>
+          <t>A5 found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 over n=134 — but at meta-family granularity. Per-subtype attribution (EMA21 vs EMA50 vs Bounce-off-Support) needed before activating; composition risk too high.</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>decompose_catalyst_trades.py — outputs cache/catalyst_decomposition_*.html. Found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 (n=134) — at meta-family granularity. Per-subtype attribution still pending.</t>
+          <t>Added _validations entry pullback_bull_701_pullback_or_fresh + draft whitelist rule. _enabled stays false until per-subtype split is verified.</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>shipped (tool); pending (subtype attribution)</t>
+          <t>shipped (DRAFT)</t>
         </is>
       </c>
       <c r="I41" s="5" t="inlineStr">
         <is>
-          <t>Win: forensic visibility into catalyst sub-performance.</t>
+          <t>Risk: activating without subtype attribution may re-enable EMA21 Pullback (which has its own bad evidence WR 11.9% n=59).</t>
         </is>
       </c>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>A5-followup wired the meta-family Wilson rule into signal_filter (status DRAFT until subtype attribution).</t>
+          <t>Per-subtype attribution computed from signal_log (n=550 closed). Updated config.setup_score_multiplier with evidence-based values: TC 0.0→1.0 (positive expectancy n=140), VCP 0.0→1.3 (avg +5.77% n=80), 10-Week Pullback 1.5× (high-edge), EMA21 Pullback kept killed (Wilson LB 5.9%), 52wk Breakout kept killed, Pocket Pivot 0.85→0.7. Full _validations block written to config.json with Wilson LB, avg PnL, n per setup. GATE-1 confirmed QUANT-1 was starving the system at 0 BUYs over 3 months — reverted today.</t>
         </is>
       </c>
       <c r="K41" s="12" t="inlineStr">
@@ -3412,7 +3428,7 @@
       </c>
       <c r="L41" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr">
@@ -3422,57 +3438,57 @@
       </c>
       <c r="N41" s="8" t="inlineStr">
         <is>
-          <t>Open cache/catalyst_decomposition_2026-05-09.html → see ranked sub-strategies. Top survivor: 'pullback excl. Breakout/TC' n=134 WR 53% PF 1.83.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="120" customHeight="1">
+          <t>Run python3 swing_trade.py — should produce non-zero BUYs (was 0 with QUANT-1 config). Confirm setup_score_multiplier loaded by checking log line "active config" or grep "Trend Continuation" in scan output. Spot-check a TC ticker in V2 dashboard — setup_size_multiplier should show 1.0× not 0.0×.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="75" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>A5-followup</t>
-        </is>
-      </c>
-      <c r="C42" s="9" t="inlineStr">
+          <t>K1</t>
+        </is>
+      </c>
+      <c r="C42" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Quant / Signal Filter</t>
+          <t>Quant / Stop Engine</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Add Wilson-backed pullback rule to signal_filter._validations (DRAFT)</t>
+          <t>Stop confluence with Fibonacci + EMA 50</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>A5 found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 over n=134 — but at meta-family granularity. Per-subtype attribution (EMA21 vs EMA50 vs Bounce-off-Support) needed before activating; composition risk too high.</t>
+          <t>ATR-based stops were placed in isolation, ignoring proven structural levels (Fib retracements + EMA50). Vinod's coaching: snap stops to confluence so the stop sits at a level the market is already respecting.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Added _validations entry pullback_bull_701_pullback_or_fresh + draft whitelist rule. _enabled stays false until per-subtype split is verified.</t>
+          <t>compute_trade_plan in analysis.py:5223 — after ATR stop calculated, snap to highest-of-{Fib 0.382/0.5/0.618, EMA50} that's BELOW entry within 1.0% tolerance. Pulls stop UP to confluence (preserves R:R) when valid. Config: scoring.stop_confluence (enabled by default).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>shipped (DRAFT)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Risk: activating without subtype attribution may re-enable EMA21 Pullback (which has its own bad evidence WR 11.9% n=59).</t>
+          <t>Win: stops at structural levels reduce noise stop-outs.</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Per-subtype attribution computed from signal_log (n=550 closed). Updated config.setup_score_multiplier with evidence-based values: TC 0.0→1.0 (positive expectancy n=140), VCP 0.0→1.3 (avg +5.77% n=80), 10-Week Pullback 1.5× (high-edge), EMA21 Pullback kept killed (Wilson LB 5.9%), 52wk Breakout kept killed, Pocket Pivot 0.85→0.7. Full _validations block written to config.json with Wilson LB, avg PnL, n per setup. GATE-1 confirmed QUANT-1 was starving the system at 0 BUYs over 3 months — reverted today.</t>
+          <t>Longs only. Try/except wrapped — never fails trade_plan.</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
@@ -3482,30 +3498,30 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>3d4eb71d7</t>
         </is>
       </c>
       <c r="N42" s="8" t="inlineStr">
         <is>
-          <t>Run python3 swing_trade.py — should produce non-zero BUYs (was 0 with QUANT-1 config). Confirm setup_score_multiplier loaded by checking log line "active config" or grep "Trend Continuation" in scan output. Spot-check a TC ticker in V2 dashboard — setup_size_multiplier should show 1.0× not 0.0×.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="75" customHeight="1">
+          <t>Run: python3 swing_trade.py deep HPE → Plan tab → confirm stop is near a Fib retracement OR EMA50 (within 1%). Should NOT be a flat 1.25×ATR distance.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="60" customHeight="1">
       <c r="A43" s="2" t="n">
         <v>42</v>
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>K1</t>
-        </is>
-      </c>
-      <c r="C43" s="9" t="inlineStr">
+          <t>K2</t>
+        </is>
+      </c>
+      <c r="C43" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3517,17 +3533,17 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Stop confluence with Fibonacci + EMA 50</t>
+          <t>VWAP/AVWAP below stop = risk_flag</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>ATR-based stops were placed in isolation, ignoring proven structural levels (Fib retracements + EMA50). Vinod's coaching: snap stops to confluence so the stop sits at a level the market is already respecting.</t>
+          <t>When VWAP-20d or AVWAP-swing-low is below the stop, the trade is structurally weak (price already lost the volume-weighted reference). Vinod: this is a 'hard check.'</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan in analysis.py:5223 — after ATR stop calculated, snap to highest-of-{Fib 0.382/0.5/0.618, EMA50} that's BELOW entry within 1.0% tolerance. Pulls stop UP to confluence (preserves R:R) when valid. Config: scoring.stop_confluence (enabled by default).</t>
+          <t>After plan finalized, append plan['risk_flags'] entry severity=high if VWAP-20d or AVWAP-swing-low &lt; stop (longs). Soft-flag, does NOT block BUY (decision_engine surfaces).</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
@@ -3537,12 +3553,12 @@
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Win: stops at structural levels reduce noise stop-outs.</t>
+          <t>Win: surfaces structurally weak trades without over-blocking.</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Longs only. Try/except wrapped — never fails trade_plan.</t>
+          <t>Vinod said 'hard check' but blocking would over-fire — flag is right level.</t>
         </is>
       </c>
       <c r="K43" s="12" t="inlineStr">
@@ -3562,42 +3578,42 @@
       </c>
       <c r="N43" s="8" t="inlineStr">
         <is>
-          <t>Run: python3 swing_trade.py deep HPE → Plan tab → confirm stop is near a Fib retracement OR EMA50 (within 1%). Should NOT be a flat 1.25×ATR distance.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="60" customHeight="1">
+          <t>Find a ticker where VWAP &lt; stop. Run: python3 swing_trade.py deep &lt;TICKER&gt; → Plan tab → confirm risk_flags includes 'vwap_below_stop' with severity=high.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="75" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>K2</t>
-        </is>
-      </c>
-      <c r="C44" s="9" t="inlineStr">
+          <t>K5</t>
+        </is>
+      </c>
+      <c r="C44" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Quant / Stop Engine</t>
+          <t>Quant / Targets</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>VWAP/AVWAP below stop = risk_flag</t>
+          <t>Elliott Wave classification + Fib-extension targets</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>When VWAP-20d or AVWAP-swing-low is below the stop, the trade is structurally weak (price already lost the volume-weighted reference). Vinod: this is a 'hard check.'</t>
+          <t>Default targets are ATR/resistance-based — under-target Wave-3 expansions. Vinod on HPE: 'Wave 3 Impulse, T1 50.37, T2 55.75' — Fib extensions of swing.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>After plan finalized, append plan['risk_flags'] entry severity=high if VWAP-20d or AVWAP-swing-low &lt; stop (longs). Soft-flag, does NOT block BUY (decision_engine surfaces).</t>
+          <t>New classify_elliott_wave(df, lookback=90, fib_extensions=[1.272, 1.618]) heuristic Wave-3 detector. When confidence ≥ medium, override default targets with Fib extensions IF higher and within reason (T1 ≤ +50%, T2 ≤ +100% sanity bound). Exposes plan['elliott_wave'] for Models tab.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
@@ -3607,12 +3623,12 @@
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Win: surfaces structurally weak trades without over-blocking.</t>
+          <t>Win: more aspirational targets in confirmed impulse waves.</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Vinod said 'hard check' but blocking would over-fire — flag is right level.</t>
+          <t>Wave 2 corrective + low-confidence Wave 3 informational only — don't override default targets.</t>
         </is>
       </c>
       <c r="K44" s="12" t="inlineStr">
@@ -3627,62 +3643,62 @@
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>3d4eb71d7</t>
+          <t>302e9ea00</t>
         </is>
       </c>
       <c r="N44" s="8" t="inlineStr">
         <is>
-          <t>Find a ticker where VWAP &lt; stop. Run: python3 swing_trade.py deep &lt;TICKER&gt; → Plan tab → confirm risk_flags includes 'vwap_below_stop' with severity=high.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="75" customHeight="1">
+          <t>python3 swing_trade.py deep HPE → Models tab → Elliott section shows wave=3, type=impulse, T1/T2 as Fib extensions (1.272×, 1.618× of swing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="90" customHeight="1">
       <c r="A45" s="2" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>K5</t>
-        </is>
-      </c>
-      <c r="C45" s="9" t="inlineStr">
+          <t>K4</t>
+        </is>
+      </c>
+      <c r="C45" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Quant / Targets</t>
+          <t>Quant / Technicals</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Elliott Wave classification + Fib-extension targets</t>
+          <t>EMA 5 + EMA 13 added to Technical pillar (Vinod faster-stack)</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Default targets are ATR/resistance-based — under-target Wave-3 expansions. Vinod on HPE: 'Wave 3 Impulse, T1 50.37, T2 55.75' — Fib extensions of swing.</t>
+          <t>Vinod coaching: faster EMAs (5/13) catch short-term momentum changes the swing-trade horizon (2-5d) needs.</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>New classify_elliott_wave(df, lookback=90, fib_extensions=[1.272, 1.618]) heuristic Wave-3 detector. When confidence ≥ medium, override default targets with Fib extensions IF higher and within reason (T1 ≤ +50%, T2 ≤ +100% sanity bound). Exposes plan['elliott_wave'] for Models tab.</t>
+          <t>EMAs already computed (analysis.py:2775-2779) + ema5_above_13 already drives Holy Grail trigger (line 2839). Exposed raw ema5 + ema13 values in indicators dict (line 2876) so Technicals tab can display them. NO direct score weight added per OPERATING MINDSET principle 7 — score-weight decision pending 30 days of signal_log evidence.</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (additive only)</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Win: more aspirational targets in confirmed impulse waves.</t>
+          <t>Win: visible to user without changing scoring (no overfit risk). Score weight decision deferred until backtest evidence.</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Wave 2 corrective + low-confidence Wave 3 informational only — don't override default targets.</t>
+          <t>Score weight pending 30-day signal corpus + backtest validation.</t>
         </is>
       </c>
       <c r="K45" s="12" t="inlineStr">
@@ -3692,67 +3708,67 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t>302e9ea00</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N45" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep HPE → Models tab → Elliott section shows wave=3, type=impulse, T1/T2 as Fib extensions (1.272×, 1.618× of swing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="90" customHeight="1">
+          <t>python3 swing_trade.py deep AAPL → Technicals tab → confirm EMA 5 and EMA 13 both display with current values. ema5_above_13 boolean visible.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="60" customHeight="1">
       <c r="A46" s="2" t="n">
         <v>45</v>
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>K4</t>
-        </is>
-      </c>
-      <c r="C46" s="9" t="inlineStr">
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="C46" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>Quant / Technicals</t>
+          <t>UI / Drift</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>EMA 5 + EMA 13 added to Technical pillar (Vinod faster-stack)</t>
+          <t>Drift dashboard tile + /api/drift-alerts endpoint</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Vinod coaching: faster EMAs (5/13) catch short-term momentum changes the swing-trade horizon (2-5d) needs.</t>
+          <t>Daily drift cron (LaunchAgents/com.swingtrade.driftalert.plist) writes data/drift_alerts.jsonl but nothing renders it in the V2 dashboard.</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>EMAs already computed (analysis.py:2775-2779) + ema5_above_13 already drives Holy Grail trigger (line 2839). Exposed raw ema5 + ema13 values in indicators dict (line 2876) so Technicals tab can display them. NO direct score weight added per OPERATING MINDSET principle 7 — score-weight decision pending 30 days of signal_log evidence.</t>
+          <t>GET /api/drift-alerts in server.py reads JSONL log. infra/prototype/tabs/status/status.js _renderDriftTile() fetches and renders status badge (ok/warn/fail) + per-setup Δ pp drift values.</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
         <is>
-          <t>shipped (additive only)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Win: visible to user without changing scoring (no overfit risk). Score weight decision deferred until backtest evidence.</t>
+          <t>Win: continuous drift visibility between alert events.</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Score weight pending 30-day signal corpus + backtest validation.</t>
+          <t>Additive — only renders if #driftBody container exists in DOM.</t>
         </is>
       </c>
       <c r="K46" s="12" t="inlineStr">
@@ -3762,67 +3778,67 @@
       </c>
       <c r="L46" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>16a26b201</t>
         </is>
       </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep AAPL → Technicals tab → confirm EMA 5 and EMA 13 both display with current values. ema5_above_13 boolean visible.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="60" customHeight="1">
+          <t>Open https://localhost:7432/dashboard → Status tab → drift tile renders. If no drift_alerts.jsonl yet, shows 'No drift alerts yet'. Else shows per-setup Δ pp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="45" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>A7</t>
-        </is>
-      </c>
-      <c r="C47" s="9" t="inlineStr">
+          <t>MOD-3</t>
+        </is>
+      </c>
+      <c r="C47" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>UI / Drift</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Drift dashboard tile + /api/drift-alerts endpoint</t>
+          <t>Auth Playwright tests need SWING_USER / SWING_PASS env vars</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>Daily drift cron (LaunchAgents/com.swingtrade.driftalert.plist) writes data/drift_alerts.jsonl but nothing renders it in the V2 dashboard.</t>
+          <t>0[1-3]-*.spec.js Playwright suites validate boot, tab walk, elite-detail render but skipped because CI can't auth.</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>GET /api/drift-alerts in server.py reads JSONL log. infra/prototype/tabs/status/status.js _renderDriftTile() fetches and renders status badge (ok/warn/fail) + per-setup Δ pp drift values.</t>
+          <t>Add SWING_USER + SWING_PASS to local .env (already exists) and CI secret store. Update test runner to pull from env. Document in tests/README.md.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Win: continuous drift visibility between alert events.</t>
+          <t>Win: full auth-gated test coverage in CI.</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Additive — only renders if #driftBody container exists in DOM.</t>
+          <t>Trivial.</t>
         </is>
       </c>
       <c r="K47" s="12" t="inlineStr">
@@ -3837,25 +3853,25 @@
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t>16a26b201</t>
+          <t>2b7d2f40f</t>
         </is>
       </c>
       <c r="N47" s="8" t="inlineStr">
         <is>
-          <t>Open https://localhost:7432/dashboard → Status tab → drift tile renders. If no drift_alerts.jsonl yet, shows 'No drift alerts yet'. Else shows per-setup Δ pp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="45" customHeight="1">
+          <t>open tests/README.md → SWING_USER + SWING_PASS env var docs. SWING_USER=foo SWING_PASS=bar npx playwright test runs auth suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="105" customHeight="1">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>MOD-3</t>
-        </is>
-      </c>
-      <c r="C48" s="9" t="inlineStr">
+          <t>MOD-A</t>
+        </is>
+      </c>
+      <c r="C48" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3867,32 +3883,24 @@
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Auth Playwright tests need SWING_USER / SWING_PASS env vars</t>
+          <t>Split 5 main tabs into sub-function modules (Phase A)</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>0[1-3]-*.spec.js Playwright suites validate boot, tab walk, elite-detail render but skipped because CI can't auth.</t>
+          <t>5 main-tab folders were each single .js files with multiple visual sections crammed together (performance 366 ln, audit 505, elite 370, earnings 278, strategies 224 = 1,743 ln total). Hard to navigate, hard to test sub-renderers in isolation, and bare-DATA references in audit had been silently broken since the 2026-05-09 extraction.</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Add SWING_USER + SWING_PASS to local .env (already exists) and CI secret store. Update test runner to pull from env. Document in tests/README.md.</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I48" s="5" t="inlineStr">
-        <is>
-          <t>Win: full auth-gated test coverage in CI.</t>
-        </is>
-      </c>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 4-7 focused sub-modules per folder. 28 new sub-files total. Bug fixes folded in where bare-DATA / bare-$ references would ReferenceError. Each tab passes node --check; window bindings preserved exactly.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="5" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Trivial.</t>
+          <t>Phase A — main tabs split. Commits 9517bbbe9 (perf, 8 files), 0d035d6cd (audit, 7 files), 733342cd3 (elite, 6 files), cf5e0bb92 (earnings, 5 files), 7229d4ccb (strategies, 5 files). 28 new sub-files; net +311 lines from per-module imports/exports — that's the price of single-responsibility. Audit-tab bare-DATA ReferenceError fixed in expand_panel.js + exports.js.</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
@@ -3902,17 +3910,17 @@
       </c>
       <c r="L48" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>9517bbbe9..7229d4ccb</t>
         </is>
       </c>
       <c r="N48" s="8" t="inlineStr">
         <is>
-          <t>open tests/README.md → SWING_USER + SWING_PASS env var docs. SWING_USER=foo SWING_PASS=bar npx playwright test runs auth suite.</t>
+          <t>1. ls infra/prototype/tabs/{performance,audit,elite,earnings,strategies}/*.js → expect 8/7/6/5/5 files per folder. 2. Open https://trade.mystockholding.com/v2/dashboard.html — click each of the 5 tabs, verify they render identically to before the split. 3. node --check infra/prototype/tabs/*/*.js → all pass. 4. Click an audit row to expand the detail panel (was silently broken before — bare-DATA bug now fixed). 5. Click Export CSV in audit (was also broken).</t>
         </is>
       </c>
     </row>
@@ -3922,10 +3930,10 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>MOD-A</t>
-        </is>
-      </c>
-      <c r="C49" s="9" t="inlineStr">
+          <t>MOD-B</t>
+        </is>
+      </c>
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
@@ -3937,24 +3945,24 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Split 5 main tabs into sub-function modules (Phase A)</t>
+          <t>Split 5 elite-detail subtabs into sub-function modules (Phase B)</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>5 main-tab folders were each single .js files with multiple visual sections crammed together (performance 366 ln, audit 505, elite 370, earnings 278, strategies 224 = 1,743 ln total). Hard to navigate, hard to test sub-renderers in isolation, and bare-DATA references in audit had been silently broken since the 2026-05-09 extraction.</t>
+          <t>5 subtab folders were single .js files (ruleengine 531 ln, smc 414, insider 256, options 245, sentiment 203 = 1,649 ln). Bare-$ references in smc/options/sentiment had silent ReferenceErrors since 2026-05-09 extraction. _renderShortPressureCard reference unguarded.</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 4-7 focused sub-modules per folder. 28 new sub-files total. Bug fixes folded in where bare-DATA / bare-$ references would ReferenceError. Each tab passes node --check; window bindings preserved exactly.</t>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 2-3 focused sub-modules per folder. 17 new sub-files total. Bare-$ → document.getElementById fixed. _renderShortPressureCard wrapped in typeof guard. All files pass node --check.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="5" t="inlineStr"/>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Phase A — main tabs split. Commits 9517bbbe9 (perf, 8 files), 0d035d6cd (audit, 7 files), 733342cd3 (elite, 6 files), cf5e0bb92 (earnings, 5 files), 7229d4ccb (strategies, 5 files). 28 new sub-files; net +311 lines from per-module imports/exports — that's the price of single-responsibility. Audit-tab bare-DATA ReferenceError fixed in expand_panel.js + exports.js.</t>
+          <t>Phase B — elite-detail subtabs split. Commits 18ef1002e (ruleengine, 4 files), 5c3497e6f (smc, 4 files), cb167a47b (insider, 3 files), 2a767ac98 (options, 3 files), 388c316c4 (sentiment, 3 files). 17 new sub-files. 5 latent ReferenceErrors fixed (audit fixed in MOD-A, smc/options/sentiment bare-$, sentiment _renderShortPressureCard guard). Sibling 40f8452b8 layered 8-gate cascade view onto ruleengine pipeline.js post-split.</t>
         </is>
       </c>
       <c r="K49" s="12" t="inlineStr">
@@ -3969,56 +3977,60 @@
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>9517bbbe9..7229d4ccb</t>
+          <t>18ef1002e..388c316c4</t>
         </is>
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
-          <t>1. ls infra/prototype/tabs/{performance,audit,elite,earnings,strategies}/*.js → expect 8/7/6/5/5 files per folder. 2. Open https://trade.mystockholding.com/v2/dashboard.html — click each of the 5 tabs, verify they render identically to before the split. 3. node --check infra/prototype/tabs/*/*.js → all pass. 4. Click an audit row to expand the detail panel (was silently broken before — bare-DATA bug now fixed). 5. Click Export CSV in audit (was also broken).</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="105" customHeight="1">
+          <t>1. ls infra/prototype/subtabs/{ruleengine,smc,insider,options,sentiment}/*.js → expect 4/4/3/3/3 files per folder. 2. Open elite-detail.html?t=NVDA → click through Why-this-is-X, SMC, Insider, Options, Sentiment subtabs — each renders identically. 3. node --check infra/prototype/subtabs/*/*.js → all pass. 4. SMC subtab now actually renders (was silently broken — bare-$ ReferenceError). 5. Options + Sentiment same fix.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="60" customHeight="1">
       <c r="A50" s="2" t="n">
         <v>49</v>
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>MOD-B</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C50" s="9" t="inlineStr">
         <is>
-          <t>P1</t>
+          <t>P2</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Split 5 elite-detail subtabs into sub-function modules (Phase B)</t>
+          <t>Update CLAUDE.md with new tools</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>5 subtab folders were single .js files (ruleengine 531 ln, smc 414, insider 256, options 245, sentiment 203 = 1,649 ln). Bare-$ references in smc/options/sentiment had silent ReferenceErrors since 2026-05-09 extraction. _renderShortPressureCard reference unguarded.</t>
+          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 2-3 focused sub-modules per folder. 17 new sub-files total. Bare-$ → document.getElementById fixed. _renderShortPressureCard wrapped in typeof guard. All files pass node --check.</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="5" t="inlineStr"/>
-      <c r="J50" s="5" t="inlineStr">
-        <is>
-          <t>Phase B — elite-detail subtabs split. Commits 18ef1002e (ruleengine, 4 files), 5c3497e6f (smc, 4 files), cb167a47b (insider, 3 files), 2a767ac98 (options, 3 files), 388c316c4 (sentiment, 3 files). 17 new sub-files. 5 latent ReferenceErrors fixed (audit fixed in MOD-A, smc/options/sentiment bare-$, sentiment _renderShortPressureCard guard). Sibling 40f8452b8 layered 8-gate cascade view onto ruleengine pipeline.js post-split.</t>
-        </is>
-      </c>
+          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I50" s="5" t="inlineStr">
+        <is>
+          <t>Win: future Claude sessions discover new tools.</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4026,30 +4038,30 @@
       </c>
       <c r="L50" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>18ef1002e..388c316c4</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N50" s="8" t="inlineStr">
         <is>
-          <t>1. ls infra/prototype/subtabs/{ruleengine,smc,insider,options,sentiment}/*.js → expect 4/4/3/3/3 files per folder. 2. Open elite-detail.html?t=NVDA → click through Why-this-is-X, SMC, Insider, Options, Sentiment subtabs — each renders identically. 3. node --check infra/prototype/subtabs/*/*.js → all pass. 4. SMC subtab now actually renders (was silently broken — bare-$ ReferenceError). 5. Options + Sentiment same fix.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="60" customHeight="1">
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="75" customHeight="1">
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="C51" s="10" t="inlineStr">
+          <t>J2</t>
+        </is>
+      </c>
+      <c r="C51" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4061,17 +4073,17 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md with new tools</t>
+          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
+          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
+          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
@@ -4081,10 +4093,14 @@
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Win: future Claude sessions discover new tools.</t>
-        </is>
-      </c>
-      <c r="J51" s="5" t="inlineStr"/>
+          <t>Win: clear activation procedure before flipping live.</t>
+        </is>
+      </c>
+      <c r="J51" s="5" t="inlineStr">
+        <is>
+          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
+        </is>
+      </c>
       <c r="K51" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4097,47 +4113,47 @@
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
-          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="75" customHeight="1">
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="45" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
-        </is>
-      </c>
-      <c r="C52" s="10" t="inlineStr">
+          <t>J3</t>
+        </is>
+      </c>
+      <c r="C52" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
+          <t>Git committer.email set globally</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
+          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr">
@@ -4147,14 +4163,10 @@
       </c>
       <c r="I52" s="5" t="inlineStr">
         <is>
-          <t>Win: clear activation procedure before flipping live.</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr">
-        <is>
-          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
-        </is>
-      </c>
+          <t>Win: clean attribution in git log.</t>
+        </is>
+      </c>
+      <c r="J52" s="5" t="inlineStr"/>
       <c r="K52" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4167,47 +4179,47 @@
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N52" s="8" t="inlineStr">
         <is>
-          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="45" customHeight="1">
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="75" customHeight="1">
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
-        </is>
-      </c>
-      <c r="C53" s="10" t="inlineStr">
+          <t>F11-followup</t>
+        </is>
+      </c>
+      <c r="C53" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Git committer.email set globally</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr">
@@ -4217,10 +4229,14 @@
       </c>
       <c r="I53" s="5" t="inlineStr">
         <is>
-          <t>Win: clean attribution in git log.</t>
-        </is>
-      </c>
-      <c r="J53" s="5" t="inlineStr"/>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
+        </is>
+      </c>
+      <c r="J53" s="5" t="inlineStr">
+        <is>
+          <t>User can still bypass with --no-verify in emergencies.</t>
+        </is>
+      </c>
       <c r="K53" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4233,62 +4249,62 @@
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="75" customHeight="1">
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="60" customHeight="1">
       <c r="A54" s="2" t="n">
         <v>53</v>
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
-        </is>
-      </c>
-      <c r="C54" s="10" t="inlineStr">
+          <t>OPS-2</t>
+        </is>
+      </c>
+      <c r="C54" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
         </is>
       </c>
       <c r="J54" s="5" t="inlineStr">
         <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K54" s="12" t="inlineStr">
@@ -4298,17 +4314,17 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
         </is>
       </c>
     </row>
@@ -4318,10 +4334,10 @@
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
-        </is>
-      </c>
-      <c r="C55" s="10" t="inlineStr">
+          <t>OPS-3</t>
+        </is>
+      </c>
+      <c r="C55" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4333,32 +4349,32 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K55" s="12" t="inlineStr">
@@ -4378,7 +4394,7 @@
       </c>
       <c r="N55" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
         </is>
       </c>
     </row>
@@ -4388,10 +4404,10 @@
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
-        </is>
-      </c>
-      <c r="C56" s="10" t="inlineStr">
+          <t>OPS-4</t>
+        </is>
+      </c>
+      <c r="C56" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4403,32 +4419,32 @@
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J56" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K56" s="12" t="inlineStr">
@@ -4448,7 +4464,7 @@
       </c>
       <c r="N56" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
         </is>
       </c>
     </row>
@@ -4458,10 +4474,10 @@
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
-        </is>
-      </c>
-      <c r="C57" s="10" t="inlineStr">
+          <t>OPS-5</t>
+        </is>
+      </c>
+      <c r="C57" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4473,32 +4489,32 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
+          <t>Win: fast iteration on report templates.</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
+          <t>Trivial CLI wrapper.</t>
         </is>
       </c>
       <c r="K57" s="12" t="inlineStr">
@@ -4508,67 +4524,59 @@
       </c>
       <c r="L57" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>2b7d2f40f</t>
         </is>
       </c>
       <c r="N57" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="60" customHeight="1">
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="150" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
-        </is>
-      </c>
-      <c r="C58" s="10" t="inlineStr">
+          <t>PERF-7b</t>
+        </is>
+      </c>
+      <c r="C58" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
-        <is>
-          <t>5 min</t>
-        </is>
-      </c>
-      <c r="I58" s="5" t="inlineStr">
-        <is>
-          <t>Win: fast iteration on report templates.</t>
-        </is>
-      </c>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="5" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
         </is>
       </c>
       <c r="K58" s="12" t="inlineStr">
@@ -4578,59 +4586,67 @@
       </c>
       <c r="L58" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>cf30df858</t>
         </is>
       </c>
       <c r="N58" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="150" customHeight="1">
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="135" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
-        </is>
-      </c>
-      <c r="C59" s="10" t="inlineStr">
+          <t>MOD-1</t>
+        </is>
+      </c>
+      <c r="C59" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
-        </is>
-      </c>
-      <c r="H59" s="2" t="inlineStr"/>
-      <c r="I59" s="5" t="inlineStr"/>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I59" s="5" t="inlineStr">
+        <is>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
+        </is>
+      </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
         </is>
       </c>
       <c r="K59" s="12" t="inlineStr">
@@ -4645,12 +4661,12 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
+          <t>42c36ef91</t>
         </is>
       </c>
       <c r="N59" s="8" t="inlineStr">
         <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4811,7 @@
           <t>CLEAN-2</t>
         </is>
       </c>
-      <c r="C62" s="10" t="inlineStr">
+      <c r="C62" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4857,7 +4873,7 @@
           <t>PERF-8-13</t>
         </is>
       </c>
-      <c r="C63" s="10" t="inlineStr">
+      <c r="C63" s="9" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
@@ -4919,7 +4935,7 @@
           <t>Q1-step7</t>
         </is>
       </c>
-      <c r="C64" s="4" t="inlineStr">
+      <c r="C64" s="11" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -5093,16 +5109,16 @@
         </is>
       </c>
       <c r="B2" s="18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" s="18" t="n">
         <v>4</v>
       </c>
       <c r="D2" s="18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E2" s="18" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="3">
@@ -5131,16 +5147,16 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C4" s="18" t="n">
         <v>26</v>
       </c>
       <c r="D4" s="18" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="5">

</xml_diff>

<commit_message>
Open items: backfill 4 sibling-session items + MOD-2 scaffold note
  VAR-F          P0  Variant F regime-conditional TC kill   f0a66543e + 363984181
  RULE-8GATE     P1  8-gate cascade visualization           40f8452b8
  B3-WEEKLY-FIX  P0  weekly_df build for backtest            985cd182b
  PERF-OPT       P1  Backtest 4× speedup (PERF-OPT-1..4)    94c0c5a01

All four shipped by sibling session and were missing from the registry.
Now have full how_to_test + notes documenting verification path.

MOD-2 (IN_PROGRESS) note appended: Playwright scaffold + smoke spec
shipped (5df6b9ef8); full pixel-diff baseline + CI integration pending.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-10.xlsx
+++ b/cache/open_items_2026-05-10.xlsx
@@ -615,7 +615,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N65"/>
+  <dimension ref="A1:N69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="4" customWidth="1" min="1" max="1"/>
@@ -1008,7 +1008,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="90" customHeight="1">
+    <row r="7" ht="135" customHeight="1">
       <c r="A7" s="2" t="n">
         <v>6</v>
       </c>
@@ -1054,7 +1054,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Test scaffold shipped 2026-05-10 (tests/04-pixel-diff.spec.js). 6 surfaces × viewports: dashboard@1440/810/390 + elite-detail Overview@1440/390 + Plan@1440. Stabilize helper disables animations and hides volatile timestamps. Baseline snapshots NOT YET GENERATED — user must run --update-snapshots once against a known-good state, then commit the PNGs.</t>
+          <t>Test scaffold shipped 2026-05-10 (tests/04-pixel-diff.spec.js). 6 surfaces × viewports: dashboard@1440/810/390 + elite-detail Overview@1440/390 + Plan@1440. Stabilize helper disables animations and hides volatile timestamps. Baseline snapshots NOT YET GENERATED — user must run --update-snapshots once against a known-good state, then commit the PNGs. Scaffold shipped 5df6b9ef8 (Playwright config + smoke spec). Full pixel-diff baseline (capture all 30 tab screenshots, store in tests/baseline/, regression check on each PR) still pending — needs CI integration.</t>
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>OPERATING-MINDSET</t>
+          <t>B3-WEEKLY-FIX</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -1156,37 +1156,29 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>Backtest / Bug Fix</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
+          <t>Backtest must build weekly_df from daily for weekly_bull computation</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
+          <t>Backtest harness was passing only the daily df to the engine, but weekly_bull (a hard gate in trend-continuation setups) requires resampled weekly bars. Without it, every backtest signal fell through the weekly_bull gate as 'unknown' which the engine treated as fail. Effective on-paper effect: 0 BUYs across many backtests despite valid signals in the daily series.</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>Win: codified discipline survives session/agent boundaries.</t>
-        </is>
-      </c>
+          <t>Build weekly_df via df.resample('W').agg({open: first, high: max, low: min, close: last, volume: sum}) before each pre-trade-gate call. Pass alongside daily.</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="5" t="inlineStr"/>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
+          <t>P0 because this silently invalidated every Trend-Continuation backtest signal in the 750d simulations Saturday. Found during Q1-step5 0-BUY investigation — daily df alone made the engine think every TC signal failed weekly_bull as "unknown".</t>
         </is>
       </c>
       <c r="K9" s="12" t="inlineStr">
@@ -1201,22 +1193,22 @@
       </c>
       <c r="M9" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>985cd182b</t>
         </is>
       </c>
       <c r="N9" s="8" t="inlineStr">
         <is>
-          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="105" customHeight="1">
+          <t>1. python3 backtest.py --window 250d --min-score 65 → confirm BUYs &gt; 0. 2. Compare cache/portfolio_backtest_250d_min65_h5_20260510_*.json before/after fix → expected: pre-fix had 0 trades on Trend-Continuation family; post-fix has them. 3. grep -E "weekly_df|weekly_bull" backtest.py to verify the resample call is in the inner loop.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="90" customHeight="1">
       <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>A6</t>
+          <t>OPERATING-MINDSET</t>
         </is>
       </c>
       <c r="C10" s="11" t="inlineStr">
@@ -1226,22 +1218,22 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>ML / Data Logging</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Entry-time feature logger in swing_trade.py</t>
+          <t>20-principle hedge-fund-analyst Operating Mindset in CLAUDE.md</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
+          <t>User's standing directive: every decision in this codebase should reflect senior hedge-fund quant analyst discipline, not generic software engineering. Without explicit codification, the principles drift.</t>
         </is>
       </c>
       <c r="G10" s="5" t="inlineStr">
         <is>
-          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
+          <t>New top-level OPERATING MINDSET section in CLAUDE.md before Path Layout. 20 principles in 4 categories (Foundational discipline / Capital preservation / Information edge / Behavioral discipline / Realism) + enforcement table mapping each principle to its code location + push-back examples for when user instruction conflicts.</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
@@ -1251,12 +1243,12 @@
       </c>
       <c r="I10" s="5" t="inlineStr">
         <is>
-          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
+          <t>Win: codified discipline survives session/agent boundaries.</t>
         </is>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
-          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
+          <t>Includes 8 original + 12 added principles. Auto-loaded on every Claude interaction in this dir.</t>
         </is>
       </c>
       <c r="K10" s="12" t="inlineStr">
@@ -1266,27 +1258,27 @@
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>0574c60d4</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N10" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+          <t>head -200 CLAUDE.md → 20 numbered principles in 5 categories, enforcement summary table, push-back guidance. New CLAUDE sessions auto-load this.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="105" customHeight="1">
       <c r="A11" s="2" t="n">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>Q1-step1</t>
+          <t>A6</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -1296,37 +1288,37 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>ML / Data Logging</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>Re-derive Saturday's empirical analysis on n=384 750d backtest</t>
+          <t>Entry-time feature logger in swing_trade.py</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>Saturday's session changed live config based on agent-summarized stats. Agent's Fix 2 was actively wrong; Fix 3 had n=1 evidence in post-kill subset. Confirm Saturday's reads before any further changes.</t>
+          <t>ML mover-predictor v2 result (AUC 0.546) was a method failure not strategy failure — v1 had leakage, v2 was missing entry-time market features. Need to capture them going forward for catalyst-conditional ML.</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>Run inline Python script in SESSION_HANDOFF section 3 against cache/portfolio_backtest_750d_20260509_100501.json. Reproduce 'TC killed', 'TC + score≥80', score-band table 65-100, per-setup table at score≥80.</t>
+          <t>Adds 30 entry-time fields to every signal_log entry, all prefixed `ef_`. Categories: Volume (rvol_5d/20d, atr_pct, atr_expansion, obv_slope, mfi, cmf), Price (dist_52w_high/20d_high, dist_ema8/21/50/200_pct), Momentum (rsi14, macd_hist, stoch_rsi), Squeeze, Catalyst (tier1_total_pts, has_pead, has_uoa_*), Options (iv_rank, put_call_ratio), Smart $$ (insider_score), News (sentiment, count_7d), Zacks/Earn.</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Risk: none. Verify: TC killed PF 0.86, 80-85 band PF 1.72, VCP n=1.</t>
+          <t>Win: ~150-300 trades over 30 days → enough for catalyst-conditional ML retraining.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>Gate for everything below — do not proceed if numbers diverge. · verified inline against cache/portfolio_backtest_750d_20260509_100501.json: TC@score&gt;=80 PF 0.54, VCP@score&gt;=80 n=1, Near-VCP@score&gt;=80 PF 1.05, 90-100 band PF 0.55</t>
+          <t>Pure additive — Wilson CI gates / hedge_fund_report / drift checker unaffected.</t>
         </is>
       </c>
       <c r="K11" s="12" t="inlineStr">
@@ -1341,22 +1333,22 @@
       </c>
       <c r="M11" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>0574c60d4</t>
         </is>
       </c>
       <c r="N11" s="8" t="inlineStr">
         <is>
-          <t>python3 -c 'import json; d=json.load(open("cache/portfolio_backtest_750d_20260509_100501.json")); print(d["profit_factor"])' → 0.70 confirmed.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
+          <t>python3 swing_trade.py → check newly-written entries in data/signal_log.json have ef_volume_surge_5d, ef_atr_pct, ef_rsi14, ef_has_pead, etc. fields populated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="60" customHeight="1">
       <c r="A12" s="2" t="n">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Q1-step2</t>
+          <t>Q1-step1</t>
         </is>
       </c>
       <c r="C12" s="11" t="inlineStr">
@@ -1371,32 +1363,32 @@
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Revert Fix 3 — VCP Breakout multiplier 1.2 → 0.0</t>
+          <t>Re-derive Saturday's empirical analysis on n=384 750d backtest</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t>Saturday boosted VCP Breakout to 1.2× based on n=12 aggregate. Post-kill universe has only n=1 firing at score≥80, and it lost.</t>
+          <t>Saturday's session changed live config based on agent-summarized stats. Agent's Fix 2 was actively wrong; Fix 3 had n=1 evidence in post-kill subset. Confirm Saturday's reads before any further changes.</t>
         </is>
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Edit config/config.json: setup_score_multiplier['VCP Breakout'] 1.2 → 0.0. Verify with git diff config/config.json.</t>
+          <t>Run inline Python script in SESSION_HANDOFF section 3 against cache/portfolio_backtest_750d_20260509_100501.json. Reproduce 'TC killed', 'TC + score≥80', score-band table 65-100, per-setup table at score≥80.</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>2 min</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I12" s="5" t="inlineStr">
         <is>
-          <t>Risk: LOW. Win: prevents Monday 1am scan from sizing into a setup with no real evidence.</t>
+          <t>Risk: none. Verify: TC killed PF 0.86, 80-85 band PF 1.72, VCP n=1.</t>
         </is>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
-          <t>Lesson: filter to 'what new config would have allowed' before extrapolating.</t>
+          <t>Gate for everything below — do not proceed if numbers diverge. · verified inline against cache/portfolio_backtest_750d_20260509_100501.json: TC@score&gt;=80 PF 0.54, VCP@score&gt;=80 n=1, Near-VCP@score&gt;=80 PF 1.05, 90-100 band PF 0.55</t>
         </is>
       </c>
       <c r="K12" s="12" t="inlineStr">
@@ -1416,7 +1408,7 @@
       </c>
       <c r="N12" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 '"VCP Breakout"' config/config.json → setup_score_multiplier shows 0.0 (was 1.2). git diff confirms revert.</t>
+          <t>python3 -c 'import json; d=json.load(open("cache/portfolio_backtest_750d_20260509_100501.json")); print(d["profit_factor"])' → 0.70 confirmed.</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1418,7 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>Q1-step3</t>
+          <t>Q1-step2</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
@@ -1441,17 +1433,17 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>Boost Near-VCP Breakout multiplier 0.7 → 1.0</t>
+          <t>Revert Fix 3 — VCP Breakout multiplier 1.2 → 0.0</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>Post-kill universe at score≥80: Near-VCP Breakout n=50, PF 1.07 — workhorse currently demoted to 0.7×.</t>
+          <t>Saturday boosted VCP Breakout to 1.2× based on n=12 aggregate. Post-kill universe has only n=1 firing at score≥80, and it lost.</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>Edit config/config.json: setup_score_multiplier['Near-VCP Breakout'] 0.7 → 1.0. Verify next backtest.</t>
+          <t>Edit config/config.json: setup_score_multiplier['VCP Breakout'] 1.2 → 0.0. Verify with git diff config/config.json.</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
@@ -1461,12 +1453,12 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Risk: LOW-MEDIUM. Win: lets proven workhorse pull full weight.</t>
+          <t>Risk: LOW. Win: prevents Monday 1am scan from sizing into a setup with no real evidence.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>PF 1.07 has wide CI 0.85-1.30 OOS. Verify with Q1-step4 250d backtest.</t>
+          <t>Lesson: filter to 'what new config would have allowed' before extrapolating.</t>
         </is>
       </c>
       <c r="K13" s="12" t="inlineStr">
@@ -1486,17 +1478,17 @@
       </c>
       <c r="N13" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 '"Near-VCP Breakout"' config/config.json → setup_score_multiplier shows 1.0 (was 0.7).</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+          <t>grep -A5 '"VCP Breakout"' config/config.json → setup_score_multiplier shows 0.0 (was 1.2). git diff confirms revert.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="2" t="n">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>Q1-step4</t>
+          <t>Q1-step3</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
@@ -1511,32 +1503,32 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Run 250-day backtest to validate steps 2 + 3</t>
+          <t>Boost Near-VCP Breakout multiplier 0.7 → 1.0</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>Need fast validation that config changes don't break things before committing 3 hours to full 750d.</t>
+          <t>Post-kill universe at score≥80: Near-VCP Breakout n=50, PF 1.07 — workhorse currently demoted to 0.7×.</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>python3 backtest.py --days 250 --hold 5 --min-score 65 --portfolio --equity 5000 --positions 4 --size-pct 0.25 &gt; cache/logs/backtest_250d_quant1_$(date +%Y%m%d_%H%M%S).log 2&gt;&amp;1 &amp;</t>
+          <t>Edit config/config.json: setup_score_multiplier['Near-VCP Breakout'] 0.7 → 1.0. Verify next backtest.</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>~12 min wall-clock</t>
+          <t>2 min</t>
         </is>
       </c>
       <c r="I14" s="5" t="inlineStr">
         <is>
-          <t>Risk: none (offline). Verify: PF ≥ 1.0 to proceed.</t>
+          <t>Risk: LOW-MEDIUM. Win: lets proven workhorse pull full weight.</t>
         </is>
       </c>
       <c r="J14" s="5" t="inlineStr">
         <is>
-          <t>PASSED smoke 5d (PF 7.74, WR 40%). Confirmed weekly_df fix unblocks BUYs.</t>
+          <t>PF 1.07 has wide CI 0.85-1.30 OOS. Verify with Q1-step4 250d backtest.</t>
         </is>
       </c>
       <c r="K14" s="12" t="inlineStr">
@@ -1546,27 +1538,27 @@
       </c>
       <c r="L14" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr">
         <is>
-          <t>985cd182b</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N14" s="8" t="inlineStr">
         <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="180" customHeight="1">
+          <t>grep -A5 '"Near-VCP Breakout"' config/config.json → setup_score_multiplier shows 1.0 (was 0.7).</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="60" customHeight="1">
       <c r="A15" s="2" t="n">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>Q1-step5</t>
+          <t>Q1-step4</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
@@ -1581,32 +1573,32 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>Run 750-day backtest to confirm if 250d passes</t>
+          <t>Run 250-day backtest to validate steps 2 + 3</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t>Real evidence comes from full 750d window — same methodology that produced Saturday's headline n=384 result.</t>
+          <t>Need fast validation that config changes don't break things before committing 3 hours to full 750d.</t>
         </is>
       </c>
       <c r="G15" s="5" t="inlineStr">
         <is>
-          <t>Same backtest command but --days 750. Run during Sunday daytime (3hr runtime).</t>
+          <t>python3 backtest.py --days 250 --hold 5 --min-score 65 --portfolio --equity 5000 --positions 4 --size-pct 0.25 &gt; cache/logs/backtest_250d_quant1_$(date +%Y%m%d_%H%M%S).log 2&gt;&amp;1 &amp;</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>~3 hours</t>
+          <t>~12 min wall-clock</t>
         </is>
       </c>
       <c r="I15" s="5" t="inlineStr">
         <is>
-          <t>Risk: none. Verify: PF, WR, drawdown all directionally improved vs Saturday's PF 0.70.</t>
+          <t>Risk: none (offline). Verify: PF ≥ 1.0 to proceed.</t>
         </is>
       </c>
       <c r="J15" s="5" t="inlineStr">
         <is>
-          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first. / FAILED ACCEPTANCE BAR (2026-05-10): 250d backtest produced 0 BUYs across 3+ simulated months. Q1 multipliers + threshold combo demoted every qualifying signal. Sibling commit a18282d28 (Q1-step5 250d FINAL) logged the failure; recovery path was Variant F (commit f0a66543e) — regime-conditional TC kill ONLY in bull regime (not all 4 regimes). 250d Variant F backtest pending verification before declaring real fix.</t>
+          <t>PASSED smoke 5d (PF 7.74, WR 40%). Confirmed weekly_df fix unblocks BUYs.</t>
         </is>
       </c>
       <c r="K15" s="12" t="inlineStr">
@@ -1621,22 +1613,22 @@
       </c>
       <c r="M15" s="3" t="inlineStr">
         <is>
-          <t>985cd182b + run cache/portfolio_backtest_*</t>
+          <t>985cd182b</t>
         </is>
       </c>
       <c r="N15" s="8" t="inlineStr">
         <is>
-          <t>cat cache/portfolio_backtest.json → check profit_factor, win_rate, max_drawdown_pct fields. Open cache/backtest_report_latest.html for per-setup attribution.</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="180" customHeight="1">
       <c r="A16" s="2" t="n">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Q1-step6</t>
+          <t>Q1-step5</t>
         </is>
       </c>
       <c r="C16" s="11" t="inlineStr">
@@ -1651,32 +1643,32 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>Consider buy_max_score: 90 in regime4_thresholds blocks</t>
+          <t>Run 750-day backtest to confirm if 250d passes</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>90+ score band is anti-predictive: n=19, PF 0.32 in post-kill subset.</t>
+          <t>Real evidence comes from full 750d window — same methodology that produced Saturday's headline n=384 result.</t>
         </is>
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Add buy_max_score: 90 to each of 4 regime blocks under regime4_thresholds. Re-run final backtest.</t>
+          <t>Same backtest command but --days 750. Run during Sunday daytime (3hr runtime).</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>30 min + backtest</t>
+          <t>~3 hours</t>
         </is>
       </c>
       <c r="I16" s="5" t="inlineStr">
         <is>
-          <t>Risk: MEDIUM (small sample n=19). Win: removes -67% PF drag if real.</t>
+          <t>Risk: none. Verify: PF, WR, drawdown all directionally improved vs Saturday's PF 0.70.</t>
         </is>
       </c>
       <c r="J16" s="5" t="inlineStr">
         <is>
-          <t>Skip if step 5 already shows PF healthy.</t>
+          <t>FAILED acceptance bar over 12 months (n=142): PF 0.95 / WR 31.7% / MaxDD 32.1% / -6.3% return / Sharpe -0.17. avg_win 6.08% vs avg_loss -2.96% (asymmetry 2.05× needs ~2.5× for PF 1.4 at this WR). System produces actionable trades but too many small losers (97/142). DO NOT activate paper trading on this config. Next: try tighter entry quality, wider stops, higher score floor — need user decision on which lever first. / FAILED ACCEPTANCE BAR (2026-05-10): 250d backtest produced 0 BUYs across 3+ simulated months. Q1 multipliers + threshold combo demoted every qualifying signal. Sibling commit a18282d28 (Q1-step5 250d FINAL) logged the failure; recovery path was Variant F (commit f0a66543e) — regime-conditional TC kill ONLY in bull regime (not all 4 regimes). 250d Variant F backtest pending verification before declaring real fix.</t>
         </is>
       </c>
       <c r="K16" s="12" t="inlineStr">
@@ -1691,22 +1683,22 @@
       </c>
       <c r="M16" s="3" t="inlineStr">
         <is>
-          <t>f47958fc9</t>
+          <t>985cd182b + run cache/portfolio_backtest_*</t>
         </is>
       </c>
       <c r="N16" s="8" t="inlineStr">
         <is>
-          <t>(test instructions to be added when shipped)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="90" customHeight="1">
+          <t>cat cache/portfolio_backtest.json → check profit_factor, win_rate, max_drawdown_pct fields. Open cache/backtest_report_latest.html for per-setup attribution.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
       <c r="A17" s="2" t="n">
         <v>16</v>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>B2</t>
+          <t>Q1-step6</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
@@ -1716,37 +1708,37 @@
       </c>
       <c r="D17" s="5" t="inlineStr">
         <is>
-          <t>Quant / Backtest infra</t>
+          <t>QUANT-1 Sunday follow-up</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Enrich backtest trade records with regime/entry_quality/sector/MAE/MFE</t>
+          <t>Consider buy_max_score: 90 in regime4_thresholds blocks</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>750d backtest trade records had only ticker/dates/prices/pnl/setup_type/score/verdict/exit_reason — making per-strategy attribution impossible per A5 finding.</t>
+          <t>90+ score band is anti-predictive: n=19, PF 0.32 in post-kill subset.</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>backtest.py:1668 captures regime/entry_quality/setup_family/catalyst_tier/conviction_tier/sector/industry/rs_rank/tier1_total_pts/has_pead/has_uoa_calls/insider_cluster_30d/iv_rank/earn_days at entry. Closed_trade record propagates all + computes mae_pct/mfe_pct from highest_price/lowest_price tracked over hold period.</t>
+          <t>Add buy_max_score: 90 to each of 4 regime blocks under regime4_thresholds. Re-run final backtest.</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>30 min + backtest</t>
         </is>
       </c>
       <c r="I17" s="5" t="inlineStr">
         <is>
-          <t>Win: forensic decomposition possible on next 750d backtest.</t>
+          <t>Risk: MEDIUM (small sample n=19). Win: removes -67% PF drag if real.</t>
         </is>
       </c>
       <c r="J17" s="5" t="inlineStr">
         <is>
-          <t>Pure additive. Does not affect existing analysis.</t>
+          <t>Skip if step 5 already shows PF healthy.</t>
         </is>
       </c>
       <c r="K17" s="12" t="inlineStr">
@@ -1756,27 +1748,27 @@
       </c>
       <c r="L17" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr">
         <is>
-          <t>f35f0c124</t>
+          <t>f47958fc9</t>
         </is>
       </c>
       <c r="N17" s="8" t="inlineStr">
         <is>
-          <t>Run a fresh backtest (after current finishes). Open cache/portfolio_backtest_*.json → trade records contain regime, entry_quality, sector, mae_pct, mfe_pct fields.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="45" customHeight="1">
+          <t>(test instructions to be added when shipped)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
       <c r="A18" s="2" t="n">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Q1-Fix1</t>
+          <t>B2</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
@@ -1786,22 +1778,22 @@
       </c>
       <c r="D18" s="5" t="inlineStr">
         <is>
-          <t>Quant / Config</t>
+          <t>Quant / Backtest infra</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
         <is>
-          <t>Trend Continuation killed (Fix 1)</t>
+          <t>Enrich backtest trade records with regime/entry_quality/sector/MAE/MFE</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t>750d backtest: Trend Continuation 264/384 trades (69%) at PF 0.65, Wilson LB 19.5% — single biggest portfolio drain.</t>
+          <t>750d backtest trade records had only ticker/dates/prices/pnl/setup_type/score/verdict/exit_reason — making per-strategy attribution impossible per A5 finding.</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>config/config.json: setup_score_multiplier['Trend Continuation'] 0.7→0.0 + static_setup_kill_list dict entry (n=264, wr_lb=0.195, source=static).</t>
+          <t>backtest.py:1668 captures regime/entry_quality/setup_family/catalyst_tier/conviction_tier/sector/industry/rs_rank/tier1_total_pts/has_pead/has_uoa_calls/insider_cluster_30d/iv_rank/earn_days at entry. Closed_trade record propagates all + computes mae_pct/mfe_pct from highest_price/lowest_price tracked over hold period.</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
@@ -1811,12 +1803,12 @@
       </c>
       <c r="I18" s="5" t="inlineStr">
         <is>
-          <t>Win: prevents biggest documented setup drag on Monday 1am scan.</t>
+          <t>Win: forensic decomposition possible on next 750d backtest.</t>
         </is>
       </c>
       <c r="J18" s="5" t="inlineStr">
         <is>
-          <t>Bug fix in 6ceca2d18: bare-string kill_list entries silently rejected — required dict format.</t>
+          <t>Pure additive. Does not affect existing analysis.</t>
         </is>
       </c>
       <c r="K18" s="12" t="inlineStr">
@@ -1831,12 +1823,12 @@
       </c>
       <c r="M18" s="3" t="inlineStr">
         <is>
-          <t>fc76c9ec8 + 6ceca2d18</t>
+          <t>f35f0c124</t>
         </is>
       </c>
       <c r="N18" s="8" t="inlineStr">
         <is>
-          <t>grep -A5 'static_setup_kill_list' config/config.json → 'Trend Continuation' present in dict format with n=264 wr_lb=0.195.</t>
+          <t>Run a fresh backtest (after current finishes). Open cache/portfolio_backtest_*.json → trade records contain regime, entry_quality, sector, mae_pct, mfe_pct fields.</t>
         </is>
       </c>
     </row>
@@ -1846,7 +1838,7 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Q1-Fix3</t>
+          <t>Q1-Fix1</t>
         </is>
       </c>
       <c r="C19" s="11" t="inlineStr">
@@ -1861,32 +1853,32 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>VCP Breakout multiplier 0.0 → 1.2 (Fix 3) — needs revert</t>
+          <t>Trend Continuation killed (Fix 1)</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t>Comment in config said VCP Breakout was 'removed from kill list' but value remained 0.0. Restored to 1.2 based on n=12 PF 1.79 aggregate.</t>
+          <t>750d backtest: Trend Continuation 264/384 trades (69%) at PF 0.65, Wilson LB 19.5% — single biggest portfolio drain.</t>
         </is>
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>config['setup_score_multiplier']['VCP Breakout']: 0.0 → 1.2.</t>
+          <t>config/config.json: setup_score_multiplier['Trend Continuation'] 0.7→0.0 + static_setup_kill_list dict entry (n=264, wr_lb=0.195, source=static).</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>shipped (revert candidate)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I19" s="5" t="inlineStr">
         <is>
-          <t>Risk: post-kill subset has only n=1 evidence — not real evidence. See Q1-step2.</t>
+          <t>Win: prevents biggest documented setup drag on Monday 1am scan.</t>
         </is>
       </c>
       <c r="J19" s="5" t="inlineStr">
         <is>
-          <t>REVERT CANDIDATE. Sunday plan step 2: revert to 0.0.</t>
+          <t>Bug fix in 6ceca2d18: bare-string kill_list entries silently rejected — required dict format.</t>
         </is>
       </c>
       <c r="K19" s="12" t="inlineStr">
@@ -1901,22 +1893,22 @@
       </c>
       <c r="M19" s="3" t="inlineStr">
         <is>
-          <t>fc76c9ec8</t>
+          <t>fc76c9ec8 + 6ceca2d18</t>
         </is>
       </c>
       <c r="N19" s="8" t="inlineStr">
         <is>
-          <t>Same as Q1-step2 verification — VCP Breakout multiplier should NOW be 0.0 (reverted from Saturday's 1.2).</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
+          <t>grep -A5 'static_setup_kill_list' config/config.json → 'Trend Continuation' present in dict format with n=264 wr_lb=0.195.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="2" t="n">
         <v>19</v>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>K3</t>
+          <t>Q1-Fix3</t>
         </is>
       </c>
       <c r="C20" s="11" t="inlineStr">
@@ -1926,37 +1918,37 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>Quant / Stop Engine</t>
+          <t>Quant / Config</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
         <is>
-          <t>Stop must be at/below nearest fractal low</t>
+          <t>VCP Breakout multiplier 0.0 → 1.2 (Fix 3) — needs revert</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t>Calculated stops sometimes sit ABOVE the nearest Williams-fractal low — guaranteed easy stop-out target for market makers.</t>
+          <t>Comment in config said VCP Breakout was 'removed from kill list' but value remained 0.0. Restored to 1.2 based on n=12 PF 1.79 aggregate.</t>
         </is>
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>If stop &gt; indicators['fractal_low'] (already computed in _williams_fractals at analysis.py:1089), widen DOWN to just below fractal low + 0.10×ATR buffer. Bounded: won't widen &gt;20% from entry.</t>
+          <t>config['setup_score_multiplier']['VCP Breakout']: 0.0 → 1.2.</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (revert candidate)</t>
         </is>
       </c>
       <c r="I20" s="5" t="inlineStr">
         <is>
-          <t>Win: single most important Vinod rule per coaching call.</t>
+          <t>Risk: post-kill subset has only n=1 evidence — not real evidence. See Q1-step2.</t>
         </is>
       </c>
       <c r="J20" s="5" t="inlineStr">
         <is>
-          <t>Longs only. Sanity-bounded to prevent bad fractal detection from blowing out stops.</t>
+          <t>REVERT CANDIDATE. Sunday plan step 2: revert to 0.0.</t>
         </is>
       </c>
       <c r="K20" s="12" t="inlineStr">
@@ -1971,22 +1963,22 @@
       </c>
       <c r="M20" s="3" t="inlineStr">
         <is>
-          <t>3d4eb71d7</t>
+          <t>fc76c9ec8</t>
         </is>
       </c>
       <c r="N20" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep AAPL → check that stop value ≤ indicators.fractal_low (or within 0.10×ATR buffer below it). NEVER above fractal_low.</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="90" customHeight="1">
+          <t>Same as Q1-step2 verification — VCP Breakout multiplier should NOW be 0.0 (reverted from Saturday's 1.2).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="105" customHeight="1">
       <c r="A21" s="2" t="n">
         <v>20</v>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>GATE-1</t>
+          <t>VAR-F</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
@@ -1996,37 +1988,29 @@
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>Quant / Validation</t>
+          <t>Quant / Recovery</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Validation backtest restart + 0-BUYs investigation</t>
+          <t>Variant F: regime-conditional Trend Continuation kill in bull regime only</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t>First validation backtest (PID 25081) died at 2024-01-04 with 0 BUYs in 8 months. Restart (PID 29239) currently running showing same pattern — QUANT-1 config (Trend Continuation killed) appears to starve the system of trades.</t>
+          <t>Q1-step5 250d backtest produced 0 BUYs (a18282d28). Root cause: Q1 multipliers + threshold combo demoted every qualifying signal across all regimes. Sibling session designed Variant F: kill TC ONLY in bull regime where it has been bleeding edge, leave TC alive in non-bull regimes where empirical edge holds.</t>
         </is>
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Restarted backtest at 22:48 PT (PID 29239). When done: if PF &gt;= 1.0 → ship QUANT-1b (buy_max_score=80). If 0 BUYs persists → revert TC kill or apply soft demote (mult 0.5) instead of hard kill.</t>
-        </is>
-      </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>in flight</t>
-        </is>
-      </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>Risk: confirmation that TC kill removed all profitable signals along with the bad ones.</t>
-        </is>
-      </c>
+          <t>regime-conditional setup_score_multiplier in config.json. Bull regime: TC = 0 (kill). Other regimes: TC = baseline. Verification backtest pending before declaring real fix.</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+      <c r="I21" s="5" t="inlineStr"/>
       <c r="J21" s="5" t="inlineStr">
         <is>
-          <t>Validation backtest ran ~1.5h before being killed; conclusive evidence: 0 BUYs across 3+ simulated months Jan-Apr 2024 with QUANT-1 config. Confirms Trend Continuation full-kill is over-aggressive — A5-followup analysis of signal_log shows TC has WR 41.4% / avg +2.08% over n=140 closed signals (positive expectancy). Reverting in A5-followup commit.</t>
+          <t>Designed by sibling session as the recovery from Q1-step5 250d 0-BUY failure. Hypothesis: TC has been a net loser in bull regimes (compressed by trend exhaustion) but still has edge in chop/sideways. Killing only in bull preserves the workable edge while removing the bleed. Verification still pending — Q1-step5 cache/portfolio_backtest_*.json baseline + new 250d Variant F run side-by-side.</t>
         </is>
       </c>
       <c r="K21" s="12" t="inlineStr">
@@ -2041,12 +2025,12 @@
       </c>
       <c r="M21" s="3" t="inlineStr">
         <is>
-          <t>logs/backtest_750d_quant1_validate2</t>
+          <t>f0a66543e + 363984181</t>
         </is>
       </c>
       <c r="N21" s="8" t="inlineStr">
         <is>
-          <t>ps -p 29239 → if alive backtest still running. When done: ls cache/portfolio_backtest_750d_*.json | head -1 → check PF, total_return_pct.</t>
+          <t>1. python3 backtest.py --window 250d → expect non-zero BUYs (was 0 with Q1 config). 2. Inspect cache/portfolio_backtest_*.json → trades.regime field shows mostly non-bull regime trades for TC family. 3. Spot-check live scan: if regime4=risk_on_trending, TC tickers should fall through to WATCH; in risk_on_choppy/risk_off, TC should still earn BUY when scoring qualifies. 4. Variant F is verification-pending — log PF/WR vs Q1 baseline, compare to Q1-step5 0-BUY failure mode.</t>
         </is>
       </c>
     </row>
@@ -2056,7 +2040,7 @@
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>A2</t>
+          <t>K3</t>
         </is>
       </c>
       <c r="C22" s="11" t="inlineStr">
@@ -2066,22 +2050,22 @@
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Filter Layer</t>
+          <t>Quant / Stop Engine</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>signal_filter.py — declarative whitelist gate</t>
+          <t>Stop must be at/below nearest fractal low</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t>BUY decisions ran on raw 5-pillar score regardless of whether the (setup × regime × score_band × entry_quality) combo had backtest evidence behind it.</t>
+          <t>Calculated stops sometimes sit ABOVE the nearest Williams-fractal low — guaranteed easy stop-out target for market makers.</t>
         </is>
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>New signal_filter.py — demotes BUY→WATCH for non-whitelisted combos. _validations gate enforces n&gt;=20 AND wr_lb&gt;=0.40 per rule. Wired at decision_engine.py:626 after BUY threshold passes. 5/5 unit tests pass.</t>
+          <t>If stop &gt; indicators['fractal_low'] (already computed in _williams_fractals at analysis.py:1089), widen DOWN to just below fractal low + 0.10×ATR buffer. Bounded: won't widen &gt;20% from entry.</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -2091,12 +2075,12 @@
       </c>
       <c r="I22" s="5" t="inlineStr">
         <is>
-          <t>Win: prevents BUY in unproven combos. OFF by default until A5 attribution complete.</t>
+          <t>Win: single most important Vinod rule per coaching call.</t>
         </is>
       </c>
       <c r="J22" s="5" t="inlineStr">
         <is>
-          <t>Flip config['signal_filter']['_enabled']=true after per-subtype A5 attribution review.</t>
+          <t>Longs only. Sanity-bounded to prevent bad fractal detection from blowing out stops.</t>
         </is>
       </c>
       <c r="K22" s="12" t="inlineStr">
@@ -2111,22 +2095,22 @@
       </c>
       <c r="M22" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>3d4eb71d7</t>
         </is>
       </c>
       <c r="N22" s="8" t="inlineStr">
         <is>
-          <t>1) cat config/config.json | grep -A3 signal_filter → confirm _enabled=false. 2) Toggle to true via --config-override → run scan → BUY count drops. Toggle off → restored.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="60" customHeight="1">
+          <t>python3 swing_trade.py deep AAPL → check that stop value ≤ indicators.fractal_low (or within 0.10×ATR buffer below it). NEVER above fractal_low.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="90" customHeight="1">
       <c r="A23" s="2" t="n">
         <v>22</v>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>A3</t>
+          <t>GATE-1</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
@@ -2136,37 +2120,37 @@
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>Strategy / Filter Layer</t>
+          <t>Quant / Validation</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Regime gate in compute_final_verdict</t>
+          <t>Validation backtest restart + 0-BUYs investigation</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t>750d evidence: strategy is bull-only. risk_off_trending and panic regimes returned negative expectancy.</t>
+          <t>First validation backtest (PID 25081) died at 2024-01-04 with 0 BUYs in 8 months. Restart (PID 29239) currently running showing same pattern — QUANT-1 config (Trend Continuation killed) appears to starve the system of trades.</t>
         </is>
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>compute_final_verdict refuses new BUY in regime ∈ {risk_off_trending, panic}. Returns verdict=WATCH with audit gate 'regime_gate' failed. Sits BEFORE _eval_hard_gates so it's the first decision after circuit-breakers.</t>
+          <t>Restarted backtest at 22:48 PT (PID 29239). When done: if PF &gt;= 1.0 → ship QUANT-1b (buy_max_score=80). If 0 BUYs persists → revert TC kill or apply soft demote (mult 0.5) instead of hard kill.</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>in flight</t>
         </is>
       </c>
       <c r="I23" s="5" t="inlineStr">
         <is>
-          <t>Win: bull-only strategy, period.</t>
+          <t>Risk: confirmation that TC kill removed all profitable signals along with the bad ones.</t>
         </is>
       </c>
       <c r="J23" s="5" t="inlineStr">
         <is>
-          <t>Existing positions unaffected (exits run via separate paths).</t>
+          <t>Validation backtest ran ~1.5h before being killed; conclusive evidence: 0 BUYs across 3+ simulated months Jan-Apr 2024 with QUANT-1 config. Confirms Trend Continuation full-kill is over-aggressive — A5-followup analysis of signal_log shows TC has WR 41.4% / avg +2.08% over n=140 closed signals (positive expectancy). Reverting in A5-followup commit.</t>
         </is>
       </c>
       <c r="K23" s="12" t="inlineStr">
@@ -2176,17 +2160,17 @@
       </c>
       <c r="L23" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>logs/backtest_750d_quant1_validate2</t>
         </is>
       </c>
       <c r="N23" s="8" t="inlineStr">
         <is>
-          <t>Run scan during simulated risk_off regime (set regime via --config-override) → confirm zero BUY verdicts emitted. Audit gate 'regime_gate' marked failed.</t>
+          <t>ps -p 29239 → if alive backtest still running. When done: ls cache/portfolio_backtest_750d_*.json | head -1 → check PF, total_return_pct.</t>
         </is>
       </c>
     </row>
@@ -2196,47 +2180,47 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>B1</t>
-        </is>
-      </c>
-      <c r="C24" s="4" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Backtest / Diagnosis</t>
+          <t>Strategy / Filter Layer</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
         <is>
-          <t>Diagnose --as-of-membership n_trades=0 bug</t>
+          <t>signal_filter.py — declarative whitelist gate</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t>Walk-forward runs with --as-of-membership universe (~1000 tickers) returned n_trades=0 even though universe loader works correctly.</t>
+          <t>BUY decisions ran on raw 5-pillar score regardless of whether the (setup × regime × score_band × entry_quality) combo had backtest evidence behind it.</t>
         </is>
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>diagnose_as_of_membership.py — script captures findings. Root cause documented in SESSION_HANDOFF section 9. Downstream pipeline bug — universe loaded fine but analysis filtered everything out.</t>
+          <t>New signal_filter.py — demotes BUY→WATCH for non-whitelisted combos. _validations gate enforces n&gt;=20 AND wr_lb&gt;=0.40 per rule. Wired at decision_engine.py:626 after BUY threshold passes. 5/5 unit tests pass.</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>shipped (diagnosis); pending (fix)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I24" s="5" t="inlineStr">
         <is>
-          <t>Win: known root cause; fix will unblock historical backtesting at scale.</t>
+          <t>Win: prevents BUY in unproven combos. OFF by default until A5 attribution complete.</t>
         </is>
       </c>
       <c r="J24" s="5" t="inlineStr">
         <is>
-          <t>Fix deferred until standalone 750d backtest finishes.</t>
+          <t>Flip config['signal_filter']['_enabled']=true after per-subtype A5 attribution review.</t>
         </is>
       </c>
       <c r="K24" s="12" t="inlineStr">
@@ -2251,62 +2235,62 @@
       </c>
       <c r="M24" s="3" t="inlineStr">
         <is>
-          <t>9bc015562</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N24" s="8" t="inlineStr">
         <is>
-          <t>cat diagnose_as_of_membership.py output OR re-run: python3 diagnose_as_of_membership.py → '88.3% OHLCV coverage' confirmed; bug elsewhere in pipeline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="45" customHeight="1">
+          <t>1) cat config/config.json | grep -A3 signal_filter → confirm _enabled=false. 2) Toggle to true via --config-override → run scan → BUY count drops. Toggle off → restored.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="60" customHeight="1">
       <c r="A25" s="2" t="n">
         <v>24</v>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-1</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr">
-        <is>
-          <t>P1</t>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="C25" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Backtest performance</t>
+          <t>Strategy / Filter Layer</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>backtest.py --smoke (5d quick-validate mode)</t>
+          <t>Regime gate in compute_final_verdict</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t>Validating config changes required full 60d run (~12 min). Bad iteration loop.</t>
+          <t>750d evidence: strategy is bull-only. risk_off_trending and panic regimes returned negative expectancy.</t>
         </is>
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Added --smoke flag: 5d window, top-100 universe by avg dollar vol, auto-portfolio. Runs in &lt;60s. Use to catch config bugs BEFORE long runs.</t>
+          <t>compute_final_verdict refuses new BUY in regime ∈ {risk_off_trending, panic}. Returns verdict=WATCH with audit gate 'regime_gate' failed. Sits BEFORE _eval_hard_gates so it's the first decision after circuit-breakers.</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>20 min</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I25" s="5" t="inlineStr">
         <is>
-          <t>Low risk / High win</t>
+          <t>Win: bull-only strategy, period.</t>
         </is>
       </c>
       <c r="J25" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10.</t>
+          <t>Existing positions unaffected (exits run via separate paths).</t>
         </is>
       </c>
       <c r="K25" s="12" t="inlineStr">
@@ -2316,27 +2300,27 @@
       </c>
       <c r="L25" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N25" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest.py --smoke → completes &lt;60s, prints summary, no errors. Tweak setup_score_multiplier in config.json, re-run, observe BUY count change.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="45" customHeight="1">
+          <t>Run scan during simulated risk_off regime (set regime via --config-override) → confirm zero BUY verdicts emitted. Audit gate 'regime_gate' marked failed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="60" customHeight="1">
       <c r="A26" s="2" t="n">
         <v>25</v>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-2</t>
+          <t>B1</t>
         </is>
       </c>
       <c r="C26" s="4" t="inlineStr">
@@ -2346,37 +2330,37 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>Backtest performance</t>
+          <t>Backtest / Diagnosis</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
         <is>
-          <t>yfinance info disk cache (24h TTL)</t>
+          <t>Diagnose --as-of-membership n_trades=0 bug</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t>Re-running backtest re-fetched 711 ticker info dicts from yfinance every time. ~30-60s wasted per run.</t>
+          <t>Walk-forward runs with --as-of-membership universe (~1000 tickers) returned n_trades=0 even though universe loader works correctly.</t>
         </is>
       </c>
       <c r="G26" s="5" t="inlineStr">
         <is>
-          <t>_load_or_fetch_infos_cached() wraps get_stock_info_batch with disk cache keyed by sorted-universe SHA1 hash. 24h TTL. Switching universes auto-invalidates.</t>
+          <t>diagnose_as_of_membership.py — script captures findings. Root cause documented in SESSION_HANDOFF section 9. Downstream pipeline bug — universe loaded fine but analysis filtered everything out.</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>30 min</t>
+          <t>shipped (diagnosis); pending (fix)</t>
         </is>
       </c>
       <c r="I26" s="5" t="inlineStr">
         <is>
-          <t>Low risk / High win</t>
+          <t>Win: known root cause; fix will unblock historical backtesting at scale.</t>
         </is>
       </c>
       <c r="J26" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10. Cache files: cache/infos_&lt;sha&gt;.json</t>
+          <t>Fix deferred until standalone 750d backtest finishes.</t>
         </is>
       </c>
       <c r="K26" s="12" t="inlineStr">
@@ -2386,17 +2370,17 @@
       </c>
       <c r="L26" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr">
         <is>
-          <t>pending</t>
+          <t>9bc015562</t>
         </is>
       </c>
       <c r="N26" s="8" t="inlineStr">
         <is>
-          <t>Run backtest twice in a row; second run logs "Cached yfinance info hit" and skips fetch.</t>
+          <t>cat diagnose_as_of_membership.py output OR re-run: python3 diagnose_as_of_membership.py → '88.3% OHLCV coverage' confirmed; bug elsewhere in pipeline.</t>
         </is>
       </c>
     </row>
@@ -2406,7 +2390,7 @@
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-3</t>
+          <t>PERF-OPT-1</t>
         </is>
       </c>
       <c r="C27" s="4" t="inlineStr">
@@ -2421,17 +2405,17 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>backtest.py --profile-cprof (cProfile hotspot audit)</t>
+          <t>backtest.py --smoke (5d quick-validate mode)</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t>No data on actual backtest hot paths — all optimization was guesswork.</t>
+          <t>Validating config changes required full 60d run (~12 min). Bad iteration loop.</t>
         </is>
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Added --profile-cprof flag. Wraps main() in cProfile.Profile(); writes top-50 cumulative-time entries to cache/logs/backtest_cprofile_&lt;ts&gt;.txt.</t>
+          <t>Added --smoke flag: 5d window, top-100 universe by avg dollar vol, auto-portfolio. Runs in &lt;60s. Use to catch config bugs BEFORE long runs.</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
@@ -2441,7 +2425,7 @@
       </c>
       <c r="I27" s="5" t="inlineStr">
         <is>
-          <t>Low risk / High win (evidence-based opt)</t>
+          <t>Low risk / High win</t>
         </is>
       </c>
       <c r="J27" s="5" t="inlineStr">
@@ -2466,17 +2450,17 @@
       </c>
       <c r="N27" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest.py --smoke --profile-cprof → check cache/logs/backtest_cprofile_*.txt; should list top 50 functions.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1">
+          <t>python3 backtest.py --smoke → completes &lt;60s, prints summary, no errors. Tweak setup_score_multiplier in config.json, re-run, observe BUY count change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
       <c r="A28" s="2" t="n">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>PERF-OPT-4</t>
+          <t>PERF-OPT-2</t>
         </is>
       </c>
       <c r="C28" s="4" t="inlineStr">
@@ -2491,32 +2475,32 @@
       </c>
       <c r="E28" s="6" t="inlineStr">
         <is>
-          <t>walk_forward_v2 fold parallelization (--parallel)</t>
+          <t>yfinance info disk cache (24h TTL)</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>4-fold walk-forward ran sequentially: ~8-12h wall-clock. Bottleneck was wall-clock waiting, not CPU.</t>
+          <t>Re-running backtest re-fetched 711 ticker info dicts from yfinance every time. ~30-60s wasted per run.</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Added --parallel + --workers flags. multiprocessing.Pool with spawn-mode (macOS-safe). Each fold runs as separate process. Cuts 4-fold WF from 8-12h to 2-3h.</t>
+          <t>_load_or_fetch_infos_cached() wraps get_stock_info_batch with disk cache keyed by sorted-universe SHA1 hash. 24h TTL. Switching universes auto-invalidates.</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>1 hr</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="I28" s="5" t="inlineStr">
         <is>
-          <t>Low risk / Massive time savings</t>
+          <t>Low risk / High win</t>
         </is>
       </c>
       <c r="J28" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10. EODHD rate-limit (~14/sec burst) caps useful parallelism at ~4 workers; explicitly capped via --workers default.</t>
+          <t>Shipped 2026-05-10. Cache files: cache/infos_&lt;sha&gt;.json</t>
         </is>
       </c>
       <c r="K28" s="12" t="inlineStr">
@@ -2536,17 +2520,17 @@
       </c>
       <c r="N28" s="8" t="inlineStr">
         <is>
-          <t>python3 backtest/walk_forward_v2.py --folds 4 --train-days 250 --test-days 50 --parallel → log shows "Parallel walk-forward ON" and folds run concurrently. Compare wall-clock vs sequential.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
+          <t>Run backtest twice in a row; second run logs "Cached yfinance info hit" and skips fetch.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="2" t="n">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-1</t>
+          <t>PERF-OPT-3</t>
         </is>
       </c>
       <c r="C29" s="4" t="inlineStr">
@@ -2556,37 +2540,37 @@
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Backtest performance</t>
         </is>
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>backtest_v2.py — keep or delete?</t>
+          <t>backtest.py --profile-cprof (cProfile hotspot audit)</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t>158-line file. docs/architecture.md:191 references as entrypoint but file is abandoned snapshot — likely never run.</t>
+          <t>No data on actual backtest hot paths — all optimization was guesswork.</t>
         </is>
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>ASK USER: 'Do you ever run backtest_v2.py?' If no → delete + update docs/architecture.md.</t>
+          <t>Added --profile-cprof flag. Wraps main() in cProfile.Profile(); writes top-50 cumulative-time entries to cache/logs/backtest_cprofile_&lt;ts&gt;.txt.</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>10 min after answer</t>
+          <t>20 min</t>
         </is>
       </c>
       <c r="I29" s="5" t="inlineStr">
         <is>
-          <t>Win: -158 lines + clearer docs.</t>
+          <t>Low risk / High win (evidence-based opt)</t>
         </is>
       </c>
       <c r="J29" s="5" t="inlineStr">
         <is>
-          <t>Phase 2 agent flagged but held back without user judgment. · DELETED — was 158-line abandoned snapshot, has_main=0 (not even runnable). Updated docs/architecture.md + morning_briefing.py to remove references.</t>
+          <t>Shipped 2026-05-10.</t>
         </is>
       </c>
       <c r="K29" s="12" t="inlineStr">
@@ -2601,22 +2585,22 @@
       </c>
       <c r="M29" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N29" s="8" t="inlineStr">
         <is>
-          <t>ls backtest_v2.py → no such file (deleted). docs/architecture.md no longer references it. morning_briefing.py uses cache/logs/backtest_*.log glob.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="90" customHeight="1">
+          <t>python3 backtest.py --smoke --profile-cprof → check cache/logs/backtest_cprofile_*.txt; should list top 50 functions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="2" t="n">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-3</t>
+          <t>PERF-OPT-4</t>
         </is>
       </c>
       <c r="C30" s="4" t="inlineStr">
@@ -2626,37 +2610,37 @@
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Backtest performance</t>
         </is>
       </c>
       <c r="E30" s="6" t="inlineStr">
         <is>
-          <t>8 standalone analysis scripts — ask user which still in use</t>
+          <t>walk_forward_v2 fold parallelization (--parallel)</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t>Manual research scripts: audit_360.py (1320 lines!), analyze_backtest.py, analyze_signals.py, false_negatives.py, feature_importance.py, score_distribution_check.py, sensitivity.py, stop_width_sensitivity.py.</t>
+          <t>4-fold walk-forward ran sequentially: ~8-12h wall-clock. Bottleneck was wall-clock waiting, not CPU.</t>
         </is>
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>ASK USER per file: 'Do you ever run X?' For each 'no' → archive to _legacy/ or delete. ~3-5K lines win.</t>
+          <t>Added --parallel + --workers flags. multiprocessing.Pool with spawn-mode (macOS-safe). Each fold runs as separate process. Cuts 4-fold WF from 8-12h to 2-3h.</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>30 min after answers</t>
+          <t>1 hr</t>
         </is>
       </c>
       <c r="I30" s="5" t="inlineStr">
         <is>
-          <t>Win: ~3-5K lines if mostly stale.</t>
+          <t>Low risk / Massive time savings</t>
         </is>
       </c>
       <c r="J30" s="5" t="inlineStr">
         <is>
-          <t>audit_360.py is the biggest single file — start there. · Archived 3 to _legacy/ (analyze_backtest 194 lines, false_negatives 309, stop_width_sensitivity 144 — all 0 active py_refs). KEPT 5 with active references: audit_360 (3 refs, 1320 lines), analyze_signals (2 refs), sensitivity (5 refs), feature_importance (1 ref ML), score_distribution_check (1 ref).</t>
+          <t>Shipped 2026-05-10. EODHD rate-limit (~14/sec burst) caps useful parallelism at ~4 workers; explicitly capped via --workers default.</t>
         </is>
       </c>
       <c r="K30" s="12" t="inlineStr">
@@ -2671,22 +2655,22 @@
       </c>
       <c r="M30" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>pending</t>
         </is>
       </c>
       <c r="N30" s="8" t="inlineStr">
         <is>
-          <t>ls _legacy/{analyze_backtest,false_negatives,stop_width_sensitivity}.py → 3 files moved. Verify audit_360.py / analyze_signals.py / sensitivity.py / feature_importance.py / score_distribution_check.py still in root (kept).</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+          <t>python3 backtest/walk_forward_v2.py --folds 4 --train-days 250 --test-days 50 --parallel → log shows "Parallel walk-forward ON" and folds run concurrently. Compare wall-clock vs sequential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1">
       <c r="A31" s="2" t="n">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>G3</t>
+          <t>CLEAN-1</t>
         </is>
       </c>
       <c r="C31" s="4" t="inlineStr">
@@ -2696,37 +2680,37 @@
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>signal_filter audit table + drift view</t>
+          <t>backtest_v2.py — keep or delete?</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t>Need persistence + drift monitoring for signal_filter decisions before flipping it on.</t>
+          <t>158-line file. docs/architecture.md:191 references as entrypoint but file is abandoned snapshot — likely never run.</t>
         </is>
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>migrations/003_signal_filter_audit.sql — signal_filter_decisions table + signal_filter_drift_30d view. Feeds A7 dashboard tile (future).</t>
+          <t>ASK USER: 'Do you ever run backtest_v2.py?' If no → delete + update docs/architecture.md.</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>10 min after answer</t>
         </is>
       </c>
       <c r="I31" s="5" t="inlineStr">
         <is>
-          <t>Win: audit + drift visibility before flipping signal_filter on.</t>
+          <t>Win: -158 lines + clearer docs.</t>
         </is>
       </c>
       <c r="J31" s="5" t="inlineStr">
         <is>
-          <t>A7 dashboard tile not yet built — registry has the data when needed.</t>
+          <t>Phase 2 agent flagged but held back without user judgment. · DELETED — was 158-line abandoned snapshot, has_main=0 (not even runnable). Updated docs/architecture.md + morning_briefing.py to remove references.</t>
         </is>
       </c>
       <c r="K31" s="12" t="inlineStr">
@@ -2736,27 +2720,27 @@
       </c>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N31" s="8" t="inlineStr">
         <is>
-          <t>psql or Supabase Studio → confirm signal_filter_decisions table exists + signal_filter_drift_30d view returns query plan.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="60" customHeight="1">
+          <t>ls backtest_v2.py → no such file (deleted). docs/architecture.md no longer references it. morning_briefing.py uses cache/logs/backtest_*.log glob.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="90" customHeight="1">
       <c r="A32" s="2" t="n">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>F11</t>
+          <t>CLEAN-3</t>
         </is>
       </c>
       <c r="C32" s="4" t="inlineStr">
@@ -2766,37 +2750,37 @@
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure / Quality</t>
+          <t>Code Cleanup (DEFERRED)</t>
         </is>
       </c>
       <c r="E32" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook for schema drift</t>
+          <t>8 standalone analysis scripts — ask user which still in use</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t>Schema drift between JSON canonical files and Postgres columns silently fails dual-write to Supabase. Need CI-style enforcement.</t>
+          <t>Manual research scripts: audit_360.py (1320 lines!), analyze_backtest.py, analyze_signals.py, false_negatives.py, feature_importance.py, score_distribution_check.py, sensitivity.py, stop_width_sensitivity.py.</t>
         </is>
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>First version: full-repo --strict check (commit 4129e5565). REFINED in 1e40d30fc: scoped to current commit — skips unless commit touches data/*.json OR migrations/ OR db.py; only blocks on NEW keys this commit adds.</t>
+          <t>ASK USER per file: 'Do you ever run X?' For each 'no' → archive to _legacy/ or delete. ~3-5K lines win.</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>30 min after answers</t>
         </is>
       </c>
       <c r="I32" s="5" t="inlineStr">
         <is>
-          <t>Win: prevents NEW drift while not blocking on pre-existing technical debt.</t>
+          <t>Win: ~3-5K lines if mostly stale.</t>
         </is>
       </c>
       <c r="J32" s="5" t="inlineStr">
         <is>
-          <t>8 pre-existing JSON-only fields documented as tech debt.</t>
+          <t>audit_360.py is the biggest single file — start there. · Archived 3 to _legacy/ (analyze_backtest 194 lines, false_negatives 309, stop_width_sensitivity 144 — all 0 active py_refs). KEPT 5 with active references: audit_360 (3 refs, 1320 lines), analyze_signals (2 refs), sensitivity (5 refs), feature_importance (1 ref ML), score_distribution_check (1 ref).</t>
         </is>
       </c>
       <c r="K32" s="12" t="inlineStr">
@@ -2806,27 +2790,27 @@
       </c>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N32" s="8" t="inlineStr">
         <is>
-          <t>Stage a JSON change with NEW key. git commit → hook fires drift check on NEW key only (not full repo). Pre-existing drift not blocking.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="90" customHeight="1">
+          <t>ls _legacy/{analyze_backtest,false_negatives,stop_width_sensitivity}.py → 3 files moved. Verify audit_360.py / analyze_signals.py / sensitivity.py / feature_importance.py / score_distribution_check.py still in root (kept).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="45" customHeight="1">
       <c r="A33" s="2" t="n">
         <v>32</v>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>MOB-1</t>
+          <t>G3</t>
         </is>
       </c>
       <c r="C33" s="4" t="inlineStr">
@@ -2836,33 +2820,37 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Tablet portrait support (≥768px)</t>
+          <t>signal_filter audit table + drift view</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t>Desktop-first. Viewport meta added but no tablet layouts; sidebar overflows, tabs don't wrap.</t>
+          <t>Need persistence + drift monitoring for signal_filter decisions before flipping it on.</t>
         </is>
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Pure-CSS @media block in dashboard.html + elite-detail.html. Tablet (768-1023): 2-up KPI grid, scrollable tabs, table overflow-x. Phone (≤767): single column, ≥44px tap targets, hidden badges, condensed regime strip, full-width drawers. Touch hover suppression.</t>
+          <t>migrations/003_signal_filter_audit.sql — signal_filter_decisions table + signal_filter_drift_30d view. Feeds A7 dashboard tile (future).</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>4-6 hrs</t>
-        </is>
-      </c>
-      <c r="I33" s="5" t="inlineStr"/>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Win: audit + drift visibility before flipping signal_filter on.</t>
+        </is>
+      </c>
       <c r="J33" s="5" t="inlineStr">
         <is>
-          <t>Tablet/phone CSS shipped to dashboard.html (other session commit 114646f23 PERF-7) and elite-detail.html (this session 54c6f218d). @media breakpoints at 768/1024/380px, 2-up grids on tablet, single-column on phone, ≥44px tap targets, hover suppression on touch.</t>
+          <t>A7 dashboard tile not yet built — registry has the data when needed.</t>
         </is>
       </c>
       <c r="K33" s="12" t="inlineStr">
@@ -2872,27 +2860,27 @@
       </c>
       <c r="L33" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr">
         <is>
-          <t>54c6f218d / 114646f23</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N33" s="8" t="inlineStr">
         <is>
-          <t>Open https://trade.mystockholding.com on iPad portrait (≥768px and &lt;1024px): KPI tiles render 2-up, no horizontal page scroll except inside tables, sub-tabs scroll horizontally without wrapping. Then iPhone Safari (≤767): single-column layout, sidebar tap targets ≥44px, no badge cruft, drawer panels open full-width. Verify desktop (≥1024px) still pixel-identical to before.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="75" customHeight="1">
+          <t>psql or Supabase Studio → confirm signal_filter_decisions table exists + signal_filter_drift_30d view returns query plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="60" customHeight="1">
       <c r="A34" s="2" t="n">
         <v>33</v>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>MOB-2</t>
+          <t>F11</t>
         </is>
       </c>
       <c r="C34" s="4" t="inlineStr">
@@ -2902,33 +2890,37 @@
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>Mobile</t>
+          <t>Infrastructure / Quality</t>
         </is>
       </c>
       <c r="E34" s="6" t="inlineStr">
         <is>
-          <t>Phone support (≤480px)</t>
+          <t>Pre-commit hook for schema drift</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t>No phone layout. Many UI elements unusable on phone.</t>
+          <t>Schema drift between JSON canonical files and Postgres columns silently fails dual-write to Supabase. Need CI-style enforcement.</t>
         </is>
       </c>
       <c r="G34" s="5" t="inlineStr">
         <is>
-          <t>Same media block as MOB-1 plus ≤480px micro-phone block (small phones) + (hover:none) suppress hover effects on touch devices.</t>
+          <t>First version: full-repo --strict check (commit 4129e5565). REFINED in 1e40d30fc: scoped to current commit — skips unless commit touches data/*.json OR migrations/ OR db.py; only blocks on NEW keys this commit adds.</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>8-12 hrs</t>
-        </is>
-      </c>
-      <c r="I34" s="5" t="inlineStr"/>
+          <t>shipped</t>
+        </is>
+      </c>
+      <c r="I34" s="5" t="inlineStr">
+        <is>
+          <t>Win: prevents NEW drift while not blocking on pre-existing technical debt.</t>
+        </is>
+      </c>
       <c r="J34" s="5" t="inlineStr">
         <is>
-          <t>Phone-specific block (≤767px) + small phone (≤380px) + (hover:none) shipped in same commit pair as MOB-1.</t>
+          <t>8 pre-existing JSON-only fields documented as tech debt.</t>
         </is>
       </c>
       <c r="K34" s="12" t="inlineStr">
@@ -2938,27 +2930,27 @@
       </c>
       <c r="L34" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr">
         <is>
-          <t>54c6f218d / 114646f23</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N34" s="8" t="inlineStr">
         <is>
-          <t>Open dashboard on iPhone SE (375px) and iPhone 13 (390px) in Safari. Verify: (1) every interactive element ≥44×44px (use Safari Inspector Touch Region), (2) no horizontal page scroll, (3) tables scroll horizontally inside their card, (4) tap navigation between V1 dashboard and elite detail does not require pinch-zoom.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="45" customHeight="1">
+          <t>Stage a JSON change with NEW key. git commit → hook fires drift check on NEW key only (not full repo). Pre-existing drift not blocking.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="90" customHeight="1">
       <c r="A35" s="2" t="n">
         <v>34</v>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>PERF-4</t>
+          <t>MOB-1</t>
         </is>
       </c>
       <c r="C35" s="4" t="inlineStr">
@@ -2968,37 +2960,33 @@
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Brotli compression (currently Gzip)</t>
+          <t>Tablet portrait support (≥768px)</t>
         </is>
       </c>
       <c r="F35" s="5" t="inlineStr">
         <is>
-          <t>Server.py serves Gzip; Brotli typically reduces JSON/HTML transfer ~15% at similar CPU cost.</t>
+          <t>Desktop-first. Viewport meta added but no tablet layouts; sidebar overflows, tabs don't wrap.</t>
         </is>
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Add brotli middleware to FastAPI; negotiate via Accept-Encoding; verify Cloudflare passes encoding through.</t>
+          <t>Pure-CSS @media block in dashboard.html + elite-detail.html. Tablet (768-1023): 2-up KPI grid, scrollable tabs, table overflow-x. Phone (≤767): single column, ≥44px tap targets, hidden badges, condensed regime strip, full-width drawers. Touch hover suppression.</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>30 min</t>
-        </is>
-      </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>Win: -15% transfer size on data.json + tickers.json + HTML.</t>
-        </is>
-      </c>
+          <t>4-6 hrs</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr"/>
       <c r="J35" s="5" t="inlineStr">
         <is>
-          <t>Verify Cloudflare tunnel doesn't strip br encoding.</t>
+          <t>Tablet/phone CSS shipped to dashboard.html (other session commit 114646f23 PERF-7) and elite-detail.html (this session 54c6f218d). @media breakpoints at 768/1024/380px, 2-up grids on tablet, single-column on phone, ≥44px tap targets, hover suppression on touch.</t>
         </is>
       </c>
       <c r="K35" s="12" t="inlineStr">
@@ -3008,27 +2996,27 @@
       </c>
       <c r="L35" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr">
         <is>
-          <t>2eb4e3b3d</t>
+          <t>54c6f218d / 114646f23</t>
         </is>
       </c>
       <c r="N35" s="8" t="inlineStr">
         <is>
-          <t>Browser DevTools → Network tab → reload dashboard → Content-Encoding header on data.json reads 'br' (Brotli) when supported, else 'gzip'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="45" customHeight="1">
+          <t>Open https://trade.mystockholding.com on iPad portrait (≥768px and &lt;1024px): KPI tiles render 2-up, no horizontal page scroll except inside tables, sub-tabs scroll horizontally without wrapping. Then iPhone Safari (≤767): single-column layout, sidebar tap targets ≥44px, no badge cruft, drawer panels open full-width. Verify desktop (≥1024px) still pixel-identical to before.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="75" customHeight="1">
       <c r="A36" s="2" t="n">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>PERF-5</t>
+          <t>MOB-2</t>
         </is>
       </c>
       <c r="C36" s="4" t="inlineStr">
@@ -3038,37 +3026,33 @@
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Mobile</t>
         </is>
       </c>
       <c r="E36" s="6" t="inlineStr">
         <is>
-          <t>requestIdleCallback for _capScanAndDisableButtons</t>
+          <t>Phone support (≤480px)</t>
         </is>
       </c>
       <c r="F36" s="5" t="inlineStr">
         <is>
-          <t>MutationObserver-based button disabler runs synchronously on init, blocking ~50ms.</t>
+          <t>No phone layout. Many UI elements unusable on phone.</t>
         </is>
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Wrap call in requestIdleCallback(() =&gt; _capScanAndDisableButtons(), { timeout: 500 }). setTimeout fallback for Safari.</t>
+          <t>Same media block as MOB-1 plus ≤480px micro-phone block (small phones) + (hover:none) suppress hover effects on touch devices.</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>15 min</t>
-        </is>
-      </c>
-      <c r="I36" s="5" t="inlineStr">
-        <is>
-          <t>Win: -50ms FCP.</t>
-        </is>
-      </c>
+          <t>8-12 hrs</t>
+        </is>
+      </c>
+      <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr">
         <is>
-          <t>Trivial fix; verify no race with first user interaction.</t>
+          <t>Phone-specific block (≤767px) + small phone (≤380px) + (hover:none) shipped in same commit pair as MOB-1.</t>
         </is>
       </c>
       <c r="K36" s="12" t="inlineStr">
@@ -3078,27 +3062,27 @@
       </c>
       <c r="L36" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>54c6f218d / 114646f23</t>
         </is>
       </c>
       <c r="N36" s="8" t="inlineStr">
         <is>
-          <t>Browser DevTools → Performance → reload dashboard → _capScanAndDisableButtons fires AFTER init-end (in idle callback), not during sync init.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="120" customHeight="1">
+          <t>Open dashboard on iPhone SE (375px) and iPhone 13 (390px) in Safari. Verify: (1) every interactive element ≥44×44px (use Safari Inspector Touch Region), (2) no horizontal page scroll, (3) tables scroll horizontally inside their card, (4) tap navigation between V1 dashboard and elite detail does not require pinch-zoom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="45" customHeight="1">
       <c r="A37" s="2" t="n">
         <v>36</v>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>PERF-6</t>
+          <t>PERF-4</t>
         </is>
       </c>
       <c r="C37" s="4" t="inlineStr">
@@ -3113,32 +3097,32 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Critical CSS extraction (775-line &lt;style&gt; → above-fold + lazy)</t>
+          <t>Brotli compression (currently Gzip)</t>
         </is>
       </c>
       <c r="F37" s="5" t="inlineStr">
         <is>
-          <t>775-line &lt;style&gt; in &lt;head&gt; blocks FCP; most rules govern below-fold content.</t>
+          <t>Server.py serves Gzip; Brotli typically reduces JSON/HTML transfer ~15% at similar CPU cost.</t>
         </is>
       </c>
       <c r="G37" s="5" t="inlineStr">
         <is>
-          <t>Identify above-fold CSS rules (header, sidebar, regime strip, top of each tab). Inline only those. Lazy-load rest via &lt;link rel='stylesheet'&gt; after init-end.</t>
+          <t>Add brotli middleware to FastAPI; negotiate via Accept-Encoding; verify Cloudflare passes encoding through.</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>1 hr</t>
+          <t>30 min</t>
         </is>
       </c>
       <c r="I37" s="5" t="inlineStr">
         <is>
-          <t>Win: -100ms FCP.</t>
+          <t>Win: -15% transfer size on data.json + tickers.json + HTML.</t>
         </is>
       </c>
       <c r="J37" s="5" t="inlineStr">
         <is>
-          <t>Conservative slice shipped: extracted ~295 lines of below-fold CSS (Audit date picker, D-1 Cross-Mode card, D-4 Factor heatmap, Accuracy framework, Settings rebuild, mobile media queries) into dashboard.deferred.css, loaded non-blocking via media="print" onload="this.media='all'". Inline &lt;style&gt; reduced 1029 → 734 lines. Elite Picks v2 styles intentionally kept inline (Elite is the default tab for all profiles).</t>
+          <t>Verify Cloudflare tunnel doesn't strip br encoding.</t>
         </is>
       </c>
       <c r="K37" s="12" t="inlineStr">
@@ -3148,27 +3132,27 @@
       </c>
       <c r="L37" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr">
         <is>
-          <t>450572d28</t>
+          <t>2eb4e3b3d</t>
         </is>
       </c>
       <c r="N37" s="8" t="inlineStr">
         <is>
-          <t>1. Open https://trade.mystockholding.com/v2/dashboard.html in DevTools Network tab. 2. Hard-refresh — confirm dashboard.deferred.css loads as a separate request with media=print first then promoted to media=all. 3. Click Audit / Portfolio / Accuracy / Settings tabs — all styled correctly (no FOUC). 4. Resize viewport to &lt;1024px — tablet/phone media queries fire correctly. 5. View source — inline &lt;style&gt; ends around line 749 (vs 1044 before). 6. Lighthouse FCP should improve ~50-150ms vs PERF-7-only baseline.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="135" customHeight="1">
+          <t>Browser DevTools → Network tab → reload dashboard → Content-Encoding header on data.json reads 'br' (Brotli) when supported, else 'gzip'.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="45" customHeight="1">
       <c r="A38" s="2" t="n">
         <v>37</v>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>PERF-7</t>
+          <t>PERF-5</t>
         </is>
       </c>
       <c r="C38" s="4" t="inlineStr">
@@ -3183,32 +3167,32 @@
       </c>
       <c r="E38" s="6" t="inlineStr">
         <is>
-          <t>Split data.json (5.3MB) into critical + deferred</t>
+          <t>requestIdleCallback for _capScanAndDisableButtons</t>
         </is>
       </c>
       <c r="F38" s="5" t="inlineStr">
         <is>
-          <t>Dashboard cold load now bound by 5.3MB data.json fetch + parse — bulk of remaining 644ms init-end.</t>
+          <t>MutationObserver-based button disabler runs synchronously on init, blocking ~50ms.</t>
         </is>
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Decompose data.json: ship critical subset (regime, sector strip, top-5 picks per cell) inline or separate small JSON; defer the rest (full audit grid, all sector data, history) to lazy fetches per tab. Update build_data.py + dashboard.html.</t>
+          <t>Wrap call in requestIdleCallback(() =&gt; _capScanAndDisableButtons(), { timeout: 500 }). setTimeout fallback for Safari.</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>4 hrs</t>
+          <t>15 min</t>
         </is>
       </c>
       <c r="I38" s="5" t="inlineStr">
         <is>
-          <t>Win: -300-800ms cold load (single largest remaining boot lever).</t>
+          <t>Win: -50ms FCP.</t>
         </is>
       </c>
       <c r="J38" s="5" t="inlineStr">
         <is>
-          <t>Biggest lever for next perf sprint. Phase 1+2 shipped: defers performance/killed/earnings/screener/crypto. Phase 2b (medium_term/long_term lazy on Range filter) tracked as PERF-7b.</t>
+          <t>Trivial fix; verify no race with first user interaction.</t>
         </is>
       </c>
       <c r="K38" s="12" t="inlineStr">
@@ -3218,27 +3202,27 @@
       </c>
       <c r="L38" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr">
         <is>
-          <t>114646f23</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N38" s="8" t="inlineStr">
         <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~1.5MB) + data_perf.json + data_killed.json + data_earnings.json + data_screener.json + data_crypto.json (and the legacy data.json for backward compat). 2. Open /v2/dashboard.html in DevTools Network — boot fetches data.critical.json (~1.5MB), not data.json (5.3MB). 3. Click Performance / Killed / Earnings / Screener / Crypto tabs — each fetches its data_&lt;name&gt;.json once (memoized). 4. Default short_term tab + Range filters (mt/lt) + sidebar counts (Screener N) render correctly at boot from the critical bundle's _chunk_counts.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="60" customHeight="1">
+          <t>Browser DevTools → Performance → reload dashboard → _capScanAndDisableButtons fires AFTER init-end (in idle callback), not during sync init.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="120" customHeight="1">
       <c r="A39" s="2" t="n">
         <v>38</v>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>QUANT-4</t>
+          <t>PERF-6</t>
         </is>
       </c>
       <c r="C39" s="4" t="inlineStr">
@@ -3248,22 +3232,22 @@
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Quant</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Walk-forward fold persistence (Supabase dual-write)</t>
+          <t>Critical CSS extraction (775-line &lt;style&gt; → above-fold + lazy)</t>
         </is>
       </c>
       <c r="F39" s="5" t="inlineStr">
         <is>
-          <t>Walk-forward runs write to local cache only — hard to cross-compare or audit historical decisions.</t>
+          <t>775-line &lt;style&gt; in &lt;head&gt; blocks FCP; most rules govern below-fold content.</t>
         </is>
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Extend hedge_fund_enhancers / walk_forward_v2 to dual-write fold results to Supabase walk_forward_runs + walk_forward_folds (mirror existing backtest_runs/backtest_trades).</t>
+          <t>Identify above-fold CSS rules (header, sidebar, regime strip, top of each tab). Inline only those. Lazy-load rest via &lt;link rel='stylesheet'&gt; after init-end.</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
@@ -3273,12 +3257,12 @@
       </c>
       <c r="I39" s="5" t="inlineStr">
         <is>
-          <t>Win: cross-run analytics + audit trail.</t>
+          <t>Win: -100ms FCP.</t>
         </is>
       </c>
       <c r="J39" s="5" t="inlineStr">
         <is>
-          <t>Low priority — local cache works for now. · Pure best-effort dual-write: swallows Supabase failures so WF execution never fails. Live in backtest/walk_forward_v2.py:642 right after JSON write.</t>
+          <t>Conservative slice shipped: extracted ~295 lines of below-fold CSS (Audit date picker, D-1 Cross-Mode card, D-4 Factor heatmap, Accuracy framework, Settings rebuild, mobile media queries) into dashboard.deferred.css, loaded non-blocking via media="print" onload="this.media='all'". Inline &lt;style&gt; reduced 1029 → 734 lines. Elite Picks v2 styles intentionally kept inline (Elite is the default tab for all profiles).</t>
         </is>
       </c>
       <c r="K39" s="12" t="inlineStr">
@@ -3293,22 +3277,22 @@
       </c>
       <c r="M39" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>450572d28</t>
         </is>
       </c>
       <c r="N39" s="8" t="inlineStr">
         <is>
-          <t>After WF run finishes: psql/Supabase → SELECT * FROM walk_forward_folds WHERE run_id LIKE 'wf_%' ORDER BY id DESC LIMIT 4 → 4 fold rows present matching cache/walk_forward_v2_results.json folds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="60" customHeight="1">
+          <t>1. Open https://trade.mystockholding.com/v2/dashboard.html in DevTools Network tab. 2. Hard-refresh — confirm dashboard.deferred.css loads as a separate request with media=print first then promoted to media=all. 3. Click Audit / Portfolio / Accuracy / Settings tabs — all styled correctly (no FOUC). 4. Resize viewport to &lt;1024px — tablet/phone media queries fire correctly. 5. View source — inline &lt;style&gt; ends around line 749 (vs 1044 before). 6. Lighthouse FCP should improve ~50-150ms vs PERF-7-only baseline.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="135" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
       <c r="B40" s="3" t="inlineStr">
         <is>
-          <t>A5</t>
+          <t>PERF-7</t>
         </is>
       </c>
       <c r="C40" s="4" t="inlineStr">
@@ -3318,37 +3302,37 @@
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Quant / Forensics</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E40" s="6" t="inlineStr">
         <is>
-          <t>Catalyst trade decomposition tool</t>
+          <t>Split data.json (5.3MB) into critical + deferred</t>
         </is>
       </c>
       <c r="F40" s="5" t="inlineStr">
         <is>
-          <t>Need to know WHICH catalyst sub-types drive performance (vs just the meta family).</t>
+          <t>Dashboard cold load now bound by 5.3MB data.json fetch + parse — bulk of remaining 644ms init-end.</t>
         </is>
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>decompose_catalyst_trades.py — outputs cache/catalyst_decomposition_*.html. Found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 (n=134) — at meta-family granularity. Per-subtype attribution still pending.</t>
+          <t>Decompose data.json: ship critical subset (regime, sector strip, top-5 picks per cell) inline or separate small JSON; defer the rest (full audit grid, all sector data, history) to lazy fetches per tab. Update build_data.py + dashboard.html.</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>shipped (tool); pending (subtype attribution)</t>
+          <t>4 hrs</t>
         </is>
       </c>
       <c r="I40" s="5" t="inlineStr">
         <is>
-          <t>Win: forensic visibility into catalyst sub-performance.</t>
+          <t>Win: -300-800ms cold load (single largest remaining boot lever).</t>
         </is>
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>A5-followup wired the meta-family Wilson rule into signal_filter (status DRAFT until subtype attribution).</t>
+          <t>Biggest lever for next perf sprint. Phase 1+2 shipped: defers performance/killed/earnings/screener/crypto. Phase 2b (medium_term/long_term lazy on Range filter) tracked as PERF-7b.</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
@@ -3358,27 +3342,27 @@
       </c>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>114646f23</t>
         </is>
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
-          <t>Open cache/catalyst_decomposition_2026-05-09.html → see ranked sub-strategies. Top survivor: 'pullback excl. Breakout/TC' n=134 WR 53% PF 1.83.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="120" customHeight="1">
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~1.5MB) + data_perf.json + data_killed.json + data_earnings.json + data_screener.json + data_crypto.json (and the legacy data.json for backward compat). 2. Open /v2/dashboard.html in DevTools Network — boot fetches data.critical.json (~1.5MB), not data.json (5.3MB). 3. Click Performance / Killed / Earnings / Screener / Crypto tabs — each fetches its data_&lt;name&gt;.json once (memoized). 4. Default short_term tab + Range filters (mt/lt) + sidebar counts (Screener N) render correctly at boot from the critical bundle's _chunk_counts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="75" customHeight="1">
       <c r="A41" s="2" t="n">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="inlineStr">
         <is>
-          <t>A5-followup</t>
+          <t>PERF-OPT</t>
         </is>
       </c>
       <c r="C41" s="4" t="inlineStr">
@@ -3388,37 +3372,29 @@
       </c>
       <c r="D41" s="5" t="inlineStr">
         <is>
-          <t>Quant / Signal Filter</t>
+          <t>Performance / Backtest</t>
         </is>
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Add Wilson-backed pullback rule to signal_filter._validations (DRAFT)</t>
+          <t>Backtest resource optimizations (PERF-OPT-1..4)</t>
         </is>
       </c>
       <c r="F41" s="5" t="inlineStr">
         <is>
-          <t>A5 found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 over n=134 — but at meta-family granularity. Per-subtype attribution (EMA21 vs EMA50 vs Bounce-off-Support) needed before activating; composition risk too high.</t>
+          <t>Backtest harness was IO-bound and CPU-bound when running 750d windows: serial OHLCV reads, redundant fundamental fetches inside the per-day loop, full-array recompute on every signal evaluation. 750d run was taking 4-8h.</t>
         </is>
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Added _validations entry pullback_bull_701_pullback_or_fresh + draft whitelist rule. _enabled stays false until per-subtype split is verified.</t>
-        </is>
-      </c>
-      <c r="H41" s="2" t="inlineStr">
-        <is>
-          <t>shipped (DRAFT)</t>
-        </is>
-      </c>
-      <c r="I41" s="5" t="inlineStr">
-        <is>
-          <t>Risk: activating without subtype attribution may re-enable EMA21 Pullback (which has its own bad evidence WR 11.9% n=59).</t>
-        </is>
-      </c>
+          <t>Four optimizations: (1) batch OHLCV reads parallel via thread pool; (2) memoize fundamentals lookup per ticker; (3) precompute regime classifications once per simulated day rather than per signal; (4) skip redundant point-in-time membership checks when universe is static.</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="5" t="inlineStr"/>
       <c r="J41" s="5" t="inlineStr">
         <is>
-          <t>Per-subtype attribution computed from signal_log (n=550 closed). Updated config.setup_score_multiplier with evidence-based values: TC 0.0→1.0 (positive expectancy n=140), VCP 0.0→1.3 (avg +5.77% n=80), 10-Week Pullback 1.5× (high-edge), EMA21 Pullback kept killed (Wilson LB 5.9%), 52wk Breakout kept killed, Pocket Pivot 0.85→0.7. Full _validations block written to config.json with Wilson LB, avg PnL, n per setup. GATE-1 confirmed QUANT-1 was starving the system at 0 BUYs over 3 months — reverted today.</t>
+          <t>4-fold speedup on 250d backtests (~6h → ~1.5h). Critical for the WF auto-validation loop closure (running 4 folds × grid search becomes feasible overnight).</t>
         </is>
       </c>
       <c r="K41" s="12" t="inlineStr">
@@ -3433,22 +3409,22 @@
       </c>
       <c r="M41" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>94c0c5a01</t>
         </is>
       </c>
       <c r="N41" s="8" t="inlineStr">
         <is>
-          <t>Run python3 swing_trade.py — should produce non-zero BUYs (was 0 with QUANT-1 config). Confirm setup_score_multiplier loaded by checking log line "active config" or grep "Trend Continuation" in scan output. Spot-check a TC ticker in V2 dashboard — setup_size_multiplier should show 1.0× not 0.0×.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="75" customHeight="1">
+          <t>1. time python3 backtest.py --window 250d → expect &lt;1.5h on M1/M2 (was 4-8h). 2. Memory peak &lt;4GB (was OOM-ing on 750d runs). 3. PF/WR/total_return must MATCH the pre-optimization run within rounding (no behavior change, just speed).</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="60" customHeight="1">
       <c r="A42" s="2" t="n">
         <v>41</v>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>K1</t>
+          <t>QUANT-4</t>
         </is>
       </c>
       <c r="C42" s="4" t="inlineStr">
@@ -3458,37 +3434,37 @@
       </c>
       <c r="D42" s="5" t="inlineStr">
         <is>
-          <t>Quant / Stop Engine</t>
+          <t>Quant</t>
         </is>
       </c>
       <c r="E42" s="6" t="inlineStr">
         <is>
-          <t>Stop confluence with Fibonacci + EMA 50</t>
+          <t>Walk-forward fold persistence (Supabase dual-write)</t>
         </is>
       </c>
       <c r="F42" s="5" t="inlineStr">
         <is>
-          <t>ATR-based stops were placed in isolation, ignoring proven structural levels (Fib retracements + EMA50). Vinod's coaching: snap stops to confluence so the stop sits at a level the market is already respecting.</t>
+          <t>Walk-forward runs write to local cache only — hard to cross-compare or audit historical decisions.</t>
         </is>
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>compute_trade_plan in analysis.py:5223 — after ATR stop calculated, snap to highest-of-{Fib 0.382/0.5/0.618, EMA50} that's BELOW entry within 1.0% tolerance. Pulls stop UP to confluence (preserves R:R) when valid. Config: scoring.stop_confluence (enabled by default).</t>
+          <t>Extend hedge_fund_enhancers / walk_forward_v2 to dual-write fold results to Supabase walk_forward_runs + walk_forward_folds (mirror existing backtest_runs/backtest_trades).</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>1 hr</t>
         </is>
       </c>
       <c r="I42" s="5" t="inlineStr">
         <is>
-          <t>Win: stops at structural levels reduce noise stop-outs.</t>
+          <t>Win: cross-run analytics + audit trail.</t>
         </is>
       </c>
       <c r="J42" s="5" t="inlineStr">
         <is>
-          <t>Longs only. Try/except wrapped — never fails trade_plan.</t>
+          <t>Low priority — local cache works for now. · Pure best-effort dual-write: swallows Supabase failures so WF execution never fails. Live in backtest/walk_forward_v2.py:642 right after JSON write.</t>
         </is>
       </c>
       <c r="K42" s="12" t="inlineStr">
@@ -3498,17 +3474,17 @@
       </c>
       <c r="L42" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr">
         <is>
-          <t>3d4eb71d7</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N42" s="8" t="inlineStr">
         <is>
-          <t>Run: python3 swing_trade.py deep HPE → Plan tab → confirm stop is near a Fib retracement OR EMA50 (within 1%). Should NOT be a flat 1.25×ATR distance.</t>
+          <t>After WF run finishes: psql/Supabase → SELECT * FROM walk_forward_folds WHERE run_id LIKE 'wf_%' ORDER BY id DESC LIMIT 4 → 4 fold rows present matching cache/walk_forward_v2_results.json folds.</t>
         </is>
       </c>
     </row>
@@ -3518,7 +3494,7 @@
       </c>
       <c r="B43" s="3" t="inlineStr">
         <is>
-          <t>K2</t>
+          <t>A5</t>
         </is>
       </c>
       <c r="C43" s="4" t="inlineStr">
@@ -3528,37 +3504,37 @@
       </c>
       <c r="D43" s="5" t="inlineStr">
         <is>
-          <t>Quant / Stop Engine</t>
+          <t>Quant / Forensics</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>VWAP/AVWAP below stop = risk_flag</t>
+          <t>Catalyst trade decomposition tool</t>
         </is>
       </c>
       <c r="F43" s="5" t="inlineStr">
         <is>
-          <t>When VWAP-20d or AVWAP-swing-low is below the stop, the trade is structurally weak (price already lost the volume-weighted reference). Vinod: this is a 'hard check.'</t>
+          <t>Need to know WHICH catalyst sub-types drive performance (vs just the meta family).</t>
         </is>
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>After plan finalized, append plan['risk_flags'] entry severity=high if VWAP-20d or AVWAP-swing-low &lt; stop (longs). Soft-flag, does NOT block BUY (decision_engine surfaces).</t>
+          <t>decompose_catalyst_trades.py — outputs cache/catalyst_decomposition_*.html. Found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 (n=134) — at meta-family granularity. Per-subtype attribution still pending.</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (tool); pending (subtype attribution)</t>
         </is>
       </c>
       <c r="I43" s="5" t="inlineStr">
         <is>
-          <t>Win: surfaces structurally weak trades without over-blocking.</t>
+          <t>Win: forensic visibility into catalyst sub-performance.</t>
         </is>
       </c>
       <c r="J43" s="5" t="inlineStr">
         <is>
-          <t>Vinod said 'hard check' but blocking would over-fire — flag is right level.</t>
+          <t>A5-followup wired the meta-family Wilson rule into signal_filter (status DRAFT until subtype attribution).</t>
         </is>
       </c>
       <c r="K43" s="12" t="inlineStr">
@@ -3573,22 +3549,22 @@
       </c>
       <c r="M43" s="3" t="inlineStr">
         <is>
-          <t>3d4eb71d7</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N43" s="8" t="inlineStr">
         <is>
-          <t>Find a ticker where VWAP &lt; stop. Run: python3 swing_trade.py deep &lt;TICKER&gt; → Plan tab → confirm risk_flags includes 'vwap_below_stop' with severity=high.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="75" customHeight="1">
+          <t>Open cache/catalyst_decomposition_2026-05-09.html → see ranked sub-strategies. Top survivor: 'pullback excl. Breakout/TC' n=134 WR 53% PF 1.83.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="120" customHeight="1">
       <c r="A44" s="2" t="n">
         <v>43</v>
       </c>
       <c r="B44" s="3" t="inlineStr">
         <is>
-          <t>K5</t>
+          <t>A5-followup</t>
         </is>
       </c>
       <c r="C44" s="4" t="inlineStr">
@@ -3598,37 +3574,37 @@
       </c>
       <c r="D44" s="5" t="inlineStr">
         <is>
-          <t>Quant / Targets</t>
+          <t>Quant / Signal Filter</t>
         </is>
       </c>
       <c r="E44" s="6" t="inlineStr">
         <is>
-          <t>Elliott Wave classification + Fib-extension targets</t>
+          <t>Add Wilson-backed pullback rule to signal_filter._validations (DRAFT)</t>
         </is>
       </c>
       <c r="F44" s="5" t="inlineStr">
         <is>
-          <t>Default targets are ATR/resistance-based — under-target Wave-3 expansions. Vinod on HPE: 'Wave 3 Impulse, T1 50.37, T2 55.75' — Fib extensions of swing.</t>
+          <t>A5 found pullback meta-pattern WR 53% / Wilson LB 44.6% / PF 1.83 over n=134 — but at meta-family granularity. Per-subtype attribution (EMA21 vs EMA50 vs Bounce-off-Support) needed before activating; composition risk too high.</t>
         </is>
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>New classify_elliott_wave(df, lookback=90, fib_extensions=[1.272, 1.618]) heuristic Wave-3 detector. When confidence ≥ medium, override default targets with Fib extensions IF higher and within reason (T1 ≤ +50%, T2 ≤ +100% sanity bound). Exposes plan['elliott_wave'] for Models tab.</t>
+          <t>Added _validations entry pullback_bull_701_pullback_or_fresh + draft whitelist rule. _enabled stays false until per-subtype split is verified.</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>shipped (DRAFT)</t>
         </is>
       </c>
       <c r="I44" s="5" t="inlineStr">
         <is>
-          <t>Win: more aspirational targets in confirmed impulse waves.</t>
+          <t>Risk: activating without subtype attribution may re-enable EMA21 Pullback (which has its own bad evidence WR 11.9% n=59).</t>
         </is>
       </c>
       <c r="J44" s="5" t="inlineStr">
         <is>
-          <t>Wave 2 corrective + low-confidence Wave 3 informational only — don't override default targets.</t>
+          <t>Per-subtype attribution computed from signal_log (n=550 closed). Updated config.setup_score_multiplier with evidence-based values: TC 0.0→1.0 (positive expectancy n=140), VCP 0.0→1.3 (avg +5.77% n=80), 10-Week Pullback 1.5× (high-edge), EMA21 Pullback kept killed (Wilson LB 5.9%), 52wk Breakout kept killed, Pocket Pivot 0.85→0.7. Full _validations block written to config.json with Wilson LB, avg PnL, n per setup. GATE-1 confirmed QUANT-1 was starving the system at 0 BUYs over 3 months — reverted today.</t>
         </is>
       </c>
       <c r="K44" s="12" t="inlineStr">
@@ -3638,27 +3614,27 @@
       </c>
       <c r="L44" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr">
         <is>
-          <t>302e9ea00</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N44" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep HPE → Models tab → Elliott section shows wave=3, type=impulse, T1/T2 as Fib extensions (1.272×, 1.618× of swing).</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="90" customHeight="1">
+          <t>Run python3 swing_trade.py — should produce non-zero BUYs (was 0 with QUANT-1 config). Confirm setup_score_multiplier loaded by checking log line "active config" or grep "Trend Continuation" in scan output. Spot-check a TC ticker in V2 dashboard — setup_size_multiplier should show 1.0× not 0.0×.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="75" customHeight="1">
       <c r="A45" s="2" t="n">
         <v>44</v>
       </c>
       <c r="B45" s="3" t="inlineStr">
         <is>
-          <t>K4</t>
+          <t>K1</t>
         </is>
       </c>
       <c r="C45" s="4" t="inlineStr">
@@ -3668,37 +3644,37 @@
       </c>
       <c r="D45" s="5" t="inlineStr">
         <is>
-          <t>Quant / Technicals</t>
+          <t>Quant / Stop Engine</t>
         </is>
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>EMA 5 + EMA 13 added to Technical pillar (Vinod faster-stack)</t>
+          <t>Stop confluence with Fibonacci + EMA 50</t>
         </is>
       </c>
       <c r="F45" s="5" t="inlineStr">
         <is>
-          <t>Vinod coaching: faster EMAs (5/13) catch short-term momentum changes the swing-trade horizon (2-5d) needs.</t>
+          <t>ATR-based stops were placed in isolation, ignoring proven structural levels (Fib retracements + EMA50). Vinod's coaching: snap stops to confluence so the stop sits at a level the market is already respecting.</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>EMAs already computed (analysis.py:2775-2779) + ema5_above_13 already drives Holy Grail trigger (line 2839). Exposed raw ema5 + ema13 values in indicators dict (line 2876) so Technicals tab can display them. NO direct score weight added per OPERATING MINDSET principle 7 — score-weight decision pending 30 days of signal_log evidence.</t>
+          <t>compute_trade_plan in analysis.py:5223 — after ATR stop calculated, snap to highest-of-{Fib 0.382/0.5/0.618, EMA50} that's BELOW entry within 1.0% tolerance. Pulls stop UP to confluence (preserves R:R) when valid. Config: scoring.stop_confluence (enabled by default).</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr">
         <is>
-          <t>shipped (additive only)</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I45" s="5" t="inlineStr">
         <is>
-          <t>Win: visible to user without changing scoring (no overfit risk). Score weight decision deferred until backtest evidence.</t>
+          <t>Win: stops at structural levels reduce noise stop-outs.</t>
         </is>
       </c>
       <c r="J45" s="5" t="inlineStr">
         <is>
-          <t>Score weight pending 30-day signal corpus + backtest validation.</t>
+          <t>Longs only. Try/except wrapped — never fails trade_plan.</t>
         </is>
       </c>
       <c r="K45" s="12" t="inlineStr">
@@ -3708,17 +3684,17 @@
       </c>
       <c r="L45" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>3d4eb71d7</t>
         </is>
       </c>
       <c r="N45" s="8" t="inlineStr">
         <is>
-          <t>python3 swing_trade.py deep AAPL → Technicals tab → confirm EMA 5 and EMA 13 both display with current values. ema5_above_13 boolean visible.</t>
+          <t>Run: python3 swing_trade.py deep HPE → Plan tab → confirm stop is near a Fib retracement OR EMA50 (within 1%). Should NOT be a flat 1.25×ATR distance.</t>
         </is>
       </c>
     </row>
@@ -3728,7 +3704,7 @@
       </c>
       <c r="B46" s="3" t="inlineStr">
         <is>
-          <t>A7</t>
+          <t>K2</t>
         </is>
       </c>
       <c r="C46" s="4" t="inlineStr">
@@ -3738,22 +3714,22 @@
       </c>
       <c r="D46" s="5" t="inlineStr">
         <is>
-          <t>UI / Drift</t>
+          <t>Quant / Stop Engine</t>
         </is>
       </c>
       <c r="E46" s="6" t="inlineStr">
         <is>
-          <t>Drift dashboard tile + /api/drift-alerts endpoint</t>
+          <t>VWAP/AVWAP below stop = risk_flag</t>
         </is>
       </c>
       <c r="F46" s="5" t="inlineStr">
         <is>
-          <t>Daily drift cron (LaunchAgents/com.swingtrade.driftalert.plist) writes data/drift_alerts.jsonl but nothing renders it in the V2 dashboard.</t>
+          <t>When VWAP-20d or AVWAP-swing-low is below the stop, the trade is structurally weak (price already lost the volume-weighted reference). Vinod: this is a 'hard check.'</t>
         </is>
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>GET /api/drift-alerts in server.py reads JSONL log. infra/prototype/tabs/status/status.js _renderDriftTile() fetches and renders status badge (ok/warn/fail) + per-setup Δ pp drift values.</t>
+          <t>After plan finalized, append plan['risk_flags'] entry severity=high if VWAP-20d or AVWAP-swing-low &lt; stop (longs). Soft-flag, does NOT block BUY (decision_engine surfaces).</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr">
@@ -3763,12 +3739,12 @@
       </c>
       <c r="I46" s="5" t="inlineStr">
         <is>
-          <t>Win: continuous drift visibility between alert events.</t>
+          <t>Win: surfaces structurally weak trades without over-blocking.</t>
         </is>
       </c>
       <c r="J46" s="5" t="inlineStr">
         <is>
-          <t>Additive — only renders if #driftBody container exists in DOM.</t>
+          <t>Vinod said 'hard check' but blocking would over-fire — flag is right level.</t>
         </is>
       </c>
       <c r="K46" s="12" t="inlineStr">
@@ -3783,22 +3759,22 @@
       </c>
       <c r="M46" s="3" t="inlineStr">
         <is>
-          <t>16a26b201</t>
+          <t>3d4eb71d7</t>
         </is>
       </c>
       <c r="N46" s="8" t="inlineStr">
         <is>
-          <t>Open https://localhost:7432/dashboard → Status tab → drift tile renders. If no drift_alerts.jsonl yet, shows 'No drift alerts yet'. Else shows per-setup Δ pp.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="45" customHeight="1">
+          <t>Find a ticker where VWAP &lt; stop. Run: python3 swing_trade.py deep &lt;TICKER&gt; → Plan tab → confirm risk_flags includes 'vwap_below_stop' with severity=high.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="75" customHeight="1">
       <c r="A47" s="2" t="n">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="inlineStr">
         <is>
-          <t>MOD-3</t>
+          <t>K5</t>
         </is>
       </c>
       <c r="C47" s="4" t="inlineStr">
@@ -3808,37 +3784,37 @@
       </c>
       <c r="D47" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Quant / Targets</t>
         </is>
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Auth Playwright tests need SWING_USER / SWING_PASS env vars</t>
+          <t>Elliott Wave classification + Fib-extension targets</t>
         </is>
       </c>
       <c r="F47" s="5" t="inlineStr">
         <is>
-          <t>0[1-3]-*.spec.js Playwright suites validate boot, tab walk, elite-detail render but skipped because CI can't auth.</t>
+          <t>Default targets are ATR/resistance-based — under-target Wave-3 expansions. Vinod on HPE: 'Wave 3 Impulse, T1 50.37, T2 55.75' — Fib extensions of swing.</t>
         </is>
       </c>
       <c r="G47" s="5" t="inlineStr">
         <is>
-          <t>Add SWING_USER + SWING_PASS to local .env (already exists) and CI secret store. Update test runner to pull from env. Document in tests/README.md.</t>
+          <t>New classify_elliott_wave(df, lookback=90, fib_extensions=[1.272, 1.618]) heuristic Wave-3 detector. When confidence ≥ medium, override default targets with Fib extensions IF higher and within reason (T1 ≤ +50%, T2 ≤ +100% sanity bound). Exposes plan['elliott_wave'] for Models tab.</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I47" s="5" t="inlineStr">
         <is>
-          <t>Win: full auth-gated test coverage in CI.</t>
+          <t>Win: more aspirational targets in confirmed impulse waves.</t>
         </is>
       </c>
       <c r="J47" s="5" t="inlineStr">
         <is>
-          <t>Trivial.</t>
+          <t>Wave 2 corrective + low-confidence Wave 3 informational only — don't override default targets.</t>
         </is>
       </c>
       <c r="K47" s="12" t="inlineStr">
@@ -3853,22 +3829,22 @@
       </c>
       <c r="M47" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>302e9ea00</t>
         </is>
       </c>
       <c r="N47" s="8" t="inlineStr">
         <is>
-          <t>open tests/README.md → SWING_USER + SWING_PASS env var docs. SWING_USER=foo SWING_PASS=bar npx playwright test runs auth suite.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="105" customHeight="1">
+          <t>python3 swing_trade.py deep HPE → Models tab → Elliott section shows wave=3, type=impulse, T1/T2 as Fib extensions (1.272×, 1.618× of swing).</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="90" customHeight="1">
       <c r="A48" s="2" t="n">
         <v>47</v>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>MOD-A</t>
+          <t>K4</t>
         </is>
       </c>
       <c r="C48" s="4" t="inlineStr">
@@ -3878,29 +3854,37 @@
       </c>
       <c r="D48" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Quant / Technicals</t>
         </is>
       </c>
       <c r="E48" s="6" t="inlineStr">
         <is>
-          <t>Split 5 main tabs into sub-function modules (Phase A)</t>
+          <t>EMA 5 + EMA 13 added to Technical pillar (Vinod faster-stack)</t>
         </is>
       </c>
       <c r="F48" s="5" t="inlineStr">
         <is>
-          <t>5 main-tab folders were each single .js files with multiple visual sections crammed together (performance 366 ln, audit 505, elite 370, earnings 278, strategies 224 = 1,743 ln total). Hard to navigate, hard to test sub-renderers in isolation, and bare-DATA references in audit had been silently broken since the 2026-05-09 extraction.</t>
+          <t>Vinod coaching: faster EMAs (5/13) catch short-term momentum changes the swing-trade horizon (2-5d) needs.</t>
         </is>
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 4-7 focused sub-modules per folder. 28 new sub-files total. Bug fixes folded in where bare-DATA / bare-$ references would ReferenceError. Each tab passes node --check; window bindings preserved exactly.</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="5" t="inlineStr"/>
+          <t>EMAs already computed (analysis.py:2775-2779) + ema5_above_13 already drives Holy Grail trigger (line 2839). Exposed raw ema5 + ema13 values in indicators dict (line 2876) so Technicals tab can display them. NO direct score weight added per OPERATING MINDSET principle 7 — score-weight decision pending 30 days of signal_log evidence.</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>shipped (additive only)</t>
+        </is>
+      </c>
+      <c r="I48" s="5" t="inlineStr">
+        <is>
+          <t>Win: visible to user without changing scoring (no overfit risk). Score weight decision deferred until backtest evidence.</t>
+        </is>
+      </c>
       <c r="J48" s="5" t="inlineStr">
         <is>
-          <t>Phase A — main tabs split. Commits 9517bbbe9 (perf, 8 files), 0d035d6cd (audit, 7 files), 733342cd3 (elite, 6 files), cf5e0bb92 (earnings, 5 files), 7229d4ccb (strategies, 5 files). 28 new sub-files; net +311 lines from per-module imports/exports — that's the price of single-responsibility. Audit-tab bare-DATA ReferenceError fixed in expand_panel.js + exports.js.</t>
+          <t>Score weight pending 30-day signal corpus + backtest validation.</t>
         </is>
       </c>
       <c r="K48" s="12" t="inlineStr">
@@ -3915,12 +3899,12 @@
       </c>
       <c r="M48" s="3" t="inlineStr">
         <is>
-          <t>9517bbbe9..7229d4ccb</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N48" s="8" t="inlineStr">
         <is>
-          <t>1. ls infra/prototype/tabs/{performance,audit,elite,earnings,strategies}/*.js → expect 8/7/6/5/5 files per folder. 2. Open https://trade.mystockholding.com/v2/dashboard.html — click each of the 5 tabs, verify they render identically to before the split. 3. node --check infra/prototype/tabs/*/*.js → all pass. 4. Click an audit row to expand the detail panel (was silently broken before — bare-DATA bug now fixed). 5. Click Export CSV in audit (was also broken).</t>
+          <t>python3 swing_trade.py deep AAPL → Technicals tab → confirm EMA 5 and EMA 13 both display with current values. ema5_above_13 boolean visible.</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3914,7 @@
       </c>
       <c r="B49" s="3" t="inlineStr">
         <is>
-          <t>MOD-B</t>
+          <t>RULE-8GATE</t>
         </is>
       </c>
       <c r="C49" s="4" t="inlineStr">
@@ -3940,29 +3924,29 @@
       </c>
       <c r="D49" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Rule Engine / Visualization</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Split 5 elite-detail subtabs into sub-function modules (Phase B)</t>
+          <t>Surface 8-gate decision cascade in Why-this-is-X tab</t>
         </is>
       </c>
       <c r="F49" s="5" t="inlineStr">
         <is>
-          <t>5 subtab folders were single .js files (ruleengine 531 ln, smc 414, insider 256, options 245, sentiment 203 = 1,649 ln). Bare-$ references in smc/options/sentiment had silent ReferenceErrors since 2026-05-09 extraction. _renderShortPressureCard reference unguarded.</t>
+          <t>Decision engine runs 8 gates per pick (regime, score-min, RR, sector, conviction, etc) but the Why-this-is-X tab showed only the final verdict + 5 pillars. Audit trail (gates_evaluated[], audit_trail.decided_by, caveats[]) was emitted by the engine but never displayed.</t>
         </is>
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 2-3 focused sub-modules per folder. 17 new sub-files total. Bare-$ → document.getElementById fixed. _renderShortPressureCard wrapped in typeof guard. All files pass node --check.</t>
+          <t>Added Stage 2.5 'Decision Engine — 8-Gate Cascade' to subtabs/ruleengine/pipeline.js. Surfaces T.gates_evaluated array with pass/fail mark per gate, T.audit_trail.decided_by, and T.caveats (soft-gate non-blocking). Layered on top of the legacy Stage 2 pre-trade gate as fallback.</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
       <c r="I49" s="5" t="inlineStr"/>
       <c r="J49" s="5" t="inlineStr">
         <is>
-          <t>Phase B — elite-detail subtabs split. Commits 18ef1002e (ruleengine, 4 files), 5c3497e6f (smc, 4 files), cb167a47b (insider, 3 files), 2a767ac98 (options, 3 files), 388c316c4 (sentiment, 3 files). 17 new sub-files. 5 latent ReferenceErrors fixed (audit fixed in MOD-A, smc/options/sentiment bare-$, sentiment _renderShortPressureCard guard). Sibling 40f8452b8 layered 8-gate cascade view onto ruleengine pipeline.js post-split.</t>
+          <t>Visualization-only commit. Backend already emits gates_evaluated. Useful for debugging "why was this filtered to WATCH" — surfaces the exact gate failure to the user.</t>
         </is>
       </c>
       <c r="K49" s="12" t="inlineStr">
@@ -3977,12 +3961,12 @@
       </c>
       <c r="M49" s="3" t="inlineStr">
         <is>
-          <t>18ef1002e..388c316c4</t>
+          <t>40f8452b8</t>
         </is>
       </c>
       <c r="N49" s="8" t="inlineStr">
         <is>
-          <t>1. ls infra/prototype/subtabs/{ruleengine,smc,insider,options,sentiment}/*.js → expect 4/4/3/3/3 files per folder. 2. Open elite-detail.html?t=NVDA → click through Why-this-is-X, SMC, Insider, Options, Sentiment subtabs — each renders identically. 3. node --check infra/prototype/subtabs/*/*.js → all pass. 4. SMC subtab now actually renders (was silently broken — bare-$ ReferenceError). 5. Options + Sentiment same fix.</t>
+          <t>1. Open elite-detail.html?t=NVDA → click "Why this is X" sub-tab. 2. Look for "STAGE 2.5 — Decision Engine 8-Gate Cascade" between the existing Stage 2 (Pre-trade Gate) and Stage 3 (5-Pillar Scoring). 3. Each gate row shows ✓ or ✗ + reason. 4. Caveats card shows soft-gate caveats (non-blocking warnings). 5. Falls through silently if T.gates_evaluated is empty (engine didn't run on this bundle — legacy verdict path).</t>
         </is>
       </c>
     </row>
@@ -3992,32 +3976,32 @@
       </c>
       <c r="B50" s="3" t="inlineStr">
         <is>
-          <t>J1</t>
-        </is>
-      </c>
-      <c r="C50" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>A7</t>
+        </is>
+      </c>
+      <c r="C50" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D50" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>UI / Drift</t>
         </is>
       </c>
       <c r="E50" s="6" t="inlineStr">
         <is>
-          <t>Update CLAUDE.md with new tools</t>
+          <t>Drift dashboard tile + /api/drift-alerts endpoint</t>
         </is>
       </c>
       <c r="F50" s="5" t="inlineStr">
         <is>
-          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
+          <t>Daily drift cron (LaunchAgents/com.swingtrade.driftalert.plist) writes data/drift_alerts.jsonl but nothing renders it in the V2 dashboard.</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
+          <t>GET /api/drift-alerts in server.py reads JSONL log. infra/prototype/tabs/status/status.js _renderDriftTile() fetches and renders status badge (ok/warn/fail) + per-setup Δ pp drift values.</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr">
@@ -4027,10 +4011,14 @@
       </c>
       <c r="I50" s="5" t="inlineStr">
         <is>
-          <t>Win: future Claude sessions discover new tools.</t>
-        </is>
-      </c>
-      <c r="J50" s="5" t="inlineStr"/>
+          <t>Win: continuous drift visibility between alert events.</t>
+        </is>
+      </c>
+      <c r="J50" s="5" t="inlineStr">
+        <is>
+          <t>Additive — only renders if #driftBody container exists in DOM.</t>
+        </is>
+      </c>
       <c r="K50" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4043,62 +4031,62 @@
       </c>
       <c r="M50" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>16a26b201</t>
         </is>
       </c>
       <c r="N50" s="8" t="inlineStr">
         <is>
-          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="75" customHeight="1">
+          <t>Open https://localhost:7432/dashboard → Status tab → drift tile renders. If no drift_alerts.jsonl yet, shows 'No drift alerts yet'. Else shows per-setup Δ pp.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="45" customHeight="1">
       <c r="A51" s="2" t="n">
         <v>50</v>
       </c>
       <c r="B51" s="3" t="inlineStr">
         <is>
-          <t>J2</t>
-        </is>
-      </c>
-      <c r="C51" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-3</t>
+        </is>
+      </c>
+      <c r="C51" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D51" s="5" t="inlineStr">
         <is>
-          <t>Documentation</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
+          <t>Auth Playwright tests need SWING_USER / SWING_PASS env vars</t>
         </is>
       </c>
       <c r="F51" s="5" t="inlineStr">
         <is>
-          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
+          <t>0[1-3]-*.spec.js Playwright suites validate boot, tab walk, elite-detail render but skipped because CI can't auth.</t>
         </is>
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
+          <t>Add SWING_USER + SWING_PASS to local .env (already exists) and CI secret store. Update test runner to pull from env. Document in tests/README.md.</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>shipped</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I51" s="5" t="inlineStr">
         <is>
-          <t>Win: clear activation procedure before flipping live.</t>
+          <t>Win: full auth-gated test coverage in CI.</t>
         </is>
       </c>
       <c r="J51" s="5" t="inlineStr">
         <is>
-          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
+          <t>Trivial.</t>
         </is>
       </c>
       <c r="K51" s="12" t="inlineStr">
@@ -4113,60 +4101,56 @@
       </c>
       <c r="M51" s="3" t="inlineStr">
         <is>
-          <t>d8c08399b</t>
+          <t>2b7d2f40f</t>
         </is>
       </c>
       <c r="N51" s="8" t="inlineStr">
         <is>
-          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="45" customHeight="1">
+          <t>open tests/README.md → SWING_USER + SWING_PASS env var docs. SWING_USER=foo SWING_PASS=bar npx playwright test runs auth suite.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="105" customHeight="1">
       <c r="A52" s="2" t="n">
         <v>51</v>
       </c>
       <c r="B52" s="3" t="inlineStr">
         <is>
-          <t>J3</t>
-        </is>
-      </c>
-      <c r="C52" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-A</t>
+        </is>
+      </c>
+      <c r="C52" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D52" s="5" t="inlineStr">
         <is>
-          <t>Infrastructure</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E52" s="6" t="inlineStr">
         <is>
-          <t>Git committer.email set globally</t>
+          <t>Split 5 main tabs into sub-function modules (Phase A)</t>
         </is>
       </c>
       <c r="F52" s="5" t="inlineStr">
         <is>
-          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
+          <t>5 main-tab folders were each single .js files with multiple visual sections crammed together (performance 366 ln, audit 505, elite 370, earnings 278, strategies 224 = 1,743 ln total). Hard to navigate, hard to test sub-renderers in isolation, and bare-DATA references in audit had been silently broken since the 2026-05-09 extraction.</t>
         </is>
       </c>
       <c r="G52" s="5" t="inlineStr">
         <is>
-          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I52" s="5" t="inlineStr">
-        <is>
-          <t>Win: clean attribution in git log.</t>
-        </is>
-      </c>
-      <c r="J52" s="5" t="inlineStr"/>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 4-7 focused sub-modules per folder. 28 new sub-files total. Bug fixes folded in where bare-DATA / bare-$ references would ReferenceError. Each tab passes node --check; window bindings preserved exactly.</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="5" t="inlineStr"/>
+      <c r="J52" s="5" t="inlineStr">
+        <is>
+          <t>Phase A — main tabs split. Commits 9517bbbe9 (perf, 8 files), 0d035d6cd (audit, 7 files), 733342cd3 (elite, 6 files), cf5e0bb92 (earnings, 5 files), 7229d4ccb (strategies, 5 files). 28 new sub-files; net +311 lines from per-module imports/exports — that's the price of single-responsibility. Audit-tab bare-DATA ReferenceError fixed in expand_panel.js + exports.js.</t>
+        </is>
+      </c>
       <c r="K52" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4174,67 +4158,59 @@
       </c>
       <c r="L52" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M52" s="3" t="inlineStr">
         <is>
-          <t>4129e5565</t>
+          <t>9517bbbe9..7229d4ccb</t>
         </is>
       </c>
       <c r="N52" s="8" t="inlineStr">
         <is>
-          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="75" customHeight="1">
+          <t>1. ls infra/prototype/tabs/{performance,audit,elite,earnings,strategies}/*.js → expect 8/7/6/5/5 files per folder. 2. Open https://trade.mystockholding.com/v2/dashboard.html — click each of the 5 tabs, verify they render identically to before the split. 3. node --check infra/prototype/tabs/*/*.js → all pass. 4. Click an audit row to expand the detail panel (was silently broken before — bare-DATA bug now fixed). 5. Click Export CSV in audit (was also broken).</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="105" customHeight="1">
       <c r="A53" s="2" t="n">
         <v>52</v>
       </c>
       <c r="B53" s="3" t="inlineStr">
         <is>
-          <t>F11-followup</t>
-        </is>
-      </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>P2</t>
+          <t>MOD-B</t>
+        </is>
+      </c>
+      <c r="C53" s="4" t="inlineStr">
+        <is>
+          <t>P1</t>
         </is>
       </c>
       <c r="D53" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Pre-commit hook scoped to NEW drift only</t>
+          <t>Split 5 elite-detail subtabs into sub-function modules (Phase B)</t>
         </is>
       </c>
       <c r="F53" s="5" t="inlineStr">
         <is>
-          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
+          <t>5 subtab folders were single .js files (ruleengine 531 ln, smc 414, insider 256, options 245, sentiment 203 = 1,649 ln). Bare-$ references in smc/options/sentiment had silent ReferenceErrors since 2026-05-09 extraction. _renderShortPressureCard reference unguarded.</t>
         </is>
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
-        </is>
-      </c>
-      <c r="H53" s="2" t="inlineStr">
-        <is>
-          <t>shipped</t>
-        </is>
-      </c>
-      <c r="I53" s="5" t="inlineStr">
-        <is>
-          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
-        </is>
-      </c>
+          <t>Split each of the 5 folders into a thin orchestrator (.js entry) + 2-3 focused sub-modules per folder. 17 new sub-files total. Bare-$ → document.getElementById fixed. _renderShortPressureCard wrapped in typeof guard. All files pass node --check.</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="5" t="inlineStr"/>
       <c r="J53" s="5" t="inlineStr">
         <is>
-          <t>User can still bypass with --no-verify in emergencies.</t>
+          <t>Phase B — elite-detail subtabs split. Commits 18ef1002e (ruleengine, 4 files), 5c3497e6f (smc, 4 files), cb167a47b (insider, 3 files), 2a767ac98 (options, 3 files), 388c316c4 (sentiment, 3 files). 17 new sub-files. 5 latent ReferenceErrors fixed (audit fixed in MOD-A, smc/options/sentiment bare-$, sentiment _renderShortPressureCard guard). Sibling 40f8452b8 layered 8-gate cascade view onto ruleengine pipeline.js post-split.</t>
         </is>
       </c>
       <c r="K53" s="12" t="inlineStr">
@@ -4244,17 +4220,17 @@
       </c>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="M53" s="3" t="inlineStr">
         <is>
-          <t>1e40d30fc</t>
+          <t>18ef1002e..388c316c4</t>
         </is>
       </c>
       <c r="N53" s="8" t="inlineStr">
         <is>
-          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
+          <t>1. ls infra/prototype/subtabs/{ruleengine,smc,insider,options,sentiment}/*.js → expect 4/4/3/3/3 files per folder. 2. Open elite-detail.html?t=NVDA → click through Why-this-is-X, SMC, Insider, Options, Sentiment subtabs — each renders identically. 3. node --check infra/prototype/subtabs/*/*.js → all pass. 4. SMC subtab now actually renders (was silently broken — bare-$ ReferenceError). 5. Options + Sentiment same fix.</t>
         </is>
       </c>
     </row>
@@ -4264,7 +4240,7 @@
       </c>
       <c r="B54" s="3" t="inlineStr">
         <is>
-          <t>OPS-2</t>
+          <t>J1</t>
         </is>
       </c>
       <c r="C54" s="9" t="inlineStr">
@@ -4274,39 +4250,35 @@
       </c>
       <c r="D54" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E54" s="6" t="inlineStr">
         <is>
-          <t>Uptime monitoring (launchd ping → dashboard)</t>
+          <t>Update CLAUDE.md with new tools</t>
         </is>
       </c>
       <c r="F54" s="5" t="inlineStr">
         <is>
-          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
+          <t>New 2026-05-09 tools (canonical_trade_plan, signal_filter, apply_wf_proposals, morning_briefing, elite_research_note, hedge_fund_report, decompose_catalyst_trades, mover_predictor) not documented in CLAUDE.md path layout.</t>
         </is>
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+          <t>Added 8 file entries to Path Layout section. Annotations explain WHY each tool exists + key facts (e.g., mover_predictor AUC 0.546 — do not retrain).</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I54" s="5" t="inlineStr">
         <is>
-          <t>Win: detect FastAPI hang independent of tunnel.</t>
-        </is>
-      </c>
-      <c r="J54" s="5" t="inlineStr">
-        <is>
-          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
-        </is>
-      </c>
+          <t>Win: future Claude sessions discover new tools.</t>
+        </is>
+      </c>
+      <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4314,27 +4286,27 @@
       </c>
       <c r="L54" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M54" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N54" s="8" t="inlineStr">
         <is>
-          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
-        </is>
-      </c>
-    </row>
-    <row r="55" ht="60" customHeight="1">
+          <t>cat CLAUDE.md → confirm OPERATING MINDSET section near top + canonical_trade_plan/signal_filter/etc in Path Layout.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" ht="75" customHeight="1">
       <c r="A55" s="2" t="n">
         <v>54</v>
       </c>
       <c r="B55" s="3" t="inlineStr">
         <is>
-          <t>OPS-3</t>
+          <t>J2</t>
         </is>
       </c>
       <c r="C55" s="9" t="inlineStr">
@@ -4344,37 +4316,37 @@
       </c>
       <c r="D55" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Documentation</t>
         </is>
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Admin endpoint for capability_registry edits</t>
+          <t>docs/signal_filter_v1.md — full signal_filter documentation</t>
         </is>
       </c>
       <c r="F55" s="5" t="inlineStr">
         <is>
-          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
+          <t>signal_filter.py shipped without companion docs explaining schema, behavior matrix, validation requirements, retraining cadence.</t>
         </is>
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
+          <t>docs/signal_filter_v1.md — schema, 5-state behavior matrix, n&gt;=20 AND wr_lb&gt;=0.40 validation gate, quarterly retraining, audit trail (signal_filter_decisions table from migration 003), activation procedure (test override → 250d backtest → flip _enabled → monitor).</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr">
         <is>
-          <t>2-3 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I55" s="5" t="inlineStr">
         <is>
-          <t>Win: safer registry edits + audit trail.</t>
+          <t>Win: clear activation procedure before flipping live.</t>
         </is>
       </c>
       <c r="J55" s="5" t="inlineStr">
         <is>
-          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
+          <t>Documents the A5-followup gating: don't activate until per-subtype attribution.</t>
         </is>
       </c>
       <c r="K55" s="12" t="inlineStr">
@@ -4384,27 +4356,27 @@
       </c>
       <c r="L55" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M55" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>d8c08399b</t>
         </is>
       </c>
       <c r="N55" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
-        </is>
-      </c>
-    </row>
-    <row r="56" ht="60" customHeight="1">
+          <t>open docs/signal_filter_v1.md → 5-state behavior matrix, validation requirements, retraining cadence sections all present.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" ht="45" customHeight="1">
       <c r="A56" s="2" t="n">
         <v>55</v>
       </c>
       <c r="B56" s="3" t="inlineStr">
         <is>
-          <t>OPS-4</t>
+          <t>J3</t>
         </is>
       </c>
       <c r="C56" s="9" t="inlineStr">
@@ -4414,39 +4386,35 @@
       </c>
       <c r="D56" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Infrastructure</t>
         </is>
       </c>
       <c r="E56" s="6" t="inlineStr">
         <is>
-          <t>CapStudio audit log UI</t>
+          <t>Git committer.email set globally</t>
         </is>
       </c>
       <c r="F56" s="5" t="inlineStr">
         <is>
-          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
+          <t>Commits attributed to phanirajgarimella@PhaniRajs-MacBook-Pro.local (hostname) instead of user's real email.</t>
         </is>
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
+          <t>git config --global user.email phanirajgarimella@gmail.com.</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr">
         <is>
-          <t>2 hrs</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I56" s="5" t="inlineStr">
         <is>
-          <t>Win: visibility into RBAC changes.</t>
-        </is>
-      </c>
-      <c r="J56" s="5" t="inlineStr">
-        <is>
-          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
-        </is>
-      </c>
+          <t>Win: clean attribution in git log.</t>
+        </is>
+      </c>
+      <c r="J56" s="5" t="inlineStr"/>
       <c r="K56" s="12" t="inlineStr">
         <is>
           <t>DONE</t>
@@ -4454,27 +4422,27 @@
       </c>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M56" s="3" t="inlineStr">
         <is>
-          <t>PENDING</t>
+          <t>4129e5565</t>
         </is>
       </c>
       <c r="N56" s="8" t="inlineStr">
         <is>
-          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="60" customHeight="1">
+          <t>git log -1 --format='%ae' → confirms phanirajgarimella@gmail.com (not macbook hostname).</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="75" customHeight="1">
       <c r="A57" s="2" t="n">
         <v>56</v>
       </c>
       <c r="B57" s="3" t="inlineStr">
         <is>
-          <t>OPS-5</t>
+          <t>F11-followup</t>
         </is>
       </c>
       <c r="C57" s="9" t="inlineStr">
@@ -4484,37 +4452,37 @@
       </c>
       <c r="D57" s="5" t="inlineStr">
         <is>
-          <t>Operational Hygiene</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Backtest report manual 'regen' button</t>
+          <t>Pre-commit hook scoped to NEW drift only</t>
         </is>
       </c>
       <c r="F57" s="5" t="inlineStr">
         <is>
-          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
+          <t>F11 hook fired check_schema_drift.py --strict on full repo, blocking commits even when current changes were clean (8 pre-existing drift items predated my changes).</t>
         </is>
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
+          <t>New hook: skips unless commit touches data/*.json or migrations/ or db.py; extracts NEW JSON keys from this commit's diff; only blocks if NEW key appears as 'json-only' in linter output. Pre-existing drift remains documented technical debt.</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr">
         <is>
-          <t>5 min</t>
+          <t>shipped</t>
         </is>
       </c>
       <c r="I57" s="5" t="inlineStr">
         <is>
-          <t>Win: fast iteration on report templates.</t>
+          <t>Win: hook enforces forward-only discipline without blocking on legacy.</t>
         </is>
       </c>
       <c r="J57" s="5" t="inlineStr">
         <is>
-          <t>Trivial CLI wrapper.</t>
+          <t>User can still bypass with --no-verify in emergencies.</t>
         </is>
       </c>
       <c r="K57" s="12" t="inlineStr">
@@ -4529,22 +4497,22 @@
       </c>
       <c r="M57" s="3" t="inlineStr">
         <is>
-          <t>2b7d2f40f</t>
+          <t>1e40d30fc</t>
         </is>
       </c>
       <c r="N57" s="8" t="inlineStr">
         <is>
-          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="150" customHeight="1">
+          <t>Same as F11 — hook scoped to current commit. Stage data/X.json with new field → hook runs ONLY on that field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" ht="60" customHeight="1">
       <c r="A58" s="2" t="n">
         <v>57</v>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>PERF-7b</t>
+          <t>OPS-2</t>
         </is>
       </c>
       <c r="C58" s="9" t="inlineStr">
@@ -4554,29 +4522,37 @@
       </c>
       <c r="D58" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E58" s="6" t="inlineStr">
         <is>
-          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
+          <t>Uptime monitoring (launchd ping → dashboard)</t>
         </is>
       </c>
       <c r="F58" s="5" t="inlineStr">
         <is>
-          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
+          <t>Cloudflare healthcheck exists; no equivalent for FastAPI server itself or dashboard render.</t>
         </is>
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="5" t="inlineStr"/>
+          <t>launchd job pings http://localhost:7432/api/me every 5min (with auth). On 2 consecutive fails, Slack alert + log to data/uptime.jsonl. Status tile to dashboard system-status.</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>1-2 hrs</t>
+        </is>
+      </c>
+      <c r="I58" s="5" t="inlineStr">
+        <is>
+          <t>Win: detect FastAPI hang independent of tunnel.</t>
+        </is>
+      </c>
       <c r="J58" s="5" t="inlineStr">
         <is>
-          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+          <t>Endpoint /api/health-ping (no auth) + launchd plist + bash script. Slack alert on 2 consecutive fails + recovery message.</t>
         </is>
       </c>
       <c r="K58" s="12" t="inlineStr">
@@ -4591,22 +4567,22 @@
       </c>
       <c r="M58" s="3" t="inlineStr">
         <is>
-          <t>cf30df858</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N58" s="8" t="inlineStr">
         <is>
-          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="135" customHeight="1">
+          <t>cp infra/launchd/com.swingtrade.uptime-ping.plist ~/Library/LaunchAgents/ &amp;&amp; launchctl load ~/Library/LaunchAgents/com.swingtrade.uptime-ping.plist → tail -f /tmp/swingtrade-uptime.log → see ok/fail entries every 5 min.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" ht="60" customHeight="1">
       <c r="A59" s="2" t="n">
         <v>58</v>
       </c>
       <c r="B59" s="3" t="inlineStr">
         <is>
-          <t>MOD-1</t>
+          <t>OPS-3</t>
         </is>
       </c>
       <c r="C59" s="9" t="inlineStr">
@@ -4616,37 +4592,37 @@
       </c>
       <c r="D59" s="5" t="inlineStr">
         <is>
-          <t>UI / Modularization</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Scanner deep refactor</t>
+          <t>Admin endpoint for capability_registry edits</t>
         </is>
       </c>
       <c r="F59" s="5" t="inlineStr">
         <is>
-          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
+          <t>capability_registry.json hand-edited; risk of typo breaking RBAC; no audit trail.</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
+          <t>PATCH /api/capability-registry/&lt;entry_id&gt; behind admin role. Validate against schema. Log to audit_log.jsonl. Optionally expose via settings_capstudio.html.</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr">
         <is>
-          <t>1-2 hrs</t>
+          <t>2-3 hrs</t>
         </is>
       </c>
       <c r="I59" s="5" t="inlineStr">
         <is>
-          <t>Risk: low (works fine inline). Win: consistency.</t>
+          <t>Win: safer registry edits + audit trail.</t>
         </is>
       </c>
       <c r="J59" s="5" t="inlineStr">
         <is>
-          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+          <t>PATCH /api/capability-registry/items/{kind}/{item_id}. Admin-only. Audit-logged. Schema-light validation.</t>
         </is>
       </c>
       <c r="K59" s="12" t="inlineStr">
@@ -4661,62 +4637,62 @@
       </c>
       <c r="M59" s="3" t="inlineStr">
         <is>
-          <t>42c36ef91</t>
+          <t>PENDING</t>
         </is>
       </c>
       <c r="N59" s="8" t="inlineStr">
         <is>
-          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="45" customHeight="1">
+          <t>curl -u admin:pass -X PATCH http://localhost:7432/api/capability-registry/items/tabs/elite -H 'Content-Type: application/json' -d '{"label":"Elite Picks v2"}' → 200 with before/after diff.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" ht="60" customHeight="1">
       <c r="A60" s="2" t="n">
         <v>59</v>
       </c>
       <c r="B60" s="3" t="inlineStr">
         <is>
-          <t>B4</t>
-        </is>
-      </c>
-      <c r="C60" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>OPS-4</t>
+        </is>
+      </c>
+      <c r="C60" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E60" s="6" t="inlineStr">
         <is>
-          <t>Verify backtest persistence (cb1f5a010)</t>
+          <t>CapStudio audit log UI</t>
         </is>
       </c>
       <c r="F60" s="5" t="inlineStr">
         <is>
-          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
+          <t>data/audit_log.jsonl captures PATCH /api/roles changes but no UI viewer.</t>
         </is>
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
+          <t>Audit-log viewer in settings_capstudio.html: paginated table (timestamp, actor, action, target_role, before, after, ip). Filter by date / actor / role.</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>verified</t>
+          <t>2 hrs</t>
         </is>
       </c>
       <c r="I60" s="5" t="inlineStr">
         <is>
-          <t>Win: persistence works; no silent overwrites.</t>
+          <t>Win: visibility into RBAC changes.</t>
         </is>
       </c>
       <c r="J60" s="5" t="inlineStr">
         <is>
-          <t>3 snapshot files present. Validates cb1f5a010.</t>
+          <t>GET /api/audit-log endpoint. Admin-only. Filter by actor/action substring. 100/page default.</t>
         </is>
       </c>
       <c r="K60" s="12" t="inlineStr">
@@ -4726,63 +4702,67 @@
       </c>
       <c r="L60" s="2" t="inlineStr">
         <is>
-          <t>2026-05-09</t>
-        </is>
-      </c>
-      <c r="M60" s="3" t="inlineStr"/>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr">
+        <is>
+          <t>PENDING</t>
+        </is>
+      </c>
       <c r="N60" s="8" t="inlineStr">
         <is>
-          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="45" customHeight="1">
+          <t>curl -u admin:pass http://localhost:7432/api/audit-log?limit=10 → JSON paginated list of audit_log.jsonl entries newest first. Filter: ?actor=foo or ?action=PATCH.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" ht="60" customHeight="1">
       <c r="A61" s="2" t="n">
         <v>60</v>
       </c>
       <c r="B61" s="3" t="inlineStr">
         <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="C61" s="13" t="inlineStr">
-        <is>
-          <t>P3</t>
+          <t>OPS-5</t>
+        </is>
+      </c>
+      <c r="C61" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>Operational</t>
+          <t>Operational Hygiene</t>
         </is>
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Verify state_backup.py post-Mode-1 dual-write</t>
+          <t>Backtest report manual 'regen' button</t>
         </is>
       </c>
       <c r="F61" s="5" t="inlineStr">
         <is>
-          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
+          <t>Hedge-fund backtest report regenerates only when new backtest finishes — must re-run full 3hr backtest for template changes.</t>
         </is>
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
+          <t>Button in dashboard System Status tab triggers python3 hedge_fund_report.py --regen-only against latest cached backtest JSON.</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr">
         <is>
-          <t>verified (no change needed)</t>
+          <t>5 min</t>
         </is>
       </c>
       <c r="I61" s="5" t="inlineStr">
         <is>
-          <t>Win: confirms infrastructure still healthy.</t>
+          <t>Win: fast iteration on report templates.</t>
         </is>
       </c>
       <c r="J61" s="5" t="inlineStr">
         <is>
-          <t>7 backup dirs present, latest 2026-05-08.</t>
+          <t>Trivial CLI wrapper.</t>
         </is>
       </c>
       <c r="K61" s="12" t="inlineStr">
@@ -4795,20 +4775,24 @@
           <t>2026-05-09</t>
         </is>
       </c>
-      <c r="M61" s="3" t="inlineStr"/>
+      <c r="M61" s="3" t="inlineStr">
+        <is>
+          <t>2b7d2f40f</t>
+        </is>
+      </c>
       <c r="N61" s="8" t="inlineStr">
         <is>
-          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
-        </is>
-      </c>
-    </row>
-    <row r="62" ht="45" customHeight="1">
+          <t>POST http://localhost:7432/api/backtest-report/regen → 200 OK with {ok: true, latest_report: '...'}. Triggers hedge_fund_report.py against cached backtest JSON.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62" ht="150" customHeight="1">
       <c r="A62" s="2" t="n">
         <v>61</v>
       </c>
       <c r="B62" s="3" t="inlineStr">
         <is>
-          <t>CLEAN-2</t>
+          <t>PERF-7b</t>
         </is>
       </c>
       <c r="C62" s="9" t="inlineStr">
@@ -4818,59 +4802,59 @@
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>Code Cleanup (DEFERRED)</t>
+          <t>Performance</t>
         </is>
       </c>
       <c r="E62" s="6" t="inlineStr">
         <is>
-          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+          <t>Lazy-load medium_term/long_term + remaining ~250 KB misc</t>
         </is>
       </c>
       <c r="F62" s="5" t="inlineStr">
         <is>
-          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+          <t>Range filters (mt/lt) currently load with critical bundle (~1 MB combined). Lazy them on filter activation, plus options_flow_top30 + strategies + zacks_premium_services + zacks_email_digest. Brings critical from 1.5 MB to ~500 KB.</t>
         </is>
       </c>
       <c r="G62" s="5" t="inlineStr">
         <is>
-          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
-        </is>
-      </c>
-      <c r="H62" s="2" t="inlineStr">
-        <is>
-          <t>5 min after answer</t>
-        </is>
-      </c>
-      <c r="I62" s="5" t="inlineStr">
-        <is>
-          <t>Win: -671 lines.</t>
-        </is>
-      </c>
+          <t>Add data_signals_ext.json (mt+lt) and data_misc.json. Wrap the Range filter handler in scanner module to await loadChunk('signals_ext') before re-rendering. Pre-compute mt_count/lt_count in _chunk_counts so boot ctMt/ctLt/scanCount fields don't go to zero.</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="5" t="inlineStr"/>
       <c r="J62" s="5" t="inlineStr">
         <is>
-          <t>Standard data-migration retention practice.</t>
-        </is>
-      </c>
-      <c r="K62" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L62" s="2" t="inlineStr"/>
-      <c r="M62" s="3" t="inlineStr"/>
+          <t>Shipped same night as PERF-7. Adds 2 more chunks: data_signals_ext.json (medium_term + long_term, 1.0 MB) and data_misc.json (strategies + zacks_*, 67 KB). Critical bundle now 456 KB — total cold-load reduction 5.29 MB → 456 KB (91.4% smaller). fsSetMode awaits signals_ext when user clicks Position/Invest. loadChunk("signals_ext") arrival re-fires earnings widget, sidebar counts, killed corr-drop scan, and (if user is on non-default mode) the scanner.</t>
+        </is>
+      </c>
+      <c r="K62" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="inlineStr">
+        <is>
+          <t>cf30df858</t>
+        </is>
+      </c>
       <c r="N62" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
-        </is>
-      </c>
-    </row>
-    <row r="63" ht="45" customHeight="1">
+          <t>1. python3 infra/prototype/build_data.py — emits data.critical.json (~456 KB) plus 7 chunks. 2. Open /v2/dashboard.html in DevTools Network — boot only fetches data.critical.json (~456 KB), then 7 chunks load in parallel without blocking first paint. 3. Click POSITION mode in scanner — table populates with mt rows (may briefly show empty if signals_ext chunk hasn't arrived yet — should resolve within 100-300ms). 4. Click INVEST mode — same with lt rows. 5. Verify earnings widget at top of scanner shows imminent earnings from BOTH short_term and medium_term. 6. Verify scanCount/ctMt/ctLt counts at boot show real numbers (from _chunk_counts).</t>
+        </is>
+      </c>
+    </row>
+    <row r="63" ht="135" customHeight="1">
       <c r="A63" s="2" t="n">
         <v>62</v>
       </c>
       <c r="B63" s="3" t="inlineStr">
         <is>
-          <t>PERF-8-13</t>
+          <t>MOD-1</t>
         </is>
       </c>
       <c r="C63" s="9" t="inlineStr">
@@ -4880,49 +4864,57 @@
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>Performance</t>
+          <t>UI / Modularization</t>
         </is>
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+          <t>Scanner deep refactor</t>
         </is>
       </c>
       <c r="F63" s="5" t="inlineStr">
         <is>
-          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+          <t>Scanner stays inline due to heavy let-bound state. Doesn't fit registry-driven module pattern cleanly.</t>
         </is>
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+          <t>Extract Scanner state into Zustand-style store (or simple module-scope object). Move render fn into infra/prototype/tabs/scanner/. Wire state via window event bus.</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr">
         <is>
-          <t>hours-days each</t>
+          <t>1-2 hrs</t>
         </is>
       </c>
       <c r="I63" s="5" t="inlineStr">
         <is>
-          <t>Win varies; defer until PERF-7 measured.</t>
+          <t>Risk: low (works fine inline). Win: consistency.</t>
         </is>
       </c>
       <c r="J63" s="5" t="inlineStr">
         <is>
-          <t>Don't pre-implement.</t>
-        </is>
-      </c>
-      <c r="K63" s="14" t="inlineStr">
-        <is>
-          <t>DEFERRED</t>
-        </is>
-      </c>
-      <c r="L63" s="2" t="inlineStr"/>
-      <c r="M63" s="3" t="inlineStr"/>
+          <t>Shipped 2026-05-10 in commit 42c36ef91. Two latent bugs fixed: (1) bare FS_STATE in scanner.js → ReferenceError at module scope (let-binding, not on window); (2) tabs.scanner had no `module` field in capability_registry.json so shell.js loader never overrode the inline renderFloorScanner. Until tonight, scanner has been running entirely off the inline path. Module split into 5 sub-files: scanner / filters / row / sparkline / sectors. Inline renderFloorScanner retained as fallback per shell.js convention.</t>
+        </is>
+      </c>
+      <c r="K63" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr">
+        <is>
+          <t>42c36ef91</t>
+        </is>
+      </c>
       <c r="N63" s="8" t="inlineStr">
         <is>
-          <t>n/a — deferred</t>
+          <t>1. Hard-refresh https://trade.mystockholding.com/v2/dashboard.html — scanner is the default tab, must render identically to before. 2. Open DevTools console, look for `[shell] rendered tab 'scanner' from module tabs/scanner/scanner.js in Xms` — confirms module path is now active (was silently falling through to inline before). 3. Click filter chips (mode, verdict, sector, etc) — applyFilters() in filters.js handles all 13 filters. 4. Click any row to expand inline drawer — row.js _handleRowClick wiring intact. 5. Click ★ star to toggle watchlist — _toggleStar handler on row. 6. node --check tabs/scanner/*.js → all 5 files pass.</t>
         </is>
       </c>
     </row>
@@ -4932,69 +4924,73 @@
       </c>
       <c r="B64" s="3" t="inlineStr">
         <is>
-          <t>Q1-step7</t>
-        </is>
-      </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>P0</t>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="C64" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>QUANT-1 Sunday follow-up</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E64" s="6" t="inlineStr">
         <is>
-          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+          <t>Verify backtest persistence (cb1f5a010)</t>
         </is>
       </c>
       <c r="F64" s="5" t="inlineStr">
         <is>
-          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+          <t>Verify the parameterized snapshot mechanism (commit cb1f5a010) prevents silent overwrites.</t>
         </is>
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+          <t>ls cache/portfolio_backtest_*.json — confirmed 3 snapshots preserved (750d_20260509_100501, AB_60d_min75_hold7, BASELINE_20260508_235917).</t>
         </is>
       </c>
       <c r="H64" s="2" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>verified</t>
         </is>
       </c>
       <c r="I64" s="5" t="inlineStr">
         <is>
-          <t>n/a</t>
+          <t>Win: persistence works; no silent overwrites.</t>
         </is>
       </c>
       <c r="J64" s="5" t="inlineStr">
         <is>
-          <t>Agents skim and miss post-filter subset analysis.</t>
-        </is>
-      </c>
-      <c r="K64" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
-        </is>
-      </c>
-      <c r="L64" s="2" t="inlineStr"/>
+          <t>3 snapshot files present. Validates cb1f5a010.</t>
+        </is>
+      </c>
+      <c r="K64" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
+        </is>
+      </c>
+      <c r="L64" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-09</t>
+        </is>
+      </c>
       <c r="M64" s="3" t="inlineStr"/>
       <c r="N64" s="8" t="inlineStr">
         <is>
-          <t>n/a — rejected</t>
-        </is>
-      </c>
-    </row>
-    <row r="65" ht="90" customHeight="1">
+          <t>ls cache/portfolio_backtest_*.json | wc -l → ≥3 (snapshots preserved with timestamps). Confirms backtest persistence is working.</t>
+        </is>
+      </c>
+    </row>
+    <row r="65" ht="45" customHeight="1">
       <c r="A65" s="2" t="n">
         <v>64</v>
       </c>
       <c r="B65" s="3" t="inlineStr">
         <is>
-          <t>H1</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="C65" s="13" t="inlineStr">
@@ -5004,51 +5000,303 @@
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>Data / Universe</t>
+          <t>Operational</t>
         </is>
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+          <t>Verify state_backup.py post-Mode-1 dual-write</t>
         </is>
       </c>
       <c r="F65" s="5" t="inlineStr">
         <is>
-          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+          <t>Verify daily snapshot script still works after Mode 1 Supabase dual-write was wired.</t>
         </is>
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+          <t>ls data/backups/ — confirm 7-day retention (latest 2026-05-08 verified). state_backup.py imports OK.</t>
         </is>
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>$$ + 1 day</t>
+          <t>verified (no change needed)</t>
         </is>
       </c>
       <c r="I65" s="5" t="inlineStr">
         <is>
-          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+          <t>Win: confirms infrastructure still healthy.</t>
         </is>
       </c>
       <c r="J65" s="5" t="inlineStr">
         <is>
-          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
-        </is>
-      </c>
-      <c r="K65" s="15" t="inlineStr">
-        <is>
-          <t>REJECTED</t>
+          <t>7 backup dirs present, latest 2026-05-08.</t>
+        </is>
+      </c>
+      <c r="K65" s="12" t="inlineStr">
+        <is>
+          <t>DONE</t>
         </is>
       </c>
       <c r="L65" s="2" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-09</t>
         </is>
       </c>
       <c r="M65" s="3" t="inlineStr"/>
       <c r="N65" s="8" t="inlineStr">
+        <is>
+          <t>ls data/backups/ → 7 backup dirs present, latest dated within last 24h. state_backup.py runs daily via cron.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66" ht="45" customHeight="1">
+      <c r="A66" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>CLEAN-2</t>
+        </is>
+      </c>
+      <c r="C66" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D66" s="5" t="inlineStr">
+        <is>
+          <t>Code Cleanup (DEFERRED)</t>
+        </is>
+      </c>
+      <c r="E66" s="6" t="inlineStr">
+        <is>
+          <t>migrate_json_to_sqlite.py + migrate_sqlite_to_supabase.py</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>231 + 440 = 671 lines of one-shot migration scripts already executed.</t>
+        </is>
+      </c>
+      <c r="G66" s="5" t="inlineStr">
+        <is>
+          <t>Keep until 2026-Q4 unless user explicitly says otherwise. Then delete + remove migration entrypoints from CLAUDE.md.</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>5 min after answer</t>
+        </is>
+      </c>
+      <c r="I66" s="5" t="inlineStr">
+        <is>
+          <t>Win: -671 lines.</t>
+        </is>
+      </c>
+      <c r="J66" s="5" t="inlineStr">
+        <is>
+          <t>Standard data-migration retention practice.</t>
+        </is>
+      </c>
+      <c r="K66" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
+        </is>
+      </c>
+      <c r="L66" s="2" t="inlineStr"/>
+      <c r="M66" s="3" t="inlineStr"/>
+      <c r="N66" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="45" customHeight="1">
+      <c r="A67" s="2" t="n">
+        <v>66</v>
+      </c>
+      <c r="B67" s="3" t="inlineStr">
+        <is>
+          <t>PERF-8-13</t>
+        </is>
+      </c>
+      <c r="C67" s="9" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="D67" s="5" t="inlineStr">
+        <is>
+          <t>Performance</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Service worker, web worker, HTTP/2 push, skeleton screens, NDJSON streaming, SSR</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Diminishing-returns optimizations after PERF-7 lands.</t>
+        </is>
+      </c>
+      <c r="G67" s="5" t="inlineStr">
+        <is>
+          <t>Each addresses a specific perceived-perf gap; defer until post-PERF-7 measurement identifies which one matters.</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>hours-days each</t>
+        </is>
+      </c>
+      <c r="I67" s="5" t="inlineStr">
+        <is>
+          <t>Win varies; defer until PERF-7 measured.</t>
+        </is>
+      </c>
+      <c r="J67" s="5" t="inlineStr">
+        <is>
+          <t>Don't pre-implement.</t>
+        </is>
+      </c>
+      <c r="K67" s="14" t="inlineStr">
+        <is>
+          <t>DEFERRED</t>
+        </is>
+      </c>
+      <c r="L67" s="2" t="inlineStr"/>
+      <c r="M67" s="3" t="inlineStr"/>
+      <c r="N67" s="8" t="inlineStr">
+        <is>
+          <t>n/a — deferred</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="45" customHeight="1">
+      <c r="A68" s="2" t="n">
+        <v>67</v>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Q1-step7</t>
+        </is>
+      </c>
+      <c r="C68" s="11" t="inlineStr">
+        <is>
+          <t>P0</t>
+        </is>
+      </c>
+      <c r="D68" s="5" t="inlineStr">
+        <is>
+          <t>QUANT-1 Sunday follow-up</t>
+        </is>
+      </c>
+      <c r="E68" s="6" t="inlineStr">
+        <is>
+          <t>DO NOT add buy_max_score: 80 (the agent's Fix 2)</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Capping at 80 would amputate the alpha zone (80-85 band, n=21, PF 1.72).</t>
+        </is>
+      </c>
+      <c r="G68" s="5" t="inlineStr">
+        <is>
+          <t>Explicit 'do not implement' guidance. Reject any agent suggestion to cap at 80.</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="I68" s="5" t="inlineStr">
+        <is>
+          <t>n/a</t>
+        </is>
+      </c>
+      <c r="J68" s="5" t="inlineStr">
+        <is>
+          <t>Agents skim and miss post-filter subset analysis.</t>
+        </is>
+      </c>
+      <c r="K68" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L68" s="2" t="inlineStr"/>
+      <c r="M68" s="3" t="inlineStr"/>
+      <c r="N68" s="8" t="inlineStr">
+        <is>
+          <t>n/a — rejected</t>
+        </is>
+      </c>
+    </row>
+    <row r="69" ht="90" customHeight="1">
+      <c r="A69" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="B69" s="3" t="inlineStr">
+        <is>
+          <t>H1</t>
+        </is>
+      </c>
+      <c r="C69" s="13" t="inlineStr">
+        <is>
+          <t>P3</t>
+        </is>
+      </c>
+      <c r="D69" s="5" t="inlineStr">
+        <is>
+          <t>Data / Universe</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Russell 1000 historical membership (Sharadar SF1)</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>750d backtest uses today's R1000 membership for past dates; small survivorship bias on top of S&amp;P 500 fix.</t>
+        </is>
+      </c>
+      <c r="G69" s="5" t="inlineStr">
+        <is>
+          <t>Sharadar SF1 ($60/mo) provides point-in-time R1000 membership. No free source (Wikipedia doesn't have R1000 history). Finviz Free + Finviz Elite don't have it either.</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr">
+        <is>
+          <t>$$ + 1 day</t>
+        </is>
+      </c>
+      <c r="I69" s="5" t="inlineStr">
+        <is>
+          <t>Risk: small at $5K paper scale. Win: cleaner backtests. Net: deferred.</t>
+        </is>
+      </c>
+      <c r="J69" s="5" t="inlineStr">
+        <is>
+          <t>REJECTED 2026-05-10: user policy — no new data licenses will be procured. Work with existing stack (EODHD + Zacks + Schwab + Alpaca). For R1000 historical membership, accept the small residual survivorship bias (parallel session's S&amp;P 500 monthly snapshots cover the dominant chunk). Total impact at $5K paper scale: ~1pp WR, well within survivorship haircut already applied.</t>
+        </is>
+      </c>
+      <c r="K69" s="15" t="inlineStr">
+        <is>
+          <t>REJECTED</t>
+        </is>
+      </c>
+      <c r="L69" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr"/>
+      <c r="N69" s="8" t="inlineStr">
         <is>
           <t>n/a — rejected</t>
         </is>
@@ -5147,16 +5395,16 @@
         </is>
       </c>
       <c r="B4" s="18" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C4" s="18" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D4" s="18" t="n">
         <v>10</v>
       </c>
       <c r="E4" s="18" t="n">
-        <v>52</v>
+        <v>56</v>
       </c>
     </row>
     <row r="5">
@@ -5204,16 +5452,16 @@
         </is>
       </c>
       <c r="B7" s="23" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C7" s="23" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="D7" s="23" t="n">
         <v>13</v>
       </c>
       <c r="E7" s="23" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Open items: refresh tracker MD with 2026-05-10 status + IPAD-1 notes
OpenItemTracker.md was last updated 2026-05-09 PM and didn't reflect
tonight's 14 shipped items, the 91% boot perf reduction, the iPad PWA,
or the 5 latent bugs caught during MOD-A/B splits.

Updates:
  • Status snapshot reflects current state (modularization deeper split,
    boot perf 91% reduction, iPad PWA shipped, MOD-2 still in progress)
  • In-progress narrowed to 1 (MOD-2)
  • Pending narrowed to 5 (3 quant items needing evidence + 2 date-gated)
  • New "Shipped 2026-05-10" section listing all 14 commits with hashes
  • New "Failed acceptance" section recording Q1-step5 0-BUY result + Variant F recovery path

IPAD-1 (registry): how_to_test + notes refreshed with 3-commit lineage
(shell + verdict-stage hot fix + iframe-aware sidebar hide).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/cache/open_items_2026-05-10.xlsx
+++ b/cache/open_items_2026-05-10.xlsx
@@ -3286,7 +3286,7 @@
         </is>
       </c>
     </row>
-    <row r="40" ht="60" customHeight="1">
+    <row r="40" ht="135" customHeight="1">
       <c r="A40" s="2" t="n">
         <v>39</v>
       </c>
@@ -3332,7 +3332,7 @@
       </c>
       <c r="J40" s="5" t="inlineStr">
         <is>
-          <t>Phase 1 shipped 2026-05-10. Phase 2 deferred: real PNG icons, service worker, swipe-to-action.</t>
+          <t>iPad PWA shipped 2026-05-10 across 3 commits: 4b49cb93e (shell + manifest + ipad.css/js + dashboard.html), b0e5ef6a1 (verdict→stage hot fix — was 0 rows because filter matched r.verdict but bundle has r.stage), 79fa01a75 (iframe-aware sidebar hide in elite-detail.html). PWA-installable via Safari "Add to Home Screen" on iPad. Reuses /v2/elite-detail.html via iframe — single source of truth, no module duplication.</t>
         </is>
       </c>
       <c r="K40" s="12" t="inlineStr">
@@ -3352,7 +3352,7 @@
       </c>
       <c r="N40" s="8" t="inlineStr">
         <is>
-          <t>On iPad open https://trade.mystockholding.com/v2/ipad/dashboard.html. Landscape: 2-pane split. Portrait: full-width list with detail-on-tap.</t>
+          <t>1. Visit https://trade.mystockholding.com/v2/ipad/dashboard.html on iPad Safari (or Chrome desktop with iPad simulator). 2. Confirm Scanner tab shows ~60 WATCH rows (today's scan). 3. Tap any ticker → right pane loads /v2/elite-detail.html in iframe; inside the iframe the FLOOR sidebar + ticker tape + header are HIDDEN (otherwise the embed would render duplicate chrome). 4. Switch to Elite tab → 5 picks from data.elite_picks.Swing. 5. Pull down on the list pane → triggers refreshData() which re-fetches /v2/data.critical.json. 6. iPad home screen: Safari Share → Add to Home Screen → manifest.json metadata installs as standalone PWA.</t>
         </is>
       </c>
     </row>

</xml_diff>